<commit_message>
minor fixes for document generation for new test cases
</commit_message>
<xml_diff>
--- a/core/UAT Plan.xlsx
+++ b/core/UAT Plan.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <workbookPr/>
   <bookViews>
-    <workbookView xWindow="360" yWindow="15" windowWidth="20955" windowHeight="9720" activeTab="0"/>
+    <workbookView xWindow="360" yWindow="15" windowWidth="20955" windowHeight="9720" activeTab="3"/>
   </bookViews>
   <sheets>
     <sheet name="Demo person 1" sheetId="1" state="visible" r:id="rId4"/>
@@ -19,7 +19,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="104" uniqueCount="104">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="148" uniqueCount="148">
   <si>
     <t xml:space="preserve">Test Case #</t>
   </si>
@@ -340,14 +340,157 @@
     <t>Code</t>
   </si>
   <si>
-    <t>Others</t>
+    <t xml:space="preserve">Patient 6</t>
+  </si>
+  <si>
+    <t>Gastroenterology</t>
+  </si>
+  <si>
+    <t>43239</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Upper GI Endoscopy with Biopsy (EGD)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1. Initial complaint of epigastric discomfort</t>
+  </si>
+  <si>
+    <t xml:space="preserve">No prior treatment documented; no H. pylori test, no PPI trial, no imaging</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Requires failed PPI therapy (min. 4–8 weeks), H. pylori test result, or documented alarm symptoms (dysphagia, weight loss, hematemesis)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2. PPI therapy trial documented
+3. H. pylori test result included
+4. Alarm symptoms noted in chart</t>
+  </si>
+  <si>
+    <t xml:space="preserve">All required supporting documentation present</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Patient 7</t>
+  </si>
+  <si>
+    <t>45378</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Colonoscopy, Diagnostic</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1. Patient complaint of occasional rectal bleeding</t>
+  </si>
+  <si>
+    <t xml:space="preserve">No prior colonoscopy record; no family history of colorectal cancer noted; patient under age 45 with no high-risk indicators</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Requires documentation of high-risk criteria (age 45+, family history of CRC, prior polyps, IBD diagnosis) or symptomatic indicators with clinical notes (persistent bleeding, iron deficiency anemia)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2. Family history of colorectal cancer documented
+3. Iron deficiency anemia confirmed via lab results
+4. Persistent rectal bleeding noted over 3+ months</t>
+  </si>
+  <si>
+    <t xml:space="preserve">High-risk family history and symptomatic indicators fully documented</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Patient 8</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1. PPI therapy (omeprazole 20mg) documented for 8 weeks with no improvement
+2. H. pylori urea breath test: Positive</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Failed PPI trial documented; positive H. pylori confirmed; dysphagia reported in clinical note</t>
+  </si>
+  <si>
+    <t xml:space="preserve">3. Physician note confirming dysphagia and 8 lb unintentional weight loss</t>
+  </si>
+  <si>
+    <t xml:space="preserve">All alarm symptom criteria and prior treatment failure documented — high likelihood of approval</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Patient 9</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1. Patient age 52 with documented family history of colorectal cancer (parent)
+2. Prior adenomatous polyp removal 5 years ago</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Age criteria met; high-risk family history confirmed; prior polyp history documented</t>
+  </si>
+  <si>
+    <t xml:space="preserve">3. Gastroenterologist order with medical necessity justification for surveillance colonoscopy</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Multiple high-risk indicators confirmed with specialist order — strong approval likelihood</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Patient 10</t>
+  </si>
+  <si>
+    <t>OB/GYN</t>
+  </si>
+  <si>
+    <t>S0190</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Mifepristone (Abortion Medication)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1. Confirmed intrauterine pregnancy ≤10 weeks gestation via ultrasound</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Gestational age confirmed within FDA-approved window; patient counseled and consented; mifepristone prescribed per protocol</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Requires confirmed intrauterine pregnancy ≤10 weeks gestation; provider must be certified under REMS program; documentation of informed consent and patient counseling</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2. REMS-certified provider attestation on file
+3. Informed consent signed
+4. Follow-up plan documented</t>
+  </si>
+  <si>
+    <t xml:space="preserve">All FDA REMS criteria met; gestational age confirmed; full protocol documentation present</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Patient 11</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Physical Therapy</t>
+  </si>
+  <si>
+    <t>97110</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Therapeutic Exercise (Post-injury Physiotherapy)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1. ER visit report: acute knee sprain sustained during basketball game
+2. MRI confirming Grade II MCL tear
+3. Orthopedic physician referral for physical therapy</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Acute sports injury documented with imaging; orthopedic referral with PT order specifying diagnosis, frequency, and duration; functional impairment noted</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Requires physician referral with diagnosis code, imaging or clinical documentation of injury, PT evaluation with functional goals, and treatment plan specifying visit frequency and expected duration</t>
+  </si>
+  <si>
+    <t xml:space="preserve">4. PT evaluation with measurable functional goals
+5. Treatment plan: 2x/week for 8 weeks</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Complete documentation package with referral, imaging, and PT treatment plan — high approval likelihood</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
-  <fonts count="3">
+  <fonts count="4">
     <font>
       <sz val="11.000000"/>
       <color theme="1"/>
@@ -363,8 +506,12 @@
     </font>
     <font>
       <sz val="11.000000"/>
+      <name val="Aptos Narrow"/>
+    </font>
+    <font>
+      <sz val="12.000000"/>
       <color indexed="64"/>
-      <name val="Aptos Narrow"/>
+      <name val="Times"/>
     </font>
   </fonts>
   <fills count="4">
@@ -385,7 +532,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="4">
+  <borders count="6">
     <border>
       <left style="none"/>
       <right style="none"/>
@@ -395,50 +542,76 @@
     </border>
     <border>
       <left style="thin">
-        <color indexed="64"/>
+        <color auto="1"/>
       </left>
       <right style="thin">
-        <color indexed="64"/>
+        <color auto="1"/>
       </right>
       <top style="thin">
-        <color indexed="64"/>
+        <color auto="1"/>
       </top>
       <bottom style="thin">
-        <color indexed="64"/>
+        <color auto="1"/>
       </bottom>
       <diagonal style="none"/>
     </border>
     <border>
       <left style="thin">
-        <color indexed="64"/>
+        <color auto="1"/>
       </left>
       <right style="thin">
-        <color indexed="64"/>
+        <color auto="1"/>
       </right>
       <top style="thin">
-        <color indexed="64"/>
+        <color auto="1"/>
       </top>
       <bottom style="none"/>
       <diagonal style="none"/>
     </border>
     <border>
       <left style="thin">
-        <color indexed="64"/>
+        <color auto="1"/>
       </left>
       <right style="thin">
-        <color indexed="64"/>
+        <color auto="1"/>
       </right>
       <top style="none"/>
       <bottom style="thin">
-        <color indexed="64"/>
+        <color auto="1"/>
       </bottom>
       <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top/>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
     </border>
   </borders>
   <cellStyleXfs count="1">
     <xf fontId="0" fillId="0" borderId="0" numFmtId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
   </cellStyleXfs>
-  <cellXfs count="24">
+  <cellXfs count="38">
     <xf fontId="0" fillId="0" borderId="0" numFmtId="0" xfId="0"/>
     <xf fontId="0" fillId="0" borderId="0" numFmtId="0" xfId="0" applyAlignment="1">
       <alignment vertical="center"/>
@@ -504,8 +677,50 @@
     <xf fontId="0" fillId="0" borderId="1" numFmtId="0" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf fontId="0" fillId="0" borderId="1" numFmtId="0" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf fontId="2" fillId="0" borderId="1" numFmtId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf fontId="2" fillId="0" borderId="4" numFmtId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf fontId="2" fillId="0" borderId="4" numFmtId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf fontId="2" fillId="0" borderId="1" numFmtId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf fontId="2" fillId="0" borderId="1" numFmtId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf fontId="2" fillId="0" borderId="1" numFmtId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf fontId="2" fillId="0" borderId="0" numFmtId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf fontId="2" fillId="0" borderId="5" numFmtId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf fontId="2" fillId="0" borderId="5" numFmtId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf fontId="2" fillId="0" borderId="0" numFmtId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf fontId="2" fillId="0" borderId="0" numFmtId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf fontId="2" fillId="0" borderId="0" numFmtId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf fontId="2" fillId="0" borderId="0" numFmtId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf fontId="2" fillId="0" borderId="0" numFmtId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf fontId="3" fillId="0" borderId="0" numFmtId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -2032,194 +2247,337 @@
       </c>
     </row>
     <row r="2" ht="27.75" customHeight="1">
-      <c r="A2" s="8" t="s">
-        <v>8</v>
-      </c>
-      <c r="B2" s="23" t="s">
+      <c r="A2" s="23" t="s">
         <v>103</v>
       </c>
-      <c r="C2" s="8"/>
-      <c r="D2" s="17" t="s">
-        <v>72</v>
-      </c>
-      <c r="E2" s="17" t="s">
-        <v>73</v>
-      </c>
-      <c r="F2" s="20" t="s">
-        <v>74</v>
-      </c>
-      <c r="G2" s="19" t="s">
+      <c r="B2" s="24" t="s">
+        <v>104</v>
+      </c>
+      <c r="C2" s="25" t="s">
+        <v>105</v>
+      </c>
+      <c r="D2" s="24" t="s">
+        <v>106</v>
+      </c>
+      <c r="E2" s="26" t="s">
+        <v>107</v>
+      </c>
+      <c r="F2" s="27" t="s">
+        <v>108</v>
+      </c>
+      <c r="G2" s="28" t="s">
         <v>13</v>
       </c>
-      <c r="H2" s="17" t="s">
-        <v>75</v>
-      </c>
-      <c r="I2" s="1">
-        <v>250</v>
+      <c r="H2" s="26" t="s">
+        <v>109</v>
+      </c>
+      <c r="I2" s="29">
+        <v>260</v>
       </c>
       <c r="J2" s="1"/>
     </row>
     <row r="3" ht="50.25" customHeight="1">
-      <c r="A3" s="8" t="s">
-        <v>8</v>
-      </c>
-      <c r="B3" s="22"/>
-      <c r="C3" s="8"/>
-      <c r="D3" s="17"/>
-      <c r="E3" s="17" t="s">
-        <v>76</v>
-      </c>
-      <c r="F3" s="20" t="s">
-        <v>77</v>
-      </c>
-      <c r="G3" s="19" t="s">
+      <c r="A3" s="23" t="s">
+        <v>103</v>
+      </c>
+      <c r="B3" s="30"/>
+      <c r="C3" s="31"/>
+      <c r="D3" s="30"/>
+      <c r="E3" s="26" t="s">
+        <v>110</v>
+      </c>
+      <c r="F3" s="27" t="s">
+        <v>111</v>
+      </c>
+      <c r="G3" s="28" t="s">
+        <v>17</v>
+      </c>
+      <c r="H3" s="20"/>
+      <c r="I3" s="29">
+        <v>261</v>
+      </c>
+      <c r="J3" s="1"/>
+    </row>
+    <row r="4">
+      <c r="A4" s="23" t="s">
+        <v>112</v>
+      </c>
+      <c r="B4" s="24" t="s">
+        <v>104</v>
+      </c>
+      <c r="C4" s="25" t="s">
+        <v>113</v>
+      </c>
+      <c r="D4" s="24" t="s">
+        <v>114</v>
+      </c>
+      <c r="E4" s="26" t="s">
+        <v>115</v>
+      </c>
+      <c r="F4" s="27" t="s">
+        <v>116</v>
+      </c>
+      <c r="G4" s="28" t="s">
+        <v>13</v>
+      </c>
+      <c r="H4" s="26" t="s">
+        <v>117</v>
+      </c>
+      <c r="I4" s="29">
+        <v>262</v>
+      </c>
+      <c r="J4" s="1"/>
+    </row>
+    <row r="5" ht="43.5">
+      <c r="A5" s="23" t="s">
+        <v>112</v>
+      </c>
+      <c r="B5" s="30"/>
+      <c r="C5" s="31"/>
+      <c r="D5" s="30"/>
+      <c r="E5" s="26" t="s">
+        <v>118</v>
+      </c>
+      <c r="F5" s="27" t="s">
+        <v>119</v>
+      </c>
+      <c r="G5" s="28" t="s">
+        <v>17</v>
+      </c>
+      <c r="H5" s="20"/>
+      <c r="I5" s="29">
+        <v>263</v>
+      </c>
+      <c r="J5" s="1"/>
+    </row>
+    <row r="6" ht="29.25" customHeight="1">
+      <c r="A6" s="23" t="s">
+        <v>120</v>
+      </c>
+      <c r="B6" s="24" t="s">
+        <v>104</v>
+      </c>
+      <c r="C6" s="25" t="s">
+        <v>105</v>
+      </c>
+      <c r="D6" s="24" t="s">
+        <v>106</v>
+      </c>
+      <c r="E6" s="26" t="s">
+        <v>121</v>
+      </c>
+      <c r="F6" s="27" t="s">
+        <v>122</v>
+      </c>
+      <c r="G6" s="28" t="s">
+        <v>17</v>
+      </c>
+      <c r="H6" s="26" t="s">
+        <v>109</v>
+      </c>
+      <c r="I6" s="29">
+        <v>264</v>
+      </c>
+      <c r="J6" s="1"/>
+    </row>
+    <row r="7">
+      <c r="A7" s="23" t="s">
+        <v>120</v>
+      </c>
+      <c r="B7" s="30"/>
+      <c r="C7" s="31"/>
+      <c r="D7" s="30"/>
+      <c r="E7" s="26" t="s">
+        <v>123</v>
+      </c>
+      <c r="F7" s="27" t="s">
+        <v>124</v>
+      </c>
+      <c r="G7" s="28" t="s">
         <v>78</v>
       </c>
-      <c r="H3" s="17"/>
-      <c r="I3" s="1"/>
-      <c r="J3" s="1"/>
-    </row>
-    <row r="4">
-      <c r="A4" s="8" t="s">
-        <v>18</v>
-      </c>
-      <c r="B4" s="22"/>
-      <c r="C4" s="8">
-        <v>21196</v>
-      </c>
-      <c r="D4" s="17"/>
-      <c r="E4" s="17"/>
-      <c r="F4" s="20"/>
-      <c r="G4" s="19"/>
-      <c r="H4" s="17"/>
-      <c r="I4" s="1"/>
-      <c r="J4" s="1"/>
-    </row>
-    <row r="5" ht="43.5">
-      <c r="A5" s="8" t="s">
-        <v>18</v>
-      </c>
-      <c r="B5" s="22"/>
-      <c r="C5" s="8"/>
-      <c r="D5" s="17"/>
-      <c r="E5" s="17"/>
-      <c r="F5" s="20"/>
-      <c r="G5" s="19"/>
-      <c r="H5" s="17"/>
-      <c r="I5" s="1"/>
-      <c r="J5" s="1"/>
-    </row>
-    <row r="6" ht="29.25" customHeight="1">
-      <c r="A6" s="8" t="s">
-        <v>25</v>
-      </c>
-      <c r="B6" s="22"/>
-      <c r="C6" s="8">
-        <v>21210</v>
-      </c>
-      <c r="D6" s="17"/>
-      <c r="E6" s="17"/>
-      <c r="F6" s="18"/>
-      <c r="G6" s="19"/>
-      <c r="H6" s="17"/>
-      <c r="I6" s="1"/>
-      <c r="J6" s="1"/>
-    </row>
-    <row r="7">
-      <c r="A7" s="8" t="s">
-        <v>25</v>
-      </c>
-      <c r="B7" s="22"/>
-      <c r="C7" s="8"/>
-      <c r="D7" s="17"/>
-      <c r="E7" s="17"/>
-      <c r="F7" s="18"/>
-      <c r="G7" s="19"/>
-      <c r="H7" s="17"/>
-      <c r="I7" s="1"/>
+      <c r="H7" s="20"/>
+      <c r="I7" s="29">
+        <v>265</v>
+      </c>
       <c r="J7" s="1"/>
     </row>
     <row r="8">
-      <c r="A8" s="8" t="s">
-        <v>32</v>
-      </c>
-      <c r="B8" s="22"/>
-      <c r="C8" s="8">
-        <v>21085</v>
-      </c>
-      <c r="D8" s="17"/>
-      <c r="E8" s="17"/>
-      <c r="F8" s="20"/>
-      <c r="G8" s="19"/>
-      <c r="H8" s="17"/>
-      <c r="I8" s="1"/>
+      <c r="A8" s="23" t="s">
+        <v>125</v>
+      </c>
+      <c r="B8" s="24" t="s">
+        <v>104</v>
+      </c>
+      <c r="C8" s="25" t="s">
+        <v>113</v>
+      </c>
+      <c r="D8" s="24" t="s">
+        <v>114</v>
+      </c>
+      <c r="E8" s="26" t="s">
+        <v>126</v>
+      </c>
+      <c r="F8" s="27" t="s">
+        <v>127</v>
+      </c>
+      <c r="G8" s="28" t="s">
+        <v>17</v>
+      </c>
+      <c r="H8" s="26" t="s">
+        <v>117</v>
+      </c>
+      <c r="I8" s="29">
+        <v>266</v>
+      </c>
       <c r="J8" s="1"/>
     </row>
     <row r="9" ht="29.25">
-      <c r="A9" s="8" t="s">
-        <v>32</v>
-      </c>
-      <c r="B9" s="22"/>
-      <c r="C9" s="8"/>
-      <c r="D9" s="17"/>
-      <c r="E9" s="17"/>
-      <c r="F9" s="20"/>
-      <c r="G9" s="19"/>
-      <c r="H9" s="17"/>
-      <c r="I9" s="1"/>
+      <c r="A9" s="23" t="s">
+        <v>125</v>
+      </c>
+      <c r="B9" s="30"/>
+      <c r="C9" s="31"/>
+      <c r="D9" s="30"/>
+      <c r="E9" s="26" t="s">
+        <v>128</v>
+      </c>
+      <c r="F9" s="27" t="s">
+        <v>129</v>
+      </c>
+      <c r="G9" s="28" t="s">
+        <v>78</v>
+      </c>
+      <c r="H9" s="20"/>
+      <c r="I9" s="29">
+        <v>267</v>
+      </c>
       <c r="J9" s="1"/>
     </row>
     <row r="10" ht="18.75" customHeight="1">
-      <c r="A10" s="8" t="s">
-        <v>38</v>
-      </c>
-      <c r="B10" s="22"/>
-      <c r="C10" s="8">
-        <v>21235</v>
-      </c>
-      <c r="D10" s="17"/>
-      <c r="E10" s="17"/>
-      <c r="F10" s="20"/>
-      <c r="G10" s="19"/>
-      <c r="H10" s="17"/>
-      <c r="I10" s="1"/>
+      <c r="A10" s="23" t="s">
+        <v>130</v>
+      </c>
+      <c r="B10" s="24" t="s">
+        <v>131</v>
+      </c>
+      <c r="C10" s="25" t="s">
+        <v>132</v>
+      </c>
+      <c r="D10" s="24" t="s">
+        <v>133</v>
+      </c>
+      <c r="E10" s="26" t="s">
+        <v>134</v>
+      </c>
+      <c r="F10" s="27" t="s">
+        <v>135</v>
+      </c>
+      <c r="G10" s="28" t="s">
+        <v>17</v>
+      </c>
+      <c r="H10" s="26" t="s">
+        <v>136</v>
+      </c>
+      <c r="I10" s="29">
+        <v>268</v>
+      </c>
       <c r="J10" s="1"/>
     </row>
     <row r="11" ht="29.25" customHeight="1">
-      <c r="A11" s="8" t="s">
-        <v>38</v>
-      </c>
-      <c r="B11" s="22"/>
-      <c r="C11" s="8"/>
-      <c r="D11" s="17"/>
-      <c r="E11" s="17"/>
-      <c r="F11" s="20"/>
-      <c r="G11" s="19"/>
-      <c r="H11" s="17"/>
-      <c r="I11" s="1"/>
+      <c r="A11" s="23" t="s">
+        <v>130</v>
+      </c>
+      <c r="B11" s="30"/>
+      <c r="C11" s="31"/>
+      <c r="D11" s="30"/>
+      <c r="E11" s="26" t="s">
+        <v>137</v>
+      </c>
+      <c r="F11" s="27" t="s">
+        <v>138</v>
+      </c>
+      <c r="G11" s="28" t="s">
+        <v>78</v>
+      </c>
+      <c r="H11" s="20"/>
+      <c r="I11" s="29">
+        <v>269</v>
+      </c>
       <c r="J11" s="1"/>
     </row>
+    <row r="12" ht="15">
+      <c r="A12" s="32" t="s">
+        <v>139</v>
+      </c>
+      <c r="B12" s="33" t="s">
+        <v>140</v>
+      </c>
+      <c r="C12" s="34" t="s">
+        <v>141</v>
+      </c>
+      <c r="D12" s="33" t="s">
+        <v>142</v>
+      </c>
+      <c r="E12" s="35" t="s">
+        <v>143</v>
+      </c>
+      <c r="F12" s="36" t="s">
+        <v>144</v>
+      </c>
+      <c r="G12" s="29" t="s">
+        <v>17</v>
+      </c>
+      <c r="H12" s="35" t="s">
+        <v>145</v>
+      </c>
+      <c r="I12" s="29">
+        <v>270</v>
+      </c>
+    </row>
     <row r="13">
-      <c r="A13" s="21"/>
+      <c r="A13" s="32" t="s">
+        <v>139</v>
+      </c>
+      <c r="B13" s="33"/>
+      <c r="C13" s="34"/>
+      <c r="D13" s="33"/>
+      <c r="E13" s="35" t="s">
+        <v>146</v>
+      </c>
+      <c r="F13" s="36" t="s">
+        <v>147</v>
+      </c>
+      <c r="G13" s="29" t="s">
+        <v>78</v>
+      </c>
+      <c r="I13" s="29">
+        <v>271</v>
+      </c>
+    </row>
+    <row r="14" ht="15">
+      <c r="A14" s="37"/>
     </row>
   </sheetData>
-  <mergeCells count="16">
-    <mergeCell ref="B2:B11"/>
+  <mergeCells count="18">
+    <mergeCell ref="B2:B3"/>
     <mergeCell ref="C2:C3"/>
     <mergeCell ref="D2:D3"/>
-    <mergeCell ref="H2:H3"/>
+    <mergeCell ref="B4:B5"/>
     <mergeCell ref="C4:C5"/>
     <mergeCell ref="D4:D5"/>
-    <mergeCell ref="H4:H5"/>
+    <mergeCell ref="B6:B7"/>
     <mergeCell ref="C6:C7"/>
     <mergeCell ref="D6:D7"/>
-    <mergeCell ref="H6:H7"/>
+    <mergeCell ref="B8:B9"/>
     <mergeCell ref="C8:C9"/>
     <mergeCell ref="D8:D9"/>
-    <mergeCell ref="H8:H9"/>
+    <mergeCell ref="B10:B11"/>
     <mergeCell ref="C10:C11"/>
     <mergeCell ref="D10:D11"/>
-    <mergeCell ref="H10:H11"/>
+    <mergeCell ref="B12:B13"/>
+    <mergeCell ref="C12:C13"/>
+    <mergeCell ref="D12:D13"/>
   </mergeCells>
   <printOptions headings="0" gridLines="0"/>
   <pageMargins left="0.69999999999999996" right="0.69999999999999996" top="0.75" bottom="0.75" header="0.29999999999999999" footer="0.29999999999999999"/>

</xml_diff>

<commit_message>
Implement job cancellation with rollback for single and batch patient generation, and allow specific patient selection for batch processing.
</commit_message>
<xml_diff>
--- a/core/UAT Plan.xlsx
+++ b/core/UAT Plan.xlsx
@@ -19,7 +19,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="148" uniqueCount="148">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="167" uniqueCount="167">
   <si>
     <t xml:space="preserve">Test Case #</t>
   </si>
@@ -355,20 +355,23 @@
     <t xml:space="preserve">1. Initial complaint of epigastric discomfort</t>
   </si>
   <si>
-    <t xml:space="preserve">No prior treatment documented; no H. pylori test, no PPI trial, no imaging</t>
+    <t xml:space="preserve">No prior treatment documented; no H. pylori test, no PPI trial, no imaging — missing all qualifying criteria for approval</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Requires failed PPI therapy (min. 4–8 weeks) AND H. pylori test result, OR documented alarm symptoms (dysphagia, weight loss, hematemesis). Rejection issued when all qualifying criteria are absent.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1. PPI therapy trial documented
+2. H. pylori test result included
+3. Alarm symptoms noted in chart</t>
+  </si>
+  <si>
+    <t xml:space="preserve">All required supporting documentation present; prior treatment failure and alarm symptoms confirmed</t>
   </si>
   <si>
     <t xml:space="preserve">Requires failed PPI therapy (min. 4–8 weeks), H. pylori test result, or documented alarm symptoms (dysphagia, weight loss, hematemesis)</t>
   </si>
   <si>
-    <t xml:space="preserve">2. PPI therapy trial documented
-3. H. pylori test result included
-4. Alarm symptoms noted in chart</t>
-  </si>
-  <si>
-    <t xml:space="preserve">All required supporting documentation present</t>
-  </si>
-  <si>
     <t xml:space="preserve">Patient 7</t>
   </si>
   <si>
@@ -381,50 +384,59 @@
     <t xml:space="preserve">1. Patient complaint of occasional rectal bleeding</t>
   </si>
   <si>
-    <t xml:space="preserve">No prior colonoscopy record; no family history of colorectal cancer noted; patient under age 45 with no high-risk indicators</t>
+    <t xml:space="preserve">No prior colonoscopy record; no family history of colorectal cancer noted; patient under age 45 with no high-risk indicators — no qualifying criterion met</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Requires documentation of high-risk criteria (age 45+, family history of CRC, prior polyps, IBD diagnosis) OR symptomatic indicators (persistent bleeding, iron deficiency anemia). Rejection issued when no qualifying criterion is present.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1. Family history of colorectal cancer documented
+2. Iron deficiency anemia confirmed via lab results
+3. Persistent rectal bleeding noted over 3+ months</t>
+  </si>
+  <si>
+    <t xml:space="preserve">High-risk family history and symptomatic indicators fully documented</t>
   </si>
   <si>
     <t xml:space="preserve">Requires documentation of high-risk criteria (age 45+, family history of CRC, prior polyps, IBD diagnosis) or symptomatic indicators with clinical notes (persistent bleeding, iron deficiency anemia)</t>
   </si>
   <si>
-    <t xml:space="preserve">2. Family history of colorectal cancer documented
-3. Iron deficiency anemia confirmed via lab results
-4. Persistent rectal bleeding noted over 3+ months</t>
-  </si>
-  <si>
-    <t xml:space="preserve">High-risk family history and symptomatic indicators fully documented</t>
-  </si>
-  <si>
     <t xml:space="preserve">Patient 8</t>
   </si>
   <si>
+    <t xml:space="preserve">1. Initial visit with vague upper abdominal discomfort
+2. No prior PPI trial documented
+3. No H. pylori testing ordered</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Incomplete workup; no prior treatment failure documented and no alarm symptoms noted — insufficient basis for EGD approval</t>
+  </si>
+  <si>
     <t xml:space="preserve">1. PPI therapy (omeprazole 20mg) documented for 8 weeks with no improvement
-2. H. pylori urea breath test: Positive</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Failed PPI trial documented; positive H. pylori confirmed; dysphagia reported in clinical note</t>
-  </si>
-  <si>
-    <t xml:space="preserve">3. Physician note confirming dysphagia and 8 lb unintentional weight loss</t>
-  </si>
-  <si>
-    <t xml:space="preserve">All alarm symptom criteria and prior treatment failure documented — high likelihood of approval</t>
+2. H. pylori urea breath test: Positive
+3. Physician note confirming dysphagia and 8 lb unintentional weight loss</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Failed PPI trial documented; positive H. pylori confirmed; alarm symptoms (dysphagia, weight loss) present — all criteria met</t>
   </si>
   <si>
     <t xml:space="preserve">Patient 9</t>
   </si>
   <si>
+    <t xml:space="preserve">1. Patient age 38 with no family history documented
+2. Single episode of loose stool reported
+3. No prior imaging or lab workup</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Patient under age 45; no family history, no prior polyps, no IBD; single non-specific symptom — no qualifying high-risk criterion present</t>
+  </si>
+  <si>
     <t xml:space="preserve">1. Patient age 52 with documented family history of colorectal cancer (parent)
-2. Prior adenomatous polyp removal 5 years ago</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Age criteria met; high-risk family history confirmed; prior polyp history documented</t>
-  </si>
-  <si>
-    <t xml:space="preserve">3. Gastroenterologist order with medical necessity justification for surveillance colonoscopy</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Multiple high-risk indicators confirmed with specialist order — strong approval likelihood</t>
+2. Prior adenomatous polyp removal 5 years ago
+3. Gastroenterologist order with medical necessity justification for surveillance colonoscopy</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Age criteria met; high-risk family history confirmed; prior polyp history documented with specialist order</t>
   </si>
   <si>
     <t xml:space="preserve">Patient 10</t>
@@ -439,16 +451,42 @@
     <t xml:space="preserve">Mifepristone (Abortion Medication)</t>
   </si>
   <si>
-    <t xml:space="preserve">1. Confirmed intrauterine pregnancy ≤10 weeks gestation via ultrasound</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Gestational age confirmed within FDA-approved window; patient counseled and consented; mifepristone prescribed per protocol</t>
+    <t xml:space="preserve">1. Confirmed intrauterine pregnancy ≤10 weeks gestation via ultrasound
+2. No REMS provider certification on file
+3. No informed consent documentation present</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Gestational age confirmed within FDA window; however, REMS certification and informed consent are absent — mandatory criteria not met</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Requires confirmed intrauterine pregnancy ≤10 weeks gestation; provider must be certified under REMS program; documentation of informed consent and patient counseling. Rejection issued when REMS certification or consent documentation is absent.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1. Confirmed intrauterine pregnancy ≤10 weeks gestation via ultrasound
+2. REMS-certified provider attestation on file
+3. Informed consent signed</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Gestational age confirmed; REMS criteria met; consent documented — sufficient for approval; follow-up plan pending</t>
   </si>
   <si>
     <t xml:space="preserve">Requires confirmed intrauterine pregnancy ≤10 weeks gestation; provider must be certified under REMS program; documentation of informed consent and patient counseling</t>
   </si>
   <si>
-    <t xml:space="preserve">2. REMS-certified provider attestation on file
+    <t xml:space="preserve">Patient 11</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Physical Therapy</t>
+  </si>
+  <si>
+    <t>97110</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Therapeutic Exercise (Post-injury Physiotherapy)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1. Confirmed intrauterine pregnancy ≤10 weeks gestation via ultrasound
+2. REMS-certified provider attestation on file
 3. Informed consent signed
 4. Follow-up plan documented</t>
   </si>
@@ -456,41 +494,73 @@
     <t xml:space="preserve">All FDA REMS criteria met; gestational age confirmed; full protocol documentation present</t>
   </si>
   <si>
-    <t xml:space="preserve">Patient 11</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Physical Therapy</t>
-  </si>
-  <si>
-    <t>97110</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Therapeutic Exercise (Post-injury Physiotherapy)</t>
-  </si>
-  <si>
     <t xml:space="preserve">1. ER visit report: acute knee sprain sustained during basketball game
-2. MRI confirming Grade II MCL tear
-3. Orthopedic physician referral for physical therapy</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Acute sports injury documented with imaging; orthopedic referral with PT order specifying diagnosis, frequency, and duration; functional impairment noted</t>
+2. MRI confirming Grade II MCL tear</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Injury and imaging documented; however, no physician referral with diagnosis code and no PT treatment plan specifying frequency or duration — key required elements missing</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Requires physician referral with diagnosis code, imaging or clinical documentation of injury, PT evaluation with functional goals, and treatment plan specifying visit frequency and expected duration. Rejection issued when referral or treatment plan is absent.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Patient 12</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Colonoscopy with Biopsy, Single or Multiple</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1. Orthopedic physician referral for physical therapy with diagnosis code
+2. PT evaluation with measurable functional goals
+3. Treatment plan: 2x/week for 8 weeks</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Complete documentation package with referral, imaging, PT evaluation and treatment plan — all criteria met</t>
   </si>
   <si>
     <t xml:space="preserve">Requires physician referral with diagnosis code, imaging or clinical documentation of injury, PT evaluation with functional goals, and treatment plan specifying visit frequency and expected duration</t>
   </si>
   <si>
-    <t xml:space="preserve">4. PT evaluation with measurable functional goals
-5. Treatment plan: 2x/week for 8 weeks</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Complete documentation package with referral, imaging, and PT treatment plan — high approval likelihood</t>
+    <t xml:space="preserve">Patient 13</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1. Patient complaint of intermittent lower abdominal pain and irregular bowel habits</t>
+  </si>
+  <si>
+    <t xml:space="preserve">New patient with no prior colonoscopy; no imaging or lab results provided; no documentation of high-risk indicators, positive FOBT, or symptomatic workup — no qualifying criterion met</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Requires documented symptomatic indicators (rectal bleeding, chronic diarrhea, abdominal pain with inconclusive workup) or high-risk criteria (age 45+, family history of CRC, prior polyps, IBD); positive FOBT or abnormal finding must be noted to justify biopsy. Rejection issued when no qualifying symptom or risk factor is documented.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Esophagogastroduodenoscopy (EGD), Diagnostic</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1. Positive fecal occult blood test (FOBT) documented
+2. Colonoscopy findings showing suspicious mucosal irregularity in descending colon
+3. Physician order with medical necessity justification for biopsy</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Positive FOBT with visible mucosal abnormality identified during scope; biopsy medically justified with complete documentation</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Requires documented symptomatic indicators (rectal bleeding, chronic diarrhea, abdominal pain with inconclusive workup) or high-risk criteria (age 45+, family history of CRC, prior polyps, IBD); abnormal finding or positive FOBT must be noted to justify biopsy</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1. Patient presents with occasional mild nausea</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Vague, non-specific symptom only; no prior PPI trial, no imaging, no alarm symptoms documented — insufficient clinical justification for diagnostic EGD</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Requires documented alarm symptoms (dysphagia, odynophagia, unexplained weight loss, hematemesis, melena) OR failed conservative treatment (PPI trial min. 4–8 weeks). Rejection issued when only vague, non-specific symptoms are present with no prior workup.</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
-  <fonts count="4">
+  <fonts count="6">
     <font>
       <sz val="11.000000"/>
       <color theme="1"/>
@@ -512,6 +582,17 @@
       <sz val="12.000000"/>
       <color indexed="64"/>
       <name val="Times"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="12.000000"/>
+      <color indexed="64"/>
+      <name val="Times"/>
+    </font>
+    <font>
+      <sz val="11.000000"/>
+      <color indexed="64"/>
+      <name val="Aptos Narrow"/>
     </font>
   </fonts>
   <fills count="4">
@@ -611,7 +692,7 @@
   <cellStyleXfs count="1">
     <xf fontId="0" fillId="0" borderId="0" numFmtId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
   </cellStyleXfs>
-  <cellXfs count="38">
+  <cellXfs count="47">
     <xf fontId="0" fillId="0" borderId="0" numFmtId="0" xfId="0"/>
     <xf fontId="0" fillId="0" borderId="0" numFmtId="0" xfId="0" applyAlignment="1">
       <alignment vertical="center"/>
@@ -677,50 +758,77 @@
     <xf fontId="0" fillId="0" borderId="1" numFmtId="0" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf fontId="0" fillId="0" borderId="0" numFmtId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf fontId="0" fillId="0" borderId="0" numFmtId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf fontId="1" fillId="0" borderId="0" numFmtId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf fontId="1" fillId="2" borderId="1" numFmtId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf fontId="1" fillId="2" borderId="1" numFmtId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
     <xf fontId="2" fillId="0" borderId="1" numFmtId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf fontId="2" fillId="0" borderId="4" numFmtId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf fontId="2" fillId="0" borderId="4" numFmtId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf fontId="2" fillId="0" borderId="1" numFmtId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf fontId="2" fillId="0" borderId="1" numFmtId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf fontId="2" fillId="0" borderId="1" numFmtId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf fontId="2" fillId="0" borderId="2" numFmtId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf fontId="2" fillId="0" borderId="2" numFmtId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf fontId="0" fillId="0" borderId="4" numFmtId="0" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf fontId="0" fillId="0" borderId="1" numFmtId="0" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf fontId="0" fillId="0" borderId="1" numFmtId="0" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
     </xf>
     <xf fontId="2" fillId="0" borderId="0" numFmtId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf fontId="2" fillId="0" borderId="5" numFmtId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf fontId="2" fillId="0" borderId="5" numFmtId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf fontId="2" fillId="0" borderId="3" numFmtId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf fontId="2" fillId="0" borderId="3" numFmtId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf fontId="0" fillId="0" borderId="5" numFmtId="0" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf fontId="3" fillId="0" borderId="1" numFmtId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf fontId="3" fillId="0" borderId="4" numFmtId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf fontId="3" fillId="0" borderId="5" numFmtId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
     <xf fontId="2" fillId="0" borderId="0" numFmtId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf fontId="2" fillId="0" borderId="0" numFmtId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf fontId="2" fillId="0" borderId="0" numFmtId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf fontId="2" fillId="0" borderId="0" numFmtId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf fontId="2" fillId="0" borderId="0" numFmtId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf fontId="0" fillId="0" borderId="0" numFmtId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf fontId="0" fillId="0" borderId="1" numFmtId="0" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf fontId="4" fillId="0" borderId="0" numFmtId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
     <xf fontId="3" fillId="0" borderId="0" numFmtId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf fontId="5" fillId="0" borderId="0" numFmtId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -2207,359 +2315,709 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac">
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultRowHeight="14.25"/>
   <cols>
-    <col customWidth="1" min="1" max="1" style="2" width="12"/>
-    <col bestFit="1" customWidth="1" min="2" max="2" style="2" width="11.85546875"/>
-    <col min="3" max="3" style="2" width="9.140625"/>
-    <col customWidth="1" min="4" max="4" style="4" width="42.85546875"/>
-    <col customWidth="1" min="5" max="5" style="3" width="42.85546875"/>
-    <col customWidth="1" min="6" max="6" style="4" width="30.85546875"/>
-    <col bestFit="1" customWidth="1" min="7" max="7" style="1" width="17.5703125"/>
-    <col customWidth="1" min="8" max="8" style="4" width="46.42578125"/>
-    <col min="9" max="16384" style="1" width="9.140625"/>
+    <col customWidth="1" min="1" max="1" style="23" width="12"/>
+    <col bestFit="1" customWidth="1" min="2" max="2" style="23" width="11.85546875"/>
+    <col min="3" max="3" style="23" width="9.140625"/>
+    <col customWidth="1" min="4" max="5" style="24" width="42.85546875"/>
+    <col customWidth="1" min="6" max="6" style="24" width="30.85546875"/>
+    <col bestFit="1" customWidth="1" min="7" max="7" style="23" width="17.5703125"/>
+    <col customWidth="1" min="8" max="8" style="24" width="46.42578125"/>
+    <col min="9" max="16384" style="23" width="9.140625"/>
   </cols>
   <sheetData>
-    <row r="1" s="5" customFormat="1">
-      <c r="A1" s="6" t="s">
+    <row r="1" s="25" customFormat="1">
+      <c r="A1" s="26" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="6" t="s">
+      <c r="B1" s="26" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="6" t="s">
+      <c r="C1" s="26" t="s">
         <v>102</v>
       </c>
-      <c r="D1" s="7" t="s">
+      <c r="D1" s="27" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="7" t="s">
+      <c r="E1" s="27" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="7" t="s">
+      <c r="F1" s="27" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="6" t="s">
+      <c r="G1" s="26" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="6" t="s">
+      <c r="H1" s="26" t="s">
         <v>7</v>
       </c>
     </row>
-    <row r="2" ht="27.75" customHeight="1">
-      <c r="A2" s="23" t="s">
+    <row r="2" ht="57">
+      <c r="A2" s="28" t="s">
         <v>103</v>
       </c>
-      <c r="B2" s="24" t="s">
+      <c r="B2" s="29" t="s">
         <v>104</v>
       </c>
-      <c r="C2" s="25" t="s">
+      <c r="C2" s="30" t="s">
         <v>105</v>
       </c>
-      <c r="D2" s="24" t="s">
+      <c r="D2" s="31" t="s">
         <v>106</v>
       </c>
-      <c r="E2" s="26" t="s">
+      <c r="E2" s="32" t="s">
         <v>107</v>
       </c>
-      <c r="F2" s="27" t="s">
+      <c r="F2" s="32" t="s">
         <v>108</v>
       </c>
-      <c r="G2" s="28" t="s">
+      <c r="G2" s="33" t="s">
         <v>13</v>
       </c>
-      <c r="H2" s="26" t="s">
+      <c r="H2" s="32" t="s">
         <v>109</v>
       </c>
-      <c r="I2" s="29">
+      <c r="I2" s="34">
         <v>260</v>
       </c>
-      <c r="J2" s="1"/>
+      <c r="J2" s="23"/>
     </row>
     <row r="3" ht="50.25" customHeight="1">
-      <c r="A3" s="23" t="s">
+      <c r="A3" s="28" t="s">
         <v>103</v>
       </c>
-      <c r="B3" s="30"/>
-      <c r="C3" s="31"/>
-      <c r="D3" s="30"/>
-      <c r="E3" s="26" t="s">
+      <c r="B3" s="35"/>
+      <c r="C3" s="36"/>
+      <c r="D3" s="37"/>
+      <c r="E3" s="32" t="s">
         <v>110</v>
       </c>
-      <c r="F3" s="27" t="s">
+      <c r="F3" s="32" t="s">
         <v>111</v>
       </c>
-      <c r="G3" s="28" t="s">
+      <c r="G3" s="33" t="s">
         <v>17</v>
       </c>
-      <c r="H3" s="20"/>
-      <c r="I3" s="29">
+      <c r="H3" s="32" t="s">
+        <v>112</v>
+      </c>
+      <c r="I3" s="34">
         <v>261</v>
       </c>
-      <c r="J3" s="1"/>
-    </row>
-    <row r="4">
-      <c r="A4" s="23" t="s">
+      <c r="J3" s="23"/>
+    </row>
+    <row r="4" ht="71.25">
+      <c r="A4" s="28" t="s">
+        <v>113</v>
+      </c>
+      <c r="B4" s="29" t="s">
+        <v>104</v>
+      </c>
+      <c r="C4" s="30" t="s">
+        <v>114</v>
+      </c>
+      <c r="D4" s="31" t="s">
+        <v>115</v>
+      </c>
+      <c r="E4" s="32" t="s">
+        <v>116</v>
+      </c>
+      <c r="F4" s="32" t="s">
+        <v>117</v>
+      </c>
+      <c r="G4" s="33" t="s">
+        <v>13</v>
+      </c>
+      <c r="H4" s="32" t="s">
+        <v>118</v>
+      </c>
+      <c r="I4" s="34">
+        <v>262</v>
+      </c>
+      <c r="J4" s="23"/>
+    </row>
+    <row r="5" ht="57">
+      <c r="A5" s="28" t="s">
+        <v>113</v>
+      </c>
+      <c r="B5" s="35"/>
+      <c r="C5" s="36"/>
+      <c r="D5" s="37"/>
+      <c r="E5" s="32" t="s">
+        <v>119</v>
+      </c>
+      <c r="F5" s="32" t="s">
+        <v>120</v>
+      </c>
+      <c r="G5" s="33" t="s">
+        <v>17</v>
+      </c>
+      <c r="H5" s="32" t="s">
+        <v>121</v>
+      </c>
+      <c r="I5" s="34">
+        <v>263</v>
+      </c>
+      <c r="J5" s="23"/>
+    </row>
+    <row r="6" ht="57">
+      <c r="A6" s="28" t="s">
+        <v>122</v>
+      </c>
+      <c r="B6" s="29" t="s">
+        <v>104</v>
+      </c>
+      <c r="C6" s="30" t="s">
+        <v>105</v>
+      </c>
+      <c r="D6" s="31" t="s">
+        <v>106</v>
+      </c>
+      <c r="E6" s="32" t="s">
+        <v>123</v>
+      </c>
+      <c r="F6" s="32" t="s">
+        <v>124</v>
+      </c>
+      <c r="G6" s="33" t="s">
+        <v>13</v>
+      </c>
+      <c r="H6" s="32" t="s">
+        <v>109</v>
+      </c>
+      <c r="I6" s="34">
+        <v>264</v>
+      </c>
+      <c r="J6" s="23"/>
+    </row>
+    <row r="7" ht="108.75">
+      <c r="A7" s="28" t="s">
+        <v>122</v>
+      </c>
+      <c r="B7" s="35"/>
+      <c r="C7" s="36"/>
+      <c r="D7" s="37"/>
+      <c r="E7" s="38" t="s">
+        <v>125</v>
+      </c>
+      <c r="F7" s="38" t="s">
+        <v>126</v>
+      </c>
+      <c r="G7" s="38" t="s">
+        <v>17</v>
+      </c>
+      <c r="H7" s="38" t="s">
         <v>112</v>
       </c>
-      <c r="B4" s="24" t="s">
+      <c r="I7" s="34">
+        <v>265</v>
+      </c>
+      <c r="J7" s="23"/>
+    </row>
+    <row r="8" ht="108.75">
+      <c r="A8" s="28" t="s">
+        <v>127</v>
+      </c>
+      <c r="B8" s="29" t="s">
         <v>104</v>
       </c>
-      <c r="C4" s="25" t="s">
-        <v>113</v>
-      </c>
-      <c r="D4" s="24" t="s">
+      <c r="C8" s="30" t="s">
         <v>114</v>
       </c>
-      <c r="E4" s="26" t="s">
+      <c r="D8" s="39" t="s">
         <v>115</v>
       </c>
-      <c r="F4" s="27" t="s">
-        <v>116</v>
-      </c>
-      <c r="G4" s="28" t="s">
+      <c r="E8" s="38" t="s">
+        <v>128</v>
+      </c>
+      <c r="F8" s="38" t="s">
+        <v>129</v>
+      </c>
+      <c r="G8" s="38" t="s">
         <v>13</v>
       </c>
-      <c r="H4" s="26" t="s">
-        <v>117</v>
-      </c>
-      <c r="I4" s="29">
-        <v>262</v>
-      </c>
-      <c r="J4" s="1"/>
-    </row>
-    <row r="5" ht="43.5">
-      <c r="A5" s="23" t="s">
-        <v>112</v>
-      </c>
-      <c r="B5" s="30"/>
-      <c r="C5" s="31"/>
-      <c r="D5" s="30"/>
-      <c r="E5" s="26" t="s">
+      <c r="H8" s="38" t="s">
         <v>118</v>
       </c>
-      <c r="F5" s="27" t="s">
-        <v>119</v>
-      </c>
-      <c r="G5" s="28" t="s">
+      <c r="I8" s="34">
+        <v>266</v>
+      </c>
+      <c r="J8" s="23"/>
+    </row>
+    <row r="9" ht="108.75">
+      <c r="A9" s="28" t="s">
+        <v>127</v>
+      </c>
+      <c r="B9" s="35"/>
+      <c r="C9" s="36"/>
+      <c r="D9" s="40"/>
+      <c r="E9" s="38" t="s">
+        <v>130</v>
+      </c>
+      <c r="F9" s="38" t="s">
+        <v>131</v>
+      </c>
+      <c r="G9" s="38" t="s">
         <v>17</v>
       </c>
-      <c r="H5" s="20"/>
-      <c r="I5" s="29">
-        <v>263</v>
-      </c>
-      <c r="J5" s="1"/>
-    </row>
-    <row r="6" ht="29.25" customHeight="1">
-      <c r="A6" s="23" t="s">
-        <v>120</v>
-      </c>
-      <c r="B6" s="24" t="s">
+      <c r="H9" s="38" t="s">
+        <v>121</v>
+      </c>
+      <c r="I9" s="34">
+        <v>267</v>
+      </c>
+      <c r="J9" s="23"/>
+    </row>
+    <row r="10" ht="108.75">
+      <c r="A10" s="28" t="s">
+        <v>132</v>
+      </c>
+      <c r="B10" s="29" t="s">
+        <v>133</v>
+      </c>
+      <c r="C10" s="30" t="s">
+        <v>134</v>
+      </c>
+      <c r="D10" s="39" t="s">
+        <v>135</v>
+      </c>
+      <c r="E10" s="38" t="s">
+        <v>136</v>
+      </c>
+      <c r="F10" s="38" t="s">
+        <v>137</v>
+      </c>
+      <c r="G10" s="38" t="s">
+        <v>13</v>
+      </c>
+      <c r="H10" s="38" t="s">
+        <v>138</v>
+      </c>
+      <c r="I10" s="34">
+        <v>268</v>
+      </c>
+      <c r="J10" s="23"/>
+    </row>
+    <row r="11" ht="87">
+      <c r="A11" s="28" t="s">
+        <v>132</v>
+      </c>
+      <c r="B11" s="35"/>
+      <c r="C11" s="36"/>
+      <c r="D11" s="40"/>
+      <c r="E11" s="38" t="s">
+        <v>139</v>
+      </c>
+      <c r="F11" s="38" t="s">
+        <v>140</v>
+      </c>
+      <c r="G11" s="38" t="s">
+        <v>21</v>
+      </c>
+      <c r="H11" s="38" t="s">
+        <v>141</v>
+      </c>
+      <c r="I11" s="34">
+        <v>269</v>
+      </c>
+      <c r="J11" s="23"/>
+    </row>
+    <row r="12" ht="71.25">
+      <c r="A12" s="34" t="s">
+        <v>142</v>
+      </c>
+      <c r="B12" s="41" t="s">
+        <v>143</v>
+      </c>
+      <c r="C12" s="34" t="s">
+        <v>144</v>
+      </c>
+      <c r="D12" s="42" t="s">
+        <v>145</v>
+      </c>
+      <c r="E12" s="24" t="s">
+        <v>146</v>
+      </c>
+      <c r="F12" s="24" t="s">
+        <v>147</v>
+      </c>
+      <c r="G12" s="33" t="s">
+        <v>17</v>
+      </c>
+      <c r="H12" s="24" t="s">
+        <v>141</v>
+      </c>
+      <c r="I12" s="34">
+        <v>270</v>
+      </c>
+    </row>
+    <row r="13" ht="71.25">
+      <c r="A13" s="34" t="s">
+        <v>142</v>
+      </c>
+      <c r="B13" s="41"/>
+      <c r="C13" s="34"/>
+      <c r="D13" s="42"/>
+      <c r="E13" s="24" t="s">
+        <v>148</v>
+      </c>
+      <c r="F13" s="24" t="s">
+        <v>149</v>
+      </c>
+      <c r="G13" s="33" t="s">
+        <v>13</v>
+      </c>
+      <c r="H13" s="24" t="s">
+        <v>150</v>
+      </c>
+      <c r="I13" s="34">
+        <v>271</v>
+      </c>
+    </row>
+    <row r="14" ht="71.25">
+      <c r="A14" s="28" t="s">
+        <v>151</v>
+      </c>
+      <c r="B14" s="29" t="s">
         <v>104</v>
       </c>
-      <c r="C6" s="25" t="s">
-        <v>105</v>
-      </c>
-      <c r="D6" s="24" t="s">
-        <v>106</v>
-      </c>
-      <c r="E6" s="26" t="s">
-        <v>121</v>
-      </c>
-      <c r="F6" s="27" t="s">
-        <v>122</v>
-      </c>
-      <c r="G6" s="28" t="s">
+      <c r="C14" s="30">
+        <v>45380</v>
+      </c>
+      <c r="D14" s="31" t="s">
+        <v>152</v>
+      </c>
+      <c r="E14" s="32" t="s">
+        <v>153</v>
+      </c>
+      <c r="F14" s="32" t="s">
+        <v>154</v>
+      </c>
+      <c r="G14" s="33" t="s">
         <v>17</v>
       </c>
-      <c r="H6" s="26" t="s">
-        <v>109</v>
-      </c>
-      <c r="I6" s="29">
-        <v>264</v>
-      </c>
-      <c r="J6" s="1"/>
-    </row>
-    <row r="7">
-      <c r="A7" s="23" t="s">
-        <v>120</v>
-      </c>
-      <c r="B7" s="30"/>
-      <c r="C7" s="31"/>
-      <c r="D7" s="30"/>
-      <c r="E7" s="26" t="s">
-        <v>123</v>
-      </c>
-      <c r="F7" s="27" t="s">
-        <v>124</v>
-      </c>
-      <c r="G7" s="28" t="s">
-        <v>78</v>
-      </c>
-      <c r="H7" s="20"/>
-      <c r="I7" s="29">
-        <v>265</v>
-      </c>
-      <c r="J7" s="1"/>
-    </row>
-    <row r="8">
-      <c r="A8" s="23" t="s">
-        <v>125</v>
-      </c>
-      <c r="B8" s="24" t="s">
+      <c r="H14" s="32" t="s">
+        <v>155</v>
+      </c>
+      <c r="I14" s="34">
+        <v>272</v>
+      </c>
+    </row>
+    <row r="15" ht="99.75">
+      <c r="A15" s="28" t="s">
+        <v>156</v>
+      </c>
+      <c r="B15" s="35"/>
+      <c r="C15" s="36"/>
+      <c r="D15" s="37"/>
+      <c r="E15" s="32" t="s">
+        <v>157</v>
+      </c>
+      <c r="F15" s="32" t="s">
+        <v>158</v>
+      </c>
+      <c r="G15" s="33" t="s">
+        <v>13</v>
+      </c>
+      <c r="H15" s="43" t="s">
+        <v>159</v>
+      </c>
+      <c r="I15" s="34">
+        <v>273</v>
+      </c>
+    </row>
+    <row r="16" ht="85.5">
+      <c r="A16" s="28" t="s">
+        <v>151</v>
+      </c>
+      <c r="B16" s="29" t="s">
         <v>104</v>
       </c>
-      <c r="C8" s="25" t="s">
-        <v>113</v>
-      </c>
-      <c r="D8" s="24" t="s">
-        <v>114</v>
-      </c>
-      <c r="E8" s="26" t="s">
-        <v>126</v>
-      </c>
-      <c r="F8" s="27" t="s">
-        <v>127</v>
-      </c>
-      <c r="G8" s="28" t="s">
+      <c r="C16" s="30">
+        <v>43235</v>
+      </c>
+      <c r="D16" s="31" t="s">
+        <v>160</v>
+      </c>
+      <c r="E16" s="32" t="s">
+        <v>161</v>
+      </c>
+      <c r="F16" s="32" t="s">
+        <v>162</v>
+      </c>
+      <c r="G16" s="33" t="s">
         <v>17</v>
       </c>
-      <c r="H8" s="26" t="s">
-        <v>117</v>
-      </c>
-      <c r="I8" s="29">
-        <v>266</v>
-      </c>
-      <c r="J8" s="1"/>
-    </row>
-    <row r="9" ht="29.25">
-      <c r="A9" s="23" t="s">
-        <v>125</v>
-      </c>
-      <c r="B9" s="30"/>
-      <c r="C9" s="31"/>
-      <c r="D9" s="30"/>
-      <c r="E9" s="26" t="s">
-        <v>128</v>
-      </c>
-      <c r="F9" s="27" t="s">
-        <v>129</v>
-      </c>
-      <c r="G9" s="28" t="s">
-        <v>78</v>
-      </c>
-      <c r="H9" s="20"/>
-      <c r="I9" s="29">
-        <v>267</v>
-      </c>
-      <c r="J9" s="1"/>
-    </row>
-    <row r="10" ht="18.75" customHeight="1">
-      <c r="A10" s="23" t="s">
-        <v>130</v>
-      </c>
-      <c r="B10" s="24" t="s">
-        <v>131</v>
-      </c>
-      <c r="C10" s="25" t="s">
-        <v>132</v>
-      </c>
-      <c r="D10" s="24" t="s">
-        <v>133</v>
-      </c>
-      <c r="E10" s="26" t="s">
-        <v>134</v>
-      </c>
-      <c r="F10" s="27" t="s">
-        <v>135</v>
-      </c>
-      <c r="G10" s="28" t="s">
-        <v>17</v>
-      </c>
-      <c r="H10" s="26" t="s">
-        <v>136</v>
-      </c>
-      <c r="I10" s="29">
-        <v>268</v>
-      </c>
-      <c r="J10" s="1"/>
-    </row>
-    <row r="11" ht="29.25" customHeight="1">
-      <c r="A11" s="23" t="s">
-        <v>130</v>
-      </c>
-      <c r="B11" s="30"/>
-      <c r="C11" s="31"/>
-      <c r="D11" s="30"/>
-      <c r="E11" s="26" t="s">
-        <v>137</v>
-      </c>
-      <c r="F11" s="27" t="s">
-        <v>138</v>
-      </c>
-      <c r="G11" s="28" t="s">
-        <v>78</v>
-      </c>
-      <c r="H11" s="20"/>
-      <c r="I11" s="29">
-        <v>269</v>
-      </c>
-      <c r="J11" s="1"/>
-    </row>
-    <row r="12" ht="15">
-      <c r="A12" s="32" t="s">
-        <v>139</v>
-      </c>
-      <c r="B12" s="33" t="s">
-        <v>140</v>
-      </c>
-      <c r="C12" s="34" t="s">
-        <v>141</v>
-      </c>
-      <c r="D12" s="33" t="s">
-        <v>142</v>
-      </c>
-      <c r="E12" s="35" t="s">
-        <v>143</v>
-      </c>
-      <c r="F12" s="36" t="s">
-        <v>144</v>
-      </c>
-      <c r="G12" s="29" t="s">
-        <v>17</v>
-      </c>
-      <c r="H12" s="35" t="s">
-        <v>145</v>
-      </c>
-      <c r="I12" s="29">
-        <v>270</v>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" s="32" t="s">
-        <v>139</v>
-      </c>
-      <c r="B13" s="33"/>
-      <c r="C13" s="34"/>
-      <c r="D13" s="33"/>
-      <c r="E13" s="35" t="s">
-        <v>146</v>
-      </c>
-      <c r="F13" s="36" t="s">
-        <v>147</v>
-      </c>
-      <c r="G13" s="29" t="s">
-        <v>78</v>
-      </c>
-      <c r="I13" s="29">
-        <v>271</v>
-      </c>
-    </row>
-    <row r="14" ht="15">
-      <c r="A14" s="37"/>
+      <c r="H16" s="32" t="s">
+        <v>163</v>
+      </c>
+      <c r="I16" s="34">
+        <v>274</v>
+      </c>
+    </row>
+    <row r="17" ht="71.25">
+      <c r="A17" s="28" t="s">
+        <v>156</v>
+      </c>
+      <c r="B17" s="35"/>
+      <c r="C17" s="36"/>
+      <c r="D17" s="37"/>
+      <c r="E17" s="32" t="s">
+        <v>164</v>
+      </c>
+      <c r="F17" s="32" t="s">
+        <v>165</v>
+      </c>
+      <c r="G17" s="33" t="s">
+        <v>13</v>
+      </c>
+      <c r="H17" s="32" t="s">
+        <v>166</v>
+      </c>
+      <c r="I17" s="34">
+        <v>275</v>
+      </c>
+    </row>
+    <row r="18" ht="14.25">
+      <c r="A18" s="23"/>
+      <c r="B18" s="23"/>
+      <c r="C18" s="23"/>
+      <c r="D18" s="24"/>
+      <c r="E18" s="24"/>
+      <c r="F18" s="24"/>
+      <c r="G18" s="23"/>
+      <c r="H18" s="24"/>
+      <c r="I18" s="23"/>
+    </row>
+    <row r="19" ht="14.25">
+      <c r="A19" s="23"/>
+      <c r="B19" s="23"/>
+      <c r="C19" s="23"/>
+      <c r="D19" s="24"/>
+      <c r="E19" s="24"/>
+      <c r="F19" s="24"/>
+      <c r="G19" s="23"/>
+      <c r="H19" s="24"/>
+      <c r="I19" s="23"/>
+    </row>
+    <row r="20" ht="14.25">
+      <c r="A20" s="23"/>
+      <c r="B20" s="23"/>
+      <c r="C20" s="23"/>
+      <c r="D20" s="24"/>
+      <c r="E20" s="24"/>
+      <c r="F20" s="24"/>
+      <c r="G20" s="23"/>
+      <c r="H20" s="24"/>
+    </row>
+    <row r="21" ht="14.25">
+      <c r="A21" s="23"/>
+      <c r="B21" s="23"/>
+      <c r="C21" s="23"/>
+      <c r="D21" s="24"/>
+      <c r="E21" s="24"/>
+      <c r="F21" s="24"/>
+      <c r="G21" s="23"/>
+      <c r="H21" s="24"/>
+    </row>
+    <row r="22" ht="14.25">
+      <c r="A22" s="23"/>
+      <c r="B22" s="23"/>
+      <c r="C22" s="23"/>
+      <c r="D22" s="24"/>
+      <c r="E22" s="24"/>
+      <c r="F22" s="24"/>
+      <c r="G22" s="23"/>
+      <c r="H22" s="24"/>
+    </row>
+    <row r="23" ht="21.75">
+      <c r="A23" s="44"/>
+      <c r="B23" s="44"/>
+      <c r="C23" s="44"/>
+      <c r="D23" s="44"/>
+      <c r="E23" s="44"/>
+      <c r="F23" s="44"/>
+      <c r="G23" s="44"/>
+      <c r="H23" s="44"/>
+    </row>
+    <row r="24" ht="21.75">
+      <c r="A24" s="45"/>
+      <c r="B24" s="45"/>
+      <c r="C24" s="45"/>
+      <c r="D24" s="45"/>
+      <c r="E24" s="45"/>
+      <c r="F24" s="45"/>
+      <c r="G24" s="45"/>
+      <c r="H24" s="45"/>
+    </row>
+    <row r="25" ht="21.75">
+      <c r="A25" s="45"/>
+      <c r="B25" s="24"/>
+      <c r="C25" s="24"/>
+      <c r="D25" s="24"/>
+      <c r="E25" s="45"/>
+      <c r="F25" s="45"/>
+      <c r="G25" s="45"/>
+      <c r="H25" s="45"/>
+    </row>
+    <row r="26" ht="21.75">
+      <c r="A26" s="45"/>
+      <c r="B26" s="45"/>
+      <c r="C26" s="45"/>
+      <c r="D26" s="45"/>
+      <c r="E26" s="45"/>
+      <c r="F26" s="45"/>
+      <c r="G26" s="45"/>
+      <c r="H26" s="45"/>
+    </row>
+    <row r="27" ht="21.75">
+      <c r="A27" s="45"/>
+      <c r="B27" s="24"/>
+      <c r="C27" s="24"/>
+      <c r="D27" s="24"/>
+      <c r="E27" s="45"/>
+      <c r="F27" s="45"/>
+      <c r="G27" s="45"/>
+      <c r="H27" s="45"/>
+    </row>
+    <row r="28" ht="14.25">
+      <c r="A28" s="46"/>
+      <c r="B28" s="23"/>
+      <c r="C28" s="23"/>
+      <c r="D28" s="24"/>
+      <c r="E28" s="24"/>
+      <c r="F28" s="24"/>
+      <c r="G28" s="23"/>
+      <c r="H28" s="24"/>
+    </row>
+    <row r="29" ht="14.25">
+      <c r="A29" s="23"/>
+      <c r="B29" s="23"/>
+      <c r="C29" s="23"/>
+      <c r="D29" s="24"/>
+      <c r="E29" s="24"/>
+      <c r="F29" s="24"/>
+      <c r="G29" s="23"/>
+      <c r="H29" s="24"/>
+    </row>
+    <row r="30" ht="14.25">
+      <c r="A30" s="23"/>
+      <c r="B30" s="23"/>
+      <c r="C30" s="23"/>
+      <c r="D30" s="24"/>
+      <c r="E30" s="24"/>
+      <c r="F30" s="24"/>
+      <c r="G30" s="23"/>
+      <c r="H30" s="24"/>
+    </row>
+    <row r="31" ht="14.25">
+      <c r="A31" s="23"/>
+      <c r="B31" s="23"/>
+      <c r="C31" s="23"/>
+      <c r="D31" s="24"/>
+      <c r="E31" s="24"/>
+      <c r="F31" s="24"/>
+      <c r="G31" s="23"/>
+      <c r="H31" s="24"/>
+    </row>
+    <row r="32" ht="14.25">
+      <c r="A32" s="23"/>
+      <c r="B32" s="23"/>
+      <c r="C32" s="23"/>
+      <c r="D32" s="24"/>
+      <c r="E32" s="24"/>
+      <c r="F32" s="24"/>
+      <c r="G32" s="23"/>
+      <c r="H32" s="24"/>
+    </row>
+    <row r="33" ht="14.25">
+      <c r="A33" s="23"/>
+      <c r="B33" s="23"/>
+      <c r="C33" s="23"/>
+      <c r="D33" s="24"/>
+      <c r="E33" s="24"/>
+      <c r="F33" s="24"/>
+      <c r="G33" s="23"/>
+      <c r="H33" s="24"/>
+    </row>
+    <row r="34" ht="14.25">
+      <c r="A34" s="23"/>
+      <c r="B34" s="23"/>
+      <c r="C34" s="23"/>
+      <c r="D34" s="24"/>
+      <c r="E34" s="24"/>
+      <c r="F34" s="24"/>
+      <c r="G34" s="23"/>
+      <c r="H34" s="24"/>
+    </row>
+    <row r="35" ht="14.25">
+      <c r="A35" s="23"/>
+    </row>
+    <row r="36" ht="14.25">
+      <c r="A36" s="23"/>
+    </row>
+    <row r="37" ht="14.25">
+      <c r="A37" s="23"/>
+    </row>
+    <row r="38" ht="14.25">
+      <c r="A38" s="23"/>
+    </row>
+    <row r="39" ht="14.25">
+      <c r="A39" s="23"/>
+    </row>
+    <row r="40" ht="14.25">
+      <c r="A40" s="23"/>
+    </row>
+    <row r="41" ht="14.25">
+      <c r="A41" s="23"/>
+      <c r="B41" s="23"/>
+      <c r="C41" s="23"/>
+      <c r="D41" s="24"/>
+      <c r="E41" s="24"/>
+      <c r="F41" s="24"/>
+      <c r="G41" s="23"/>
+      <c r="H41" s="24"/>
+    </row>
+    <row r="42" ht="14.25">
+      <c r="A42" s="23"/>
+      <c r="B42" s="23"/>
+      <c r="C42" s="23"/>
+      <c r="D42" s="24"/>
+      <c r="E42" s="24"/>
+      <c r="F42" s="24"/>
+      <c r="G42" s="23"/>
+      <c r="H42" s="24"/>
+    </row>
+    <row r="43" ht="14.25">
+      <c r="A43" s="23"/>
+      <c r="E43" s="24"/>
+      <c r="F43" s="24"/>
+      <c r="G43" s="23"/>
+      <c r="H43" s="24"/>
+    </row>
+    <row r="44" ht="14.25">
+      <c r="A44" s="23"/>
+      <c r="B44" s="23"/>
+      <c r="C44" s="23"/>
+      <c r="D44" s="24"/>
+      <c r="E44" s="24"/>
+      <c r="F44" s="24"/>
+      <c r="G44" s="23"/>
+      <c r="H44" s="24"/>
+    </row>
+    <row r="45" ht="14.25">
+      <c r="A45" s="23"/>
+      <c r="E45" s="24"/>
+      <c r="F45" s="24"/>
+      <c r="G45" s="23"/>
+      <c r="H45" s="24"/>
+    </row>
+    <row r="46" ht="14.25">
+      <c r="A46" s="23"/>
     </row>
   </sheetData>
-  <mergeCells count="18">
+  <mergeCells count="24">
     <mergeCell ref="B2:B3"/>
     <mergeCell ref="C2:C3"/>
     <mergeCell ref="D2:D3"/>
@@ -2578,6 +3036,12 @@
     <mergeCell ref="B12:B13"/>
     <mergeCell ref="C12:C13"/>
     <mergeCell ref="D12:D13"/>
+    <mergeCell ref="B14:B15"/>
+    <mergeCell ref="C14:C15"/>
+    <mergeCell ref="D14:D15"/>
+    <mergeCell ref="B16:B17"/>
+    <mergeCell ref="C16:C17"/>
+    <mergeCell ref="D16:D17"/>
   </mergeCells>
   <printOptions headings="0" gridLines="0"/>
   <pageMargins left="0.69999999999999996" right="0.69999999999999996" top="0.75" bottom="0.75" header="0.29999999999999999" footer="0.29999999999999999"/>

</xml_diff>

<commit_message>
implement insurance verification workflow and enhance patient data handling
</commit_message>
<xml_diff>
--- a/core/UAT Plan.xlsx
+++ b/core/UAT Plan.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <workbookPr/>
   <bookViews>
-    <workbookView xWindow="360" yWindow="15" windowWidth="20955" windowHeight="9720" activeTab="3"/>
+    <workbookView xWindow="360" yWindow="15" windowWidth="20955" windowHeight="9720" activeTab="1"/>
   </bookViews>
   <sheets>
     <sheet name="Demo person 1" sheetId="1" state="visible" r:id="rId4"/>
@@ -238,6 +238,9 @@
 3. Documentation of Abnormal Renal mass</t>
   </si>
   <si>
+    <t xml:space="preserve">Patient 6</t>
+  </si>
+  <si>
     <t xml:space="preserve">Oral and Maxillofacial Surgery</t>
   </si>
   <si>
@@ -338,9 +341,6 @@
   </si>
   <si>
     <t>Code</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Patient 6</t>
   </si>
   <si>
     <t>Gastroenterology</t>
@@ -560,7 +560,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
-  <fonts count="6">
+  <fonts count="5">
     <font>
       <sz val="11.000000"/>
       <color theme="1"/>
@@ -580,19 +580,12 @@
     </font>
     <font>
       <sz val="12.000000"/>
-      <color indexed="64"/>
       <name val="Times"/>
     </font>
     <font>
       <b/>
       <sz val="12.000000"/>
-      <color indexed="64"/>
       <name val="Times"/>
-    </font>
-    <font>
-      <sz val="11.000000"/>
-      <color indexed="64"/>
-      <name val="Aptos Narrow"/>
     </font>
   </fonts>
   <fills count="4">
@@ -613,7 +606,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="6">
+  <borders count="5">
     <border>
       <left style="none"/>
       <right style="none"/>
@@ -663,36 +656,19 @@
       <diagonal style="none"/>
     </border>
     <border>
-      <left style="thin">
-        <color auto="1"/>
-      </left>
-      <right style="thin">
-        <color auto="1"/>
-      </right>
+      <left/>
+      <right/>
       <top style="thin">
         <color auto="1"/>
       </top>
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin">
-        <color auto="1"/>
-      </left>
-      <right style="thin">
-        <color auto="1"/>
-      </right>
-      <top/>
-      <bottom style="thin">
-        <color auto="1"/>
-      </bottom>
-      <diagonal/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf fontId="0" fillId="0" borderId="0" numFmtId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
   </cellStyleXfs>
-  <cellXfs count="47">
+  <cellXfs count="49">
     <xf fontId="0" fillId="0" borderId="0" numFmtId="0" xfId="0"/>
     <xf fontId="0" fillId="0" borderId="0" numFmtId="0" xfId="0" applyAlignment="1">
       <alignment vertical="center"/>
@@ -755,6 +731,21 @@
     <xf fontId="1" fillId="0" borderId="0" numFmtId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
+    <xf fontId="0" fillId="0" borderId="4" numFmtId="0" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf fontId="0" fillId="0" borderId="0" numFmtId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf fontId="0" fillId="0" borderId="1" numFmtId="0" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf fontId="0" fillId="3" borderId="2" numFmtId="0" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf fontId="0" fillId="3" borderId="2" numFmtId="0" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
     <xf fontId="0" fillId="0" borderId="1" numFmtId="0" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -782,7 +773,7 @@
     <xf fontId="2" fillId="0" borderId="2" numFmtId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
     </xf>
-    <xf fontId="0" fillId="0" borderId="4" numFmtId="0" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf fontId="0" fillId="0" borderId="2" numFmtId="0" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
     <xf fontId="0" fillId="0" borderId="1" numFmtId="0" xfId="0" applyBorder="1" applyAlignment="1">
@@ -800,35 +791,26 @@
     <xf fontId="2" fillId="0" borderId="3" numFmtId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
     </xf>
-    <xf fontId="0" fillId="0" borderId="5" numFmtId="0" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf fontId="0" fillId="0" borderId="3" numFmtId="0" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
     <xf fontId="3" fillId="0" borderId="1" numFmtId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf fontId="3" fillId="0" borderId="4" numFmtId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf fontId="3" fillId="0" borderId="2" numFmtId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf fontId="3" fillId="0" borderId="5" numFmtId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf fontId="3" fillId="0" borderId="3" numFmtId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
     <xf fontId="2" fillId="0" borderId="0" numFmtId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf fontId="0" fillId="0" borderId="0" numFmtId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf fontId="0" fillId="0" borderId="1" numFmtId="0" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
     <xf fontId="4" fillId="0" borderId="0" numFmtId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
     <xf fontId="3" fillId="0" borderId="0" numFmtId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf fontId="5" fillId="0" borderId="0" numFmtId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1670,7 +1652,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac">
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultRowHeight="14.25"/>
   <cols>
     <col customWidth="1" min="1" max="1" style="2" width="12"/>
     <col bestFit="1" customWidth="1" min="2" max="2" style="2" width="11.85546875"/>
@@ -1680,7 +1662,7 @@
     <col customWidth="1" min="6" max="6" style="4" width="30.85546875"/>
     <col bestFit="1" customWidth="1" min="7" max="7" style="1" width="17.5703125"/>
     <col customWidth="1" min="8" max="8" style="4" width="46.42578125"/>
-    <col bestFit="1" customWidth="1" min="9" max="9" style="1" width="4.42578125"/>
+    <col customWidth="1" min="9" max="9" style="1" width="9.00390625"/>
     <col min="10" max="16384" style="1" width="9.140625"/>
   </cols>
   <sheetData>
@@ -1714,7 +1696,7 @@
       <c r="A2" s="8" t="s">
         <v>8</v>
       </c>
-      <c r="B2" s="8" t="s">
+      <c r="B2" s="22" t="s">
         <v>44</v>
       </c>
       <c r="C2" s="9">
@@ -1744,7 +1726,7 @@
       <c r="A3" s="8" t="s">
         <v>8</v>
       </c>
-      <c r="B3" s="8"/>
+      <c r="B3" s="23"/>
       <c r="C3" s="9"/>
       <c r="D3" s="11"/>
       <c r="E3" s="11" t="s">
@@ -1766,7 +1748,7 @@
       <c r="A4" s="8" t="s">
         <v>18</v>
       </c>
-      <c r="B4" s="8"/>
+      <c r="B4" s="23"/>
       <c r="C4" s="9">
         <v>36558</v>
       </c>
@@ -1790,11 +1772,11 @@
       </c>
       <c r="J4" s="1"/>
     </row>
-    <row r="5" ht="29.25">
+    <row r="5" ht="28.5">
       <c r="A5" s="8" t="s">
         <v>18</v>
       </c>
-      <c r="B5" s="8"/>
+      <c r="B5" s="23"/>
       <c r="C5" s="9"/>
       <c r="D5" s="11"/>
       <c r="E5" s="11" t="s">
@@ -1816,7 +1798,7 @@
       <c r="A6" s="8" t="s">
         <v>25</v>
       </c>
-      <c r="B6" s="8"/>
+      <c r="B6" s="23"/>
       <c r="C6" s="8">
         <v>50360</v>
       </c>
@@ -1840,11 +1822,11 @@
       </c>
       <c r="J6" s="1"/>
     </row>
-    <row r="7" ht="29.25">
+    <row r="7" ht="28.5">
       <c r="A7" s="8" t="s">
         <v>25</v>
       </c>
-      <c r="B7" s="8"/>
+      <c r="B7" s="23"/>
       <c r="C7" s="8"/>
       <c r="D7" s="17"/>
       <c r="E7" s="17" t="s">
@@ -1866,7 +1848,7 @@
       <c r="A8" s="8" t="s">
         <v>32</v>
       </c>
-      <c r="B8" s="8"/>
+      <c r="B8" s="23"/>
       <c r="C8" s="8">
         <v>50394</v>
       </c>
@@ -1894,7 +1876,7 @@
       <c r="A9" s="8" t="s">
         <v>32</v>
       </c>
-      <c r="B9" s="8"/>
+      <c r="B9" s="23"/>
       <c r="C9" s="8"/>
       <c r="D9" s="17"/>
       <c r="E9" s="17" t="s">
@@ -1916,7 +1898,7 @@
       <c r="A10" s="8" t="s">
         <v>38</v>
       </c>
-      <c r="B10" s="8"/>
+      <c r="B10" s="23"/>
       <c r="C10" s="8">
         <v>77012</v>
       </c>
@@ -1940,11 +1922,11 @@
       </c>
       <c r="J10" s="1"/>
     </row>
-    <row r="11" ht="43.5">
+    <row r="11" ht="42.75">
       <c r="A11" s="8" t="s">
         <v>38</v>
       </c>
-      <c r="B11" s="8"/>
+      <c r="B11" s="23"/>
       <c r="C11" s="8"/>
       <c r="D11" s="17"/>
       <c r="E11" s="17" t="s">
@@ -1962,12 +1944,57 @@
       </c>
       <c r="J11" s="1"/>
     </row>
-    <row r="13">
-      <c r="A13" s="21"/>
+    <row r="12" ht="14.25">
+      <c r="A12" s="24" t="s">
+        <v>71</v>
+      </c>
+      <c r="B12" s="23"/>
+      <c r="C12" s="25">
+        <v>36558</v>
+      </c>
+      <c r="D12" s="26" t="s">
+        <v>51</v>
+      </c>
+      <c r="E12" s="11" t="s">
+        <v>46</v>
+      </c>
+      <c r="F12" s="12" t="s">
+        <v>52</v>
+      </c>
+      <c r="G12" s="13" t="s">
+        <v>13</v>
+      </c>
+      <c r="H12" s="26" t="s">
+        <v>53</v>
+      </c>
+      <c r="I12" s="1">
+        <v>2221</v>
+      </c>
+    </row>
+    <row r="13" ht="28.5">
+      <c r="A13" s="24" t="s">
+        <v>71</v>
+      </c>
+      <c r="B13" s="23"/>
+      <c r="C13" s="9"/>
+      <c r="D13" s="11"/>
+      <c r="E13" s="11" t="s">
+        <v>54</v>
+      </c>
+      <c r="F13" s="12" t="s">
+        <v>55</v>
+      </c>
+      <c r="G13" s="13" t="s">
+        <v>17</v>
+      </c>
+      <c r="H13" s="11"/>
+      <c r="I13" s="1">
+        <v>2231</v>
+      </c>
     </row>
   </sheetData>
-  <mergeCells count="16">
-    <mergeCell ref="B2:B11"/>
+  <mergeCells count="19">
+    <mergeCell ref="B2:B13"/>
     <mergeCell ref="C2:C3"/>
     <mergeCell ref="D2:D3"/>
     <mergeCell ref="H2:H3"/>
@@ -1983,6 +2010,9 @@
     <mergeCell ref="C10:C11"/>
     <mergeCell ref="D10:D11"/>
     <mergeCell ref="H10:H11"/>
+    <mergeCell ref="C12:C13"/>
+    <mergeCell ref="D12:D13"/>
+    <mergeCell ref="H12:H13"/>
   </mergeCells>
   <printOptions headings="0" gridLines="0"/>
   <pageMargins left="0.69999999999999996" right="0.69999999999999996" top="0.75" bottom="0.75" header="0.29999999999999999" footer="0.29999999999999999"/>
@@ -2036,26 +2066,26 @@
       <c r="A2" s="8" t="s">
         <v>8</v>
       </c>
-      <c r="B2" s="22" t="s">
-        <v>71</v>
+      <c r="B2" s="27" t="s">
+        <v>72</v>
       </c>
       <c r="C2" s="8">
         <v>21141</v>
       </c>
       <c r="D2" s="17" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="E2" s="17" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="F2" s="20" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="G2" s="19" t="s">
         <v>13</v>
       </c>
       <c r="H2" s="17" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="I2" s="1">
         <v>230</v>
@@ -2066,17 +2096,17 @@
       <c r="A3" s="8" t="s">
         <v>8</v>
       </c>
-      <c r="B3" s="22"/>
+      <c r="B3" s="27"/>
       <c r="C3" s="8"/>
       <c r="D3" s="17"/>
       <c r="E3" s="17" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="F3" s="20" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="G3" s="19" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="H3" s="17"/>
       <c r="I3" s="1">
@@ -2088,24 +2118,24 @@
       <c r="A4" s="8" t="s">
         <v>18</v>
       </c>
-      <c r="B4" s="22"/>
+      <c r="B4" s="27"/>
       <c r="C4" s="8">
         <v>21196</v>
       </c>
       <c r="D4" s="17" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="E4" s="17" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="F4" s="20" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="G4" s="19" t="s">
         <v>13</v>
       </c>
       <c r="H4" s="17" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="I4" s="1">
         <v>232</v>
@@ -2116,14 +2146,14 @@
       <c r="A5" s="8" t="s">
         <v>18</v>
       </c>
-      <c r="B5" s="22"/>
+      <c r="B5" s="27"/>
       <c r="C5" s="8"/>
       <c r="D5" s="17"/>
       <c r="E5" s="17" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="F5" s="20" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="G5" s="19" t="s">
         <v>17</v>
@@ -2138,24 +2168,24 @@
       <c r="A6" s="8" t="s">
         <v>25</v>
       </c>
-      <c r="B6" s="22"/>
+      <c r="B6" s="27"/>
       <c r="C6" s="8">
         <v>21210</v>
       </c>
       <c r="D6" s="17" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="E6" s="17" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="F6" s="18" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="G6" s="19" t="s">
         <v>21</v>
       </c>
       <c r="H6" s="17" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="I6" s="1">
         <v>234</v>
@@ -2166,14 +2196,14 @@
       <c r="A7" s="8" t="s">
         <v>25</v>
       </c>
-      <c r="B7" s="22"/>
+      <c r="B7" s="27"/>
       <c r="C7" s="8"/>
       <c r="D7" s="17"/>
       <c r="E7" s="17" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="F7" s="18" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="G7" s="19" t="s">
         <v>17</v>
@@ -2188,24 +2218,24 @@
       <c r="A8" s="8" t="s">
         <v>32</v>
       </c>
-      <c r="B8" s="22"/>
+      <c r="B8" s="27"/>
       <c r="C8" s="8">
         <v>21085</v>
       </c>
       <c r="D8" s="17" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="E8" s="17" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="F8" s="20" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="G8" s="19" t="s">
         <v>13</v>
       </c>
       <c r="H8" s="17" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="I8" s="1">
         <v>236</v>
@@ -2216,14 +2246,14 @@
       <c r="A9" s="8" t="s">
         <v>32</v>
       </c>
-      <c r="B9" s="22"/>
+      <c r="B9" s="27"/>
       <c r="C9" s="8"/>
       <c r="D9" s="17"/>
       <c r="E9" s="17" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="F9" s="20" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="G9" s="19" t="s">
         <v>21</v>
@@ -2238,24 +2268,24 @@
       <c r="A10" s="8" t="s">
         <v>38</v>
       </c>
-      <c r="B10" s="22"/>
+      <c r="B10" s="27"/>
       <c r="C10" s="8">
         <v>21235</v>
       </c>
       <c r="D10" s="17" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="E10" s="17" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="F10" s="20" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="G10" s="19" t="s">
         <v>13</v>
       </c>
       <c r="H10" s="17" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="I10" s="1">
         <v>238</v>
@@ -2266,14 +2296,14 @@
       <c r="A11" s="8" t="s">
         <v>38</v>
       </c>
-      <c r="B11" s="22"/>
+      <c r="B11" s="27"/>
       <c r="C11" s="8"/>
       <c r="D11" s="17"/>
       <c r="E11" s="17" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="F11" s="20" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="G11" s="19" t="s">
         <v>17</v>
@@ -2317,704 +2347,704 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac">
   <sheetFormatPr defaultRowHeight="14.25"/>
   <cols>
-    <col customWidth="1" min="1" max="1" style="23" width="12"/>
-    <col bestFit="1" customWidth="1" min="2" max="2" style="23" width="11.85546875"/>
-    <col min="3" max="3" style="23" width="9.140625"/>
-    <col customWidth="1" min="4" max="5" style="24" width="42.85546875"/>
-    <col customWidth="1" min="6" max="6" style="24" width="30.85546875"/>
-    <col bestFit="1" customWidth="1" min="7" max="7" style="23" width="17.5703125"/>
-    <col customWidth="1" min="8" max="8" style="24" width="46.42578125"/>
-    <col min="9" max="16384" style="23" width="9.140625"/>
+    <col customWidth="1" min="1" max="1" style="28" width="12"/>
+    <col bestFit="1" customWidth="1" min="2" max="2" style="28" width="11.85546875"/>
+    <col min="3" max="3" style="28" width="9.140625"/>
+    <col customWidth="1" min="4" max="5" style="29" width="42.85546875"/>
+    <col customWidth="1" min="6" max="6" style="29" width="30.85546875"/>
+    <col bestFit="1" customWidth="1" min="7" max="7" style="28" width="17.5703125"/>
+    <col customWidth="1" min="8" max="8" style="29" width="46.42578125"/>
+    <col min="9" max="16384" style="28" width="9.140625"/>
   </cols>
   <sheetData>
-    <row r="1" s="25" customFormat="1">
-      <c r="A1" s="26" t="s">
+    <row r="1" s="30" customFormat="1">
+      <c r="A1" s="31" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="26" t="s">
+      <c r="B1" s="31" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="26" t="s">
-        <v>102</v>
-      </c>
-      <c r="D1" s="27" t="s">
+      <c r="C1" s="31" t="s">
+        <v>103</v>
+      </c>
+      <c r="D1" s="32" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="27" t="s">
+      <c r="E1" s="32" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="27" t="s">
+      <c r="F1" s="32" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="26" t="s">
+      <c r="G1" s="31" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="26" t="s">
+      <c r="H1" s="31" t="s">
         <v>7</v>
       </c>
     </row>
     <row r="2" ht="57">
-      <c r="A2" s="28" t="s">
-        <v>103</v>
-      </c>
-      <c r="B2" s="29" t="s">
+      <c r="A2" s="33" t="s">
+        <v>71</v>
+      </c>
+      <c r="B2" s="34" t="s">
         <v>104</v>
       </c>
-      <c r="C2" s="30" t="s">
+      <c r="C2" s="35" t="s">
         <v>105</v>
       </c>
-      <c r="D2" s="31" t="s">
+      <c r="D2" s="36" t="s">
         <v>106</v>
       </c>
-      <c r="E2" s="32" t="s">
+      <c r="E2" s="37" t="s">
         <v>107</v>
       </c>
-      <c r="F2" s="32" t="s">
+      <c r="F2" s="37" t="s">
         <v>108</v>
       </c>
-      <c r="G2" s="33" t="s">
+      <c r="G2" s="38" t="s">
         <v>13</v>
       </c>
-      <c r="H2" s="32" t="s">
+      <c r="H2" s="37" t="s">
         <v>109</v>
       </c>
-      <c r="I2" s="34">
+      <c r="I2" s="39">
         <v>260</v>
       </c>
-      <c r="J2" s="23"/>
+      <c r="J2" s="28"/>
     </row>
     <row r="3" ht="50.25" customHeight="1">
-      <c r="A3" s="28" t="s">
-        <v>103</v>
-      </c>
-      <c r="B3" s="35"/>
-      <c r="C3" s="36"/>
-      <c r="D3" s="37"/>
-      <c r="E3" s="32" t="s">
+      <c r="A3" s="33" t="s">
+        <v>71</v>
+      </c>
+      <c r="B3" s="40"/>
+      <c r="C3" s="41"/>
+      <c r="D3" s="42"/>
+      <c r="E3" s="37" t="s">
         <v>110</v>
       </c>
-      <c r="F3" s="32" t="s">
+      <c r="F3" s="37" t="s">
         <v>111</v>
       </c>
-      <c r="G3" s="33" t="s">
+      <c r="G3" s="38" t="s">
         <v>17</v>
       </c>
-      <c r="H3" s="32" t="s">
+      <c r="H3" s="37" t="s">
         <v>112</v>
       </c>
-      <c r="I3" s="34">
+      <c r="I3" s="39">
         <v>261</v>
       </c>
-      <c r="J3" s="23"/>
+      <c r="J3" s="28"/>
     </row>
     <row r="4" ht="71.25">
-      <c r="A4" s="28" t="s">
+      <c r="A4" s="33" t="s">
         <v>113</v>
       </c>
-      <c r="B4" s="29" t="s">
+      <c r="B4" s="34" t="s">
         <v>104</v>
       </c>
-      <c r="C4" s="30" t="s">
+      <c r="C4" s="35" t="s">
         <v>114</v>
       </c>
-      <c r="D4" s="31" t="s">
+      <c r="D4" s="36" t="s">
         <v>115</v>
       </c>
-      <c r="E4" s="32" t="s">
+      <c r="E4" s="37" t="s">
         <v>116</v>
       </c>
-      <c r="F4" s="32" t="s">
+      <c r="F4" s="37" t="s">
         <v>117</v>
       </c>
-      <c r="G4" s="33" t="s">
+      <c r="G4" s="38" t="s">
         <v>13</v>
       </c>
-      <c r="H4" s="32" t="s">
+      <c r="H4" s="37" t="s">
         <v>118</v>
       </c>
-      <c r="I4" s="34">
+      <c r="I4" s="39">
         <v>262</v>
       </c>
-      <c r="J4" s="23"/>
+      <c r="J4" s="28"/>
     </row>
     <row r="5" ht="57">
-      <c r="A5" s="28" t="s">
+      <c r="A5" s="33" t="s">
         <v>113</v>
       </c>
-      <c r="B5" s="35"/>
-      <c r="C5" s="36"/>
-      <c r="D5" s="37"/>
-      <c r="E5" s="32" t="s">
+      <c r="B5" s="40"/>
+      <c r="C5" s="41"/>
+      <c r="D5" s="42"/>
+      <c r="E5" s="37" t="s">
         <v>119</v>
       </c>
-      <c r="F5" s="32" t="s">
+      <c r="F5" s="37" t="s">
         <v>120</v>
       </c>
-      <c r="G5" s="33" t="s">
+      <c r="G5" s="38" t="s">
         <v>17</v>
       </c>
-      <c r="H5" s="32" t="s">
+      <c r="H5" s="37" t="s">
         <v>121</v>
       </c>
-      <c r="I5" s="34">
+      <c r="I5" s="39">
         <v>263</v>
       </c>
-      <c r="J5" s="23"/>
+      <c r="J5" s="28"/>
     </row>
     <row r="6" ht="57">
-      <c r="A6" s="28" t="s">
+      <c r="A6" s="33" t="s">
         <v>122</v>
       </c>
-      <c r="B6" s="29" t="s">
+      <c r="B6" s="34" t="s">
         <v>104</v>
       </c>
-      <c r="C6" s="30" t="s">
+      <c r="C6" s="35" t="s">
         <v>105</v>
       </c>
-      <c r="D6" s="31" t="s">
+      <c r="D6" s="36" t="s">
         <v>106</v>
       </c>
-      <c r="E6" s="32" t="s">
+      <c r="E6" s="37" t="s">
         <v>123</v>
       </c>
-      <c r="F6" s="32" t="s">
+      <c r="F6" s="37" t="s">
         <v>124</v>
       </c>
-      <c r="G6" s="33" t="s">
+      <c r="G6" s="38" t="s">
         <v>13</v>
       </c>
-      <c r="H6" s="32" t="s">
+      <c r="H6" s="37" t="s">
         <v>109</v>
       </c>
-      <c r="I6" s="34">
+      <c r="I6" s="39">
         <v>264</v>
       </c>
-      <c r="J6" s="23"/>
+      <c r="J6" s="28"/>
     </row>
     <row r="7" ht="108.75">
-      <c r="A7" s="28" t="s">
+      <c r="A7" s="33" t="s">
         <v>122</v>
       </c>
-      <c r="B7" s="35"/>
-      <c r="C7" s="36"/>
-      <c r="D7" s="37"/>
-      <c r="E7" s="38" t="s">
+      <c r="B7" s="40"/>
+      <c r="C7" s="41"/>
+      <c r="D7" s="42"/>
+      <c r="E7" s="43" t="s">
         <v>125</v>
       </c>
-      <c r="F7" s="38" t="s">
+      <c r="F7" s="43" t="s">
         <v>126</v>
       </c>
-      <c r="G7" s="38" t="s">
+      <c r="G7" s="43" t="s">
         <v>17</v>
       </c>
-      <c r="H7" s="38" t="s">
+      <c r="H7" s="43" t="s">
         <v>112</v>
       </c>
-      <c r="I7" s="34">
+      <c r="I7" s="39">
         <v>265</v>
       </c>
-      <c r="J7" s="23"/>
+      <c r="J7" s="28"/>
     </row>
     <row r="8" ht="108.75">
-      <c r="A8" s="28" t="s">
+      <c r="A8" s="33" t="s">
         <v>127</v>
       </c>
-      <c r="B8" s="29" t="s">
+      <c r="B8" s="34" t="s">
         <v>104</v>
       </c>
-      <c r="C8" s="30" t="s">
+      <c r="C8" s="35" t="s">
         <v>114</v>
       </c>
-      <c r="D8" s="39" t="s">
+      <c r="D8" s="44" t="s">
         <v>115</v>
       </c>
-      <c r="E8" s="38" t="s">
+      <c r="E8" s="43" t="s">
         <v>128</v>
       </c>
-      <c r="F8" s="38" t="s">
+      <c r="F8" s="43" t="s">
         <v>129</v>
       </c>
-      <c r="G8" s="38" t="s">
+      <c r="G8" s="43" t="s">
         <v>13</v>
       </c>
-      <c r="H8" s="38" t="s">
+      <c r="H8" s="43" t="s">
         <v>118</v>
       </c>
-      <c r="I8" s="34">
+      <c r="I8" s="39">
         <v>266</v>
       </c>
-      <c r="J8" s="23"/>
+      <c r="J8" s="28"/>
     </row>
     <row r="9" ht="108.75">
-      <c r="A9" s="28" t="s">
+      <c r="A9" s="33" t="s">
         <v>127</v>
       </c>
-      <c r="B9" s="35"/>
-      <c r="C9" s="36"/>
-      <c r="D9" s="40"/>
-      <c r="E9" s="38" t="s">
+      <c r="B9" s="40"/>
+      <c r="C9" s="41"/>
+      <c r="D9" s="45"/>
+      <c r="E9" s="43" t="s">
         <v>130</v>
       </c>
-      <c r="F9" s="38" t="s">
+      <c r="F9" s="43" t="s">
         <v>131</v>
       </c>
-      <c r="G9" s="38" t="s">
+      <c r="G9" s="43" t="s">
         <v>17</v>
       </c>
-      <c r="H9" s="38" t="s">
+      <c r="H9" s="43" t="s">
         <v>121</v>
       </c>
-      <c r="I9" s="34">
+      <c r="I9" s="39">
         <v>267</v>
       </c>
-      <c r="J9" s="23"/>
+      <c r="J9" s="28"/>
     </row>
     <row r="10" ht="108.75">
-      <c r="A10" s="28" t="s">
+      <c r="A10" s="33" t="s">
         <v>132</v>
       </c>
-      <c r="B10" s="29" t="s">
+      <c r="B10" s="34" t="s">
         <v>133</v>
       </c>
-      <c r="C10" s="30" t="s">
+      <c r="C10" s="35" t="s">
         <v>134</v>
       </c>
-      <c r="D10" s="39" t="s">
+      <c r="D10" s="44" t="s">
         <v>135</v>
       </c>
-      <c r="E10" s="38" t="s">
+      <c r="E10" s="43" t="s">
         <v>136</v>
       </c>
-      <c r="F10" s="38" t="s">
+      <c r="F10" s="43" t="s">
         <v>137</v>
       </c>
-      <c r="G10" s="38" t="s">
+      <c r="G10" s="43" t="s">
         <v>13</v>
       </c>
-      <c r="H10" s="38" t="s">
+      <c r="H10" s="43" t="s">
         <v>138</v>
       </c>
-      <c r="I10" s="34">
+      <c r="I10" s="39">
         <v>268</v>
       </c>
-      <c r="J10" s="23"/>
+      <c r="J10" s="28"/>
     </row>
     <row r="11" ht="87">
-      <c r="A11" s="28" t="s">
+      <c r="A11" s="33" t="s">
         <v>132</v>
       </c>
-      <c r="B11" s="35"/>
-      <c r="C11" s="36"/>
-      <c r="D11" s="40"/>
-      <c r="E11" s="38" t="s">
+      <c r="B11" s="40"/>
+      <c r="C11" s="41"/>
+      <c r="D11" s="45"/>
+      <c r="E11" s="43" t="s">
         <v>139</v>
       </c>
-      <c r="F11" s="38" t="s">
+      <c r="F11" s="43" t="s">
         <v>140</v>
       </c>
-      <c r="G11" s="38" t="s">
+      <c r="G11" s="43" t="s">
         <v>21</v>
       </c>
-      <c r="H11" s="38" t="s">
+      <c r="H11" s="43" t="s">
         <v>141</v>
       </c>
-      <c r="I11" s="34">
+      <c r="I11" s="39">
         <v>269</v>
       </c>
-      <c r="J11" s="23"/>
+      <c r="J11" s="28"/>
     </row>
     <row r="12" ht="71.25">
-      <c r="A12" s="34" t="s">
+      <c r="A12" s="39" t="s">
         <v>142</v>
       </c>
-      <c r="B12" s="41" t="s">
+      <c r="B12" s="46" t="s">
         <v>143</v>
       </c>
-      <c r="C12" s="34" t="s">
+      <c r="C12" s="39" t="s">
         <v>144</v>
       </c>
-      <c r="D12" s="42" t="s">
+      <c r="D12" s="29" t="s">
         <v>145</v>
       </c>
-      <c r="E12" s="24" t="s">
+      <c r="E12" s="29" t="s">
         <v>146</v>
       </c>
-      <c r="F12" s="24" t="s">
+      <c r="F12" s="29" t="s">
         <v>147</v>
       </c>
-      <c r="G12" s="33" t="s">
+      <c r="G12" s="38" t="s">
         <v>17</v>
       </c>
-      <c r="H12" s="24" t="s">
+      <c r="H12" s="29" t="s">
         <v>141</v>
       </c>
-      <c r="I12" s="34">
+      <c r="I12" s="39">
         <v>270</v>
       </c>
     </row>
     <row r="13" ht="71.25">
-      <c r="A13" s="34" t="s">
+      <c r="A13" s="39" t="s">
         <v>142</v>
       </c>
-      <c r="B13" s="41"/>
-      <c r="C13" s="34"/>
-      <c r="D13" s="42"/>
-      <c r="E13" s="24" t="s">
+      <c r="B13" s="46"/>
+      <c r="C13" s="39"/>
+      <c r="D13" s="29"/>
+      <c r="E13" s="29" t="s">
         <v>148</v>
       </c>
-      <c r="F13" s="24" t="s">
+      <c r="F13" s="29" t="s">
         <v>149</v>
       </c>
-      <c r="G13" s="33" t="s">
+      <c r="G13" s="38" t="s">
         <v>13</v>
       </c>
-      <c r="H13" s="24" t="s">
+      <c r="H13" s="29" t="s">
         <v>150</v>
       </c>
-      <c r="I13" s="34">
+      <c r="I13" s="39">
         <v>271</v>
       </c>
     </row>
-    <row r="14" ht="71.25">
-      <c r="A14" s="28" t="s">
+    <row r="14" ht="57">
+      <c r="A14" s="33" t="s">
         <v>151</v>
       </c>
-      <c r="B14" s="29" t="s">
+      <c r="B14" s="34" t="s">
         <v>104</v>
       </c>
-      <c r="C14" s="30">
+      <c r="C14" s="35">
         <v>45380</v>
       </c>
-      <c r="D14" s="31" t="s">
+      <c r="D14" s="36" t="s">
         <v>152</v>
       </c>
-      <c r="E14" s="32" t="s">
+      <c r="E14" s="37" t="s">
         <v>153</v>
       </c>
-      <c r="F14" s="32" t="s">
+      <c r="F14" s="37" t="s">
         <v>154</v>
       </c>
-      <c r="G14" s="33" t="s">
+      <c r="G14" s="38" t="s">
         <v>17</v>
       </c>
-      <c r="H14" s="32" t="s">
+      <c r="H14" s="37" t="s">
         <v>155</v>
       </c>
-      <c r="I14" s="34">
+      <c r="I14" s="39">
         <v>272</v>
       </c>
     </row>
     <row r="15" ht="99.75">
-      <c r="A15" s="28" t="s">
+      <c r="A15" s="33" t="s">
         <v>156</v>
       </c>
-      <c r="B15" s="35"/>
-      <c r="C15" s="36"/>
-      <c r="D15" s="37"/>
-      <c r="E15" s="32" t="s">
+      <c r="B15" s="40"/>
+      <c r="C15" s="41"/>
+      <c r="D15" s="42"/>
+      <c r="E15" s="37" t="s">
         <v>157</v>
       </c>
-      <c r="F15" s="32" t="s">
+      <c r="F15" s="37" t="s">
         <v>158</v>
       </c>
-      <c r="G15" s="33" t="s">
+      <c r="G15" s="38" t="s">
         <v>13</v>
       </c>
-      <c r="H15" s="43" t="s">
+      <c r="H15" s="37" t="s">
         <v>159</v>
       </c>
-      <c r="I15" s="34">
+      <c r="I15" s="39">
         <v>273</v>
       </c>
     </row>
     <row r="16" ht="85.5">
-      <c r="A16" s="28" t="s">
+      <c r="A16" s="33" t="s">
         <v>151</v>
       </c>
-      <c r="B16" s="29" t="s">
+      <c r="B16" s="34" t="s">
         <v>104</v>
       </c>
-      <c r="C16" s="30">
+      <c r="C16" s="35">
         <v>43235</v>
       </c>
-      <c r="D16" s="31" t="s">
+      <c r="D16" s="36" t="s">
         <v>160</v>
       </c>
-      <c r="E16" s="32" t="s">
+      <c r="E16" s="37" t="s">
         <v>161</v>
       </c>
-      <c r="F16" s="32" t="s">
+      <c r="F16" s="37" t="s">
         <v>162</v>
       </c>
-      <c r="G16" s="33" t="s">
+      <c r="G16" s="38" t="s">
         <v>17</v>
       </c>
-      <c r="H16" s="32" t="s">
+      <c r="H16" s="37" t="s">
         <v>163</v>
       </c>
-      <c r="I16" s="34">
+      <c r="I16" s="39">
         <v>274</v>
       </c>
     </row>
     <row r="17" ht="71.25">
-      <c r="A17" s="28" t="s">
+      <c r="A17" s="33" t="s">
         <v>156</v>
       </c>
-      <c r="B17" s="35"/>
-      <c r="C17" s="36"/>
-      <c r="D17" s="37"/>
-      <c r="E17" s="32" t="s">
+      <c r="B17" s="40"/>
+      <c r="C17" s="41"/>
+      <c r="D17" s="42"/>
+      <c r="E17" s="37" t="s">
         <v>164</v>
       </c>
-      <c r="F17" s="32" t="s">
+      <c r="F17" s="37" t="s">
         <v>165</v>
       </c>
-      <c r="G17" s="33" t="s">
+      <c r="G17" s="38" t="s">
         <v>13</v>
       </c>
-      <c r="H17" s="32" t="s">
+      <c r="H17" s="37" t="s">
         <v>166</v>
       </c>
-      <c r="I17" s="34">
+      <c r="I17" s="39">
         <v>275</v>
       </c>
     </row>
     <row r="18" ht="14.25">
-      <c r="A18" s="23"/>
-      <c r="B18" s="23"/>
-      <c r="C18" s="23"/>
-      <c r="D18" s="24"/>
-      <c r="E18" s="24"/>
-      <c r="F18" s="24"/>
-      <c r="G18" s="23"/>
-      <c r="H18" s="24"/>
-      <c r="I18" s="23"/>
+      <c r="A18" s="28"/>
+      <c r="B18" s="28"/>
+      <c r="C18" s="28"/>
+      <c r="D18" s="29"/>
+      <c r="E18" s="29"/>
+      <c r="F18" s="29"/>
+      <c r="G18" s="28"/>
+      <c r="H18" s="29"/>
+      <c r="I18" s="28"/>
     </row>
     <row r="19" ht="14.25">
-      <c r="A19" s="23"/>
-      <c r="B19" s="23"/>
-      <c r="C19" s="23"/>
-      <c r="D19" s="24"/>
-      <c r="E19" s="24"/>
-      <c r="F19" s="24"/>
-      <c r="G19" s="23"/>
-      <c r="H19" s="24"/>
-      <c r="I19" s="23"/>
+      <c r="A19" s="28"/>
+      <c r="B19" s="28"/>
+      <c r="C19" s="28"/>
+      <c r="D19" s="29"/>
+      <c r="E19" s="29"/>
+      <c r="F19" s="29"/>
+      <c r="G19" s="28"/>
+      <c r="H19" s="29"/>
+      <c r="I19" s="28"/>
     </row>
     <row r="20" ht="14.25">
-      <c r="A20" s="23"/>
-      <c r="B20" s="23"/>
-      <c r="C20" s="23"/>
-      <c r="D20" s="24"/>
-      <c r="E20" s="24"/>
-      <c r="F20" s="24"/>
-      <c r="G20" s="23"/>
-      <c r="H20" s="24"/>
+      <c r="A20" s="28"/>
+      <c r="B20" s="28"/>
+      <c r="C20" s="28"/>
+      <c r="D20" s="29"/>
+      <c r="E20" s="29"/>
+      <c r="F20" s="29"/>
+      <c r="G20" s="28"/>
+      <c r="H20" s="29"/>
     </row>
     <row r="21" ht="14.25">
-      <c r="A21" s="23"/>
-      <c r="B21" s="23"/>
-      <c r="C21" s="23"/>
-      <c r="D21" s="24"/>
-      <c r="E21" s="24"/>
-      <c r="F21" s="24"/>
-      <c r="G21" s="23"/>
-      <c r="H21" s="24"/>
+      <c r="A21" s="28"/>
+      <c r="B21" s="28"/>
+      <c r="C21" s="28"/>
+      <c r="D21" s="29"/>
+      <c r="E21" s="29"/>
+      <c r="F21" s="29"/>
+      <c r="G21" s="28"/>
+      <c r="H21" s="29"/>
     </row>
     <row r="22" ht="14.25">
-      <c r="A22" s="23"/>
-      <c r="B22" s="23"/>
-      <c r="C22" s="23"/>
-      <c r="D22" s="24"/>
-      <c r="E22" s="24"/>
-      <c r="F22" s="24"/>
-      <c r="G22" s="23"/>
-      <c r="H22" s="24"/>
+      <c r="A22" s="28"/>
+      <c r="B22" s="28"/>
+      <c r="C22" s="28"/>
+      <c r="D22" s="29"/>
+      <c r="E22" s="29"/>
+      <c r="F22" s="29"/>
+      <c r="G22" s="28"/>
+      <c r="H22" s="29"/>
     </row>
     <row r="23" ht="21.75">
-      <c r="A23" s="44"/>
-      <c r="B23" s="44"/>
-      <c r="C23" s="44"/>
-      <c r="D23" s="44"/>
-      <c r="E23" s="44"/>
-      <c r="F23" s="44"/>
-      <c r="G23" s="44"/>
-      <c r="H23" s="44"/>
+      <c r="A23" s="47"/>
+      <c r="B23" s="47"/>
+      <c r="C23" s="47"/>
+      <c r="D23" s="47"/>
+      <c r="E23" s="47"/>
+      <c r="F23" s="47"/>
+      <c r="G23" s="47"/>
+      <c r="H23" s="47"/>
     </row>
     <row r="24" ht="21.75">
-      <c r="A24" s="45"/>
-      <c r="B24" s="45"/>
-      <c r="C24" s="45"/>
-      <c r="D24" s="45"/>
-      <c r="E24" s="45"/>
-      <c r="F24" s="45"/>
-      <c r="G24" s="45"/>
-      <c r="H24" s="45"/>
+      <c r="A24" s="48"/>
+      <c r="B24" s="48"/>
+      <c r="C24" s="48"/>
+      <c r="D24" s="48"/>
+      <c r="E24" s="48"/>
+      <c r="F24" s="48"/>
+      <c r="G24" s="48"/>
+      <c r="H24" s="48"/>
     </row>
     <row r="25" ht="21.75">
-      <c r="A25" s="45"/>
-      <c r="B25" s="24"/>
-      <c r="C25" s="24"/>
-      <c r="D25" s="24"/>
-      <c r="E25" s="45"/>
-      <c r="F25" s="45"/>
-      <c r="G25" s="45"/>
-      <c r="H25" s="45"/>
+      <c r="A25" s="48"/>
+      <c r="B25" s="29"/>
+      <c r="C25" s="29"/>
+      <c r="D25" s="29"/>
+      <c r="E25" s="48"/>
+      <c r="F25" s="48"/>
+      <c r="G25" s="48"/>
+      <c r="H25" s="48"/>
     </row>
     <row r="26" ht="21.75">
-      <c r="A26" s="45"/>
-      <c r="B26" s="45"/>
-      <c r="C26" s="45"/>
-      <c r="D26" s="45"/>
-      <c r="E26" s="45"/>
-      <c r="F26" s="45"/>
-      <c r="G26" s="45"/>
-      <c r="H26" s="45"/>
+      <c r="A26" s="48"/>
+      <c r="B26" s="48"/>
+      <c r="C26" s="48"/>
+      <c r="D26" s="48"/>
+      <c r="E26" s="48"/>
+      <c r="F26" s="48"/>
+      <c r="G26" s="48"/>
+      <c r="H26" s="48"/>
     </row>
     <row r="27" ht="21.75">
-      <c r="A27" s="45"/>
-      <c r="B27" s="24"/>
-      <c r="C27" s="24"/>
-      <c r="D27" s="24"/>
-      <c r="E27" s="45"/>
-      <c r="F27" s="45"/>
-      <c r="G27" s="45"/>
-      <c r="H27" s="45"/>
+      <c r="A27" s="48"/>
+      <c r="B27" s="29"/>
+      <c r="C27" s="29"/>
+      <c r="D27" s="29"/>
+      <c r="E27" s="48"/>
+      <c r="F27" s="48"/>
+      <c r="G27" s="48"/>
+      <c r="H27" s="48"/>
     </row>
     <row r="28" ht="14.25">
-      <c r="A28" s="46"/>
-      <c r="B28" s="23"/>
-      <c r="C28" s="23"/>
-      <c r="D28" s="24"/>
-      <c r="E28" s="24"/>
-      <c r="F28" s="24"/>
-      <c r="G28" s="23"/>
-      <c r="H28" s="24"/>
+      <c r="A28" s="39"/>
+      <c r="B28" s="28"/>
+      <c r="C28" s="28"/>
+      <c r="D28" s="29"/>
+      <c r="E28" s="29"/>
+      <c r="F28" s="29"/>
+      <c r="G28" s="28"/>
+      <c r="H28" s="29"/>
     </row>
     <row r="29" ht="14.25">
-      <c r="A29" s="23"/>
-      <c r="B29" s="23"/>
-      <c r="C29" s="23"/>
-      <c r="D29" s="24"/>
-      <c r="E29" s="24"/>
-      <c r="F29" s="24"/>
-      <c r="G29" s="23"/>
-      <c r="H29" s="24"/>
+      <c r="A29" s="28"/>
+      <c r="B29" s="28"/>
+      <c r="C29" s="28"/>
+      <c r="D29" s="29"/>
+      <c r="E29" s="29"/>
+      <c r="F29" s="29"/>
+      <c r="G29" s="28"/>
+      <c r="H29" s="29"/>
     </row>
     <row r="30" ht="14.25">
-      <c r="A30" s="23"/>
-      <c r="B30" s="23"/>
-      <c r="C30" s="23"/>
-      <c r="D30" s="24"/>
-      <c r="E30" s="24"/>
-      <c r="F30" s="24"/>
-      <c r="G30" s="23"/>
-      <c r="H30" s="24"/>
+      <c r="A30" s="28"/>
+      <c r="B30" s="28"/>
+      <c r="C30" s="28"/>
+      <c r="D30" s="29"/>
+      <c r="E30" s="29"/>
+      <c r="F30" s="29"/>
+      <c r="G30" s="28"/>
+      <c r="H30" s="29"/>
     </row>
     <row r="31" ht="14.25">
-      <c r="A31" s="23"/>
-      <c r="B31" s="23"/>
-      <c r="C31" s="23"/>
-      <c r="D31" s="24"/>
-      <c r="E31" s="24"/>
-      <c r="F31" s="24"/>
-      <c r="G31" s="23"/>
-      <c r="H31" s="24"/>
+      <c r="A31" s="28"/>
+      <c r="B31" s="28"/>
+      <c r="C31" s="28"/>
+      <c r="D31" s="29"/>
+      <c r="E31" s="29"/>
+      <c r="F31" s="29"/>
+      <c r="G31" s="28"/>
+      <c r="H31" s="29"/>
     </row>
     <row r="32" ht="14.25">
-      <c r="A32" s="23"/>
-      <c r="B32" s="23"/>
-      <c r="C32" s="23"/>
-      <c r="D32" s="24"/>
-      <c r="E32" s="24"/>
-      <c r="F32" s="24"/>
-      <c r="G32" s="23"/>
-      <c r="H32" s="24"/>
+      <c r="A32" s="28"/>
+      <c r="B32" s="28"/>
+      <c r="C32" s="28"/>
+      <c r="D32" s="29"/>
+      <c r="E32" s="29"/>
+      <c r="F32" s="29"/>
+      <c r="G32" s="28"/>
+      <c r="H32" s="29"/>
     </row>
     <row r="33" ht="14.25">
-      <c r="A33" s="23"/>
-      <c r="B33" s="23"/>
-      <c r="C33" s="23"/>
-      <c r="D33" s="24"/>
-      <c r="E33" s="24"/>
-      <c r="F33" s="24"/>
-      <c r="G33" s="23"/>
-      <c r="H33" s="24"/>
+      <c r="A33" s="28"/>
+      <c r="B33" s="28"/>
+      <c r="C33" s="28"/>
+      <c r="D33" s="29"/>
+      <c r="E33" s="29"/>
+      <c r="F33" s="29"/>
+      <c r="G33" s="28"/>
+      <c r="H33" s="29"/>
     </row>
     <row r="34" ht="14.25">
-      <c r="A34" s="23"/>
-      <c r="B34" s="23"/>
-      <c r="C34" s="23"/>
-      <c r="D34" s="24"/>
-      <c r="E34" s="24"/>
-      <c r="F34" s="24"/>
-      <c r="G34" s="23"/>
-      <c r="H34" s="24"/>
+      <c r="A34" s="28"/>
+      <c r="B34" s="28"/>
+      <c r="C34" s="28"/>
+      <c r="D34" s="29"/>
+      <c r="E34" s="29"/>
+      <c r="F34" s="29"/>
+      <c r="G34" s="28"/>
+      <c r="H34" s="29"/>
     </row>
     <row r="35" ht="14.25">
-      <c r="A35" s="23"/>
+      <c r="A35" s="28"/>
     </row>
     <row r="36" ht="14.25">
-      <c r="A36" s="23"/>
+      <c r="A36" s="28"/>
     </row>
     <row r="37" ht="14.25">
-      <c r="A37" s="23"/>
+      <c r="A37" s="28"/>
     </row>
     <row r="38" ht="14.25">
-      <c r="A38" s="23"/>
+      <c r="A38" s="28"/>
     </row>
     <row r="39" ht="14.25">
-      <c r="A39" s="23"/>
+      <c r="A39" s="28"/>
     </row>
     <row r="40" ht="14.25">
-      <c r="A40" s="23"/>
+      <c r="A40" s="28"/>
     </row>
     <row r="41" ht="14.25">
-      <c r="A41" s="23"/>
-      <c r="B41" s="23"/>
-      <c r="C41" s="23"/>
-      <c r="D41" s="24"/>
-      <c r="E41" s="24"/>
-      <c r="F41" s="24"/>
-      <c r="G41" s="23"/>
-      <c r="H41" s="24"/>
+      <c r="A41" s="28"/>
+      <c r="B41" s="28"/>
+      <c r="C41" s="28"/>
+      <c r="D41" s="29"/>
+      <c r="E41" s="29"/>
+      <c r="F41" s="29"/>
+      <c r="G41" s="28"/>
+      <c r="H41" s="29"/>
     </row>
     <row r="42" ht="14.25">
-      <c r="A42" s="23"/>
-      <c r="B42" s="23"/>
-      <c r="C42" s="23"/>
-      <c r="D42" s="24"/>
-      <c r="E42" s="24"/>
-      <c r="F42" s="24"/>
-      <c r="G42" s="23"/>
-      <c r="H42" s="24"/>
+      <c r="A42" s="28"/>
+      <c r="B42" s="28"/>
+      <c r="C42" s="28"/>
+      <c r="D42" s="29"/>
+      <c r="E42" s="29"/>
+      <c r="F42" s="29"/>
+      <c r="G42" s="28"/>
+      <c r="H42" s="29"/>
     </row>
     <row r="43" ht="14.25">
-      <c r="A43" s="23"/>
-      <c r="E43" s="24"/>
-      <c r="F43" s="24"/>
-      <c r="G43" s="23"/>
-      <c r="H43" s="24"/>
+      <c r="A43" s="28"/>
+      <c r="E43" s="29"/>
+      <c r="F43" s="29"/>
+      <c r="G43" s="28"/>
+      <c r="H43" s="29"/>
     </row>
     <row r="44" ht="14.25">
-      <c r="A44" s="23"/>
-      <c r="B44" s="23"/>
-      <c r="C44" s="23"/>
-      <c r="D44" s="24"/>
-      <c r="E44" s="24"/>
-      <c r="F44" s="24"/>
-      <c r="G44" s="23"/>
-      <c r="H44" s="24"/>
+      <c r="A44" s="28"/>
+      <c r="B44" s="28"/>
+      <c r="C44" s="28"/>
+      <c r="D44" s="29"/>
+      <c r="E44" s="29"/>
+      <c r="F44" s="29"/>
+      <c r="G44" s="28"/>
+      <c r="H44" s="29"/>
     </row>
     <row r="45" ht="14.25">
-      <c r="A45" s="23"/>
-      <c r="E45" s="24"/>
-      <c r="F45" s="24"/>
-      <c r="G45" s="23"/>
-      <c r="H45" s="24"/>
+      <c r="A45" s="28"/>
+      <c r="E45" s="29"/>
+      <c r="F45" s="29"/>
+      <c r="G45" s="28"/>
+      <c r="H45" s="29"/>
     </row>
     <row r="46" ht="14.25">
-      <c r="A46" s="23"/>
+      <c r="A46" s="28"/>
     </row>
   </sheetData>
   <mergeCells count="24">

</xml_diff>

<commit_message>
modified the summary generation to have more concise details
</commit_message>
<xml_diff>
--- a/core/UAT Plan.xlsx
+++ b/core/UAT Plan.xlsx
@@ -241,6 +241,21 @@
     <t xml:space="preserve">Patient 6</t>
   </si>
   <si>
+    <t xml:space="preserve">Patient 7</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Patient 8</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Patient 9</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Patient 10</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Patient 11</t>
+  </si>
+  <si>
     <t xml:space="preserve">Oral and Maxillofacial Surgery</t>
   </si>
   <si>
@@ -372,9 +387,6 @@
     <t xml:space="preserve">Requires failed PPI therapy (min. 4–8 weeks), H. pylori test result, or documented alarm symptoms (dysphagia, weight loss, hematemesis)</t>
   </si>
   <si>
-    <t xml:space="preserve">Patient 7</t>
-  </si>
-  <si>
     <t>45378</t>
   </si>
   <si>
@@ -401,9 +413,6 @@
     <t xml:space="preserve">Requires documentation of high-risk criteria (age 45+, family history of CRC, prior polyps, IBD diagnosis) or symptomatic indicators with clinical notes (persistent bleeding, iron deficiency anemia)</t>
   </si>
   <si>
-    <t xml:space="preserve">Patient 8</t>
-  </si>
-  <si>
     <t xml:space="preserve">1. Initial visit with vague upper abdominal discomfort
 2. No prior PPI trial documented
 3. No H. pylori testing ordered</t>
@@ -420,9 +429,6 @@
     <t xml:space="preserve">Failed PPI trial documented; positive H. pylori confirmed; alarm symptoms (dysphagia, weight loss) present — all criteria met</t>
   </si>
   <si>
-    <t xml:space="preserve">Patient 9</t>
-  </si>
-  <si>
     <t xml:space="preserve">1. Patient age 38 with no family history documented
 2. Single episode of loose stool reported
 3. No prior imaging or lab workup</t>
@@ -439,9 +445,6 @@
     <t xml:space="preserve">Age criteria met; high-risk family history confirmed; prior polyp history documented with specialist order</t>
   </si>
   <si>
-    <t xml:space="preserve">Patient 10</t>
-  </si>
-  <si>
     <t>OB/GYN</t>
   </si>
   <si>
@@ -471,9 +474,6 @@
   </si>
   <si>
     <t xml:space="preserve">Requires confirmed intrauterine pregnancy ≤10 weeks gestation; provider must be certified under REMS program; documentation of informed consent and patient counseling</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Patient 11</t>
   </si>
   <si>
     <t xml:space="preserve">Physical Therapy</t>
@@ -668,7 +668,7 @@
   <cellStyleXfs count="1">
     <xf fontId="0" fillId="0" borderId="0" numFmtId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
   </cellStyleXfs>
-  <cellXfs count="49">
+  <cellXfs count="52">
     <xf fontId="0" fillId="0" borderId="0" numFmtId="0" xfId="0"/>
     <xf fontId="0" fillId="0" borderId="0" numFmtId="0" xfId="0" applyAlignment="1">
       <alignment vertical="center"/>
@@ -737,14 +737,23 @@
     <xf fontId="0" fillId="0" borderId="0" numFmtId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf fontId="0" fillId="3" borderId="2" numFmtId="0" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf fontId="0" fillId="3" borderId="2" numFmtId="0" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
     <xf fontId="0" fillId="0" borderId="1" numFmtId="0" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf fontId="0" fillId="3" borderId="2" numFmtId="0" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf fontId="0" fillId="0" borderId="2" numFmtId="0" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf fontId="0" fillId="3" borderId="2" numFmtId="0" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf fontId="0" fillId="0" borderId="2" numFmtId="0" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf fontId="2" fillId="0" borderId="1" numFmtId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
     </xf>
     <xf fontId="0" fillId="0" borderId="1" numFmtId="0" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -1945,14 +1954,14 @@
       <c r="J11" s="1"/>
     </row>
     <row r="12" ht="14.25">
-      <c r="A12" s="24" t="s">
+      <c r="A12" s="8" t="s">
         <v>71</v>
       </c>
       <c r="B12" s="23"/>
-      <c r="C12" s="25">
+      <c r="C12" s="24">
         <v>36558</v>
       </c>
-      <c r="D12" s="26" t="s">
+      <c r="D12" s="25" t="s">
         <v>51</v>
       </c>
       <c r="E12" s="11" t="s">
@@ -1964,7 +1973,7 @@
       <c r="G12" s="13" t="s">
         <v>13</v>
       </c>
-      <c r="H12" s="26" t="s">
+      <c r="H12" s="25" t="s">
         <v>53</v>
       </c>
       <c r="I12" s="1">
@@ -1972,7 +1981,7 @@
       </c>
     </row>
     <row r="13" ht="28.5">
-      <c r="A13" s="24" t="s">
+      <c r="A13" s="8" t="s">
         <v>71</v>
       </c>
       <c r="B13" s="23"/>
@@ -1992,9 +2001,255 @@
         <v>2231</v>
       </c>
     </row>
+    <row r="14" ht="28.5">
+      <c r="A14" s="26" t="s">
+        <v>72</v>
+      </c>
+      <c r="B14" s="23"/>
+      <c r="C14" s="24">
+        <v>90999</v>
+      </c>
+      <c r="D14" s="25" t="s">
+        <v>45</v>
+      </c>
+      <c r="E14" s="11" t="s">
+        <v>46</v>
+      </c>
+      <c r="F14" s="12" t="s">
+        <v>47</v>
+      </c>
+      <c r="G14" s="13" t="s">
+        <v>21</v>
+      </c>
+      <c r="H14" s="25" t="s">
+        <v>48</v>
+      </c>
+      <c r="I14" s="1">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="15" ht="28.5">
+      <c r="A15" s="26" t="s">
+        <v>72</v>
+      </c>
+      <c r="B15" s="23"/>
+      <c r="C15" s="9"/>
+      <c r="D15" s="11"/>
+      <c r="E15" s="11" t="s">
+        <v>49</v>
+      </c>
+      <c r="F15" s="12" t="s">
+        <v>50</v>
+      </c>
+      <c r="G15" s="13" t="s">
+        <v>17</v>
+      </c>
+      <c r="H15" s="11"/>
+      <c r="I15" s="1">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="16" ht="14.25">
+      <c r="A16" s="26" t="s">
+        <v>73</v>
+      </c>
+      <c r="B16" s="23"/>
+      <c r="C16" s="24">
+        <v>36558</v>
+      </c>
+      <c r="D16" s="25" t="s">
+        <v>51</v>
+      </c>
+      <c r="E16" s="11" t="s">
+        <v>46</v>
+      </c>
+      <c r="F16" s="12" t="s">
+        <v>52</v>
+      </c>
+      <c r="G16" s="13" t="s">
+        <v>13</v>
+      </c>
+      <c r="H16" s="25" t="s">
+        <v>53</v>
+      </c>
+      <c r="I16" s="1">
+        <v>112</v>
+      </c>
+    </row>
+    <row r="17" ht="28.5">
+      <c r="A17" s="8" t="s">
+        <v>73</v>
+      </c>
+      <c r="B17" s="23"/>
+      <c r="C17" s="9"/>
+      <c r="D17" s="11"/>
+      <c r="E17" s="11" t="s">
+        <v>54</v>
+      </c>
+      <c r="F17" s="12" t="s">
+        <v>55</v>
+      </c>
+      <c r="G17" s="13" t="s">
+        <v>17</v>
+      </c>
+      <c r="H17" s="11"/>
+      <c r="I17" s="1">
+        <v>113</v>
+      </c>
+    </row>
+    <row r="18" ht="28.5">
+      <c r="A18" s="26" t="s">
+        <v>74</v>
+      </c>
+      <c r="B18" s="23"/>
+      <c r="C18" s="27">
+        <v>50360</v>
+      </c>
+      <c r="D18" s="28" t="s">
+        <v>56</v>
+      </c>
+      <c r="E18" s="17" t="s">
+        <v>57</v>
+      </c>
+      <c r="F18" s="29" t="s">
+        <v>58</v>
+      </c>
+      <c r="G18" s="19" t="s">
+        <v>21</v>
+      </c>
+      <c r="H18" s="28" t="s">
+        <v>59</v>
+      </c>
+      <c r="I18" s="1">
+        <v>114</v>
+      </c>
+    </row>
+    <row r="19" ht="28.5">
+      <c r="A19" s="26" t="s">
+        <v>74</v>
+      </c>
+      <c r="B19" s="23"/>
+      <c r="C19" s="8"/>
+      <c r="D19" s="17"/>
+      <c r="E19" s="17" t="s">
+        <v>60</v>
+      </c>
+      <c r="F19" s="29" t="s">
+        <v>61</v>
+      </c>
+      <c r="G19" s="19" t="s">
+        <v>17</v>
+      </c>
+      <c r="H19" s="17"/>
+      <c r="I19" s="1">
+        <v>115</v>
+      </c>
+    </row>
+    <row r="20" ht="14.25">
+      <c r="A20" s="26" t="s">
+        <v>75</v>
+      </c>
+      <c r="B20" s="23"/>
+      <c r="C20" s="27">
+        <v>50394</v>
+      </c>
+      <c r="D20" s="28" t="s">
+        <v>62</v>
+      </c>
+      <c r="E20" s="17" t="s">
+        <v>63</v>
+      </c>
+      <c r="F20" s="20" t="s">
+        <v>64</v>
+      </c>
+      <c r="G20" s="19" t="s">
+        <v>13</v>
+      </c>
+      <c r="H20" s="28" t="s">
+        <v>65</v>
+      </c>
+      <c r="I20" s="1">
+        <v>116</v>
+      </c>
+    </row>
+    <row r="21" ht="14.25">
+      <c r="A21" s="8" t="s">
+        <v>75</v>
+      </c>
+      <c r="B21" s="23"/>
+      <c r="C21" s="8"/>
+      <c r="D21" s="17"/>
+      <c r="E21" s="17" t="s">
+        <v>66</v>
+      </c>
+      <c r="F21" s="20" t="s">
+        <v>67</v>
+      </c>
+      <c r="G21" s="19" t="s">
+        <v>21</v>
+      </c>
+      <c r="H21" s="17"/>
+      <c r="I21" s="1">
+        <v>117</v>
+      </c>
+    </row>
+    <row r="22" ht="14.25">
+      <c r="A22" s="26" t="s">
+        <v>76</v>
+      </c>
+      <c r="B22" s="23"/>
+      <c r="C22" s="27">
+        <v>77012</v>
+      </c>
+      <c r="D22" s="28" t="s">
+        <v>68</v>
+      </c>
+      <c r="E22" s="17" t="s">
+        <v>46</v>
+      </c>
+      <c r="F22" s="20" t="s">
+        <v>64</v>
+      </c>
+      <c r="G22" s="19" t="s">
+        <v>13</v>
+      </c>
+      <c r="H22" s="28" t="s">
+        <v>69</v>
+      </c>
+      <c r="I22" s="1">
+        <v>118</v>
+      </c>
+    </row>
+    <row r="23" ht="42.75">
+      <c r="A23" s="8" t="s">
+        <v>76</v>
+      </c>
+      <c r="B23" s="23"/>
+      <c r="C23" s="8"/>
+      <c r="D23" s="17"/>
+      <c r="E23" s="17" t="s">
+        <v>70</v>
+      </c>
+      <c r="F23" s="20" t="s">
+        <v>67</v>
+      </c>
+      <c r="G23" s="19" t="s">
+        <v>17</v>
+      </c>
+      <c r="H23" s="17"/>
+      <c r="I23" s="1">
+        <v>119</v>
+      </c>
+    </row>
+    <row r="24" ht="14.25">
+      <c r="H24" s="25"/>
+    </row>
+    <row r="25" ht="14.25">
+      <c r="H25" s="11"/>
+    </row>
   </sheetData>
-  <mergeCells count="19">
-    <mergeCell ref="B2:B13"/>
+  <mergeCells count="35">
+    <mergeCell ref="B2:B23"/>
     <mergeCell ref="C2:C3"/>
     <mergeCell ref="D2:D3"/>
     <mergeCell ref="H2:H3"/>
@@ -2013,6 +2268,22 @@
     <mergeCell ref="C12:C13"/>
     <mergeCell ref="D12:D13"/>
     <mergeCell ref="H12:H13"/>
+    <mergeCell ref="C14:C15"/>
+    <mergeCell ref="D14:D15"/>
+    <mergeCell ref="H14:H15"/>
+    <mergeCell ref="C16:C17"/>
+    <mergeCell ref="D16:D17"/>
+    <mergeCell ref="H16:H17"/>
+    <mergeCell ref="C18:C19"/>
+    <mergeCell ref="D18:D19"/>
+    <mergeCell ref="H18:H19"/>
+    <mergeCell ref="C20:C21"/>
+    <mergeCell ref="D20:D21"/>
+    <mergeCell ref="H20:H21"/>
+    <mergeCell ref="C22:C23"/>
+    <mergeCell ref="D22:D23"/>
+    <mergeCell ref="H22:H23"/>
+    <mergeCell ref="H24:H25"/>
   </mergeCells>
   <printOptions headings="0" gridLines="0"/>
   <pageMargins left="0.69999999999999996" right="0.69999999999999996" top="0.75" bottom="0.75" header="0.29999999999999999" footer="0.29999999999999999"/>
@@ -2066,26 +2337,26 @@
       <c r="A2" s="8" t="s">
         <v>8</v>
       </c>
-      <c r="B2" s="27" t="s">
-        <v>72</v>
+      <c r="B2" s="30" t="s">
+        <v>77</v>
       </c>
       <c r="C2" s="8">
         <v>21141</v>
       </c>
       <c r="D2" s="17" t="s">
-        <v>73</v>
+        <v>78</v>
       </c>
       <c r="E2" s="17" t="s">
-        <v>74</v>
+        <v>79</v>
       </c>
       <c r="F2" s="20" t="s">
-        <v>75</v>
+        <v>80</v>
       </c>
       <c r="G2" s="19" t="s">
         <v>13</v>
       </c>
       <c r="H2" s="17" t="s">
-        <v>76</v>
+        <v>81</v>
       </c>
       <c r="I2" s="1">
         <v>230</v>
@@ -2096,17 +2367,17 @@
       <c r="A3" s="8" t="s">
         <v>8</v>
       </c>
-      <c r="B3" s="27"/>
+      <c r="B3" s="30"/>
       <c r="C3" s="8"/>
       <c r="D3" s="17"/>
       <c r="E3" s="17" t="s">
-        <v>77</v>
+        <v>82</v>
       </c>
       <c r="F3" s="20" t="s">
-        <v>78</v>
+        <v>83</v>
       </c>
       <c r="G3" s="19" t="s">
-        <v>79</v>
+        <v>84</v>
       </c>
       <c r="H3" s="17"/>
       <c r="I3" s="1">
@@ -2118,24 +2389,24 @@
       <c r="A4" s="8" t="s">
         <v>18</v>
       </c>
-      <c r="B4" s="27"/>
+      <c r="B4" s="30"/>
       <c r="C4" s="8">
         <v>21196</v>
       </c>
       <c r="D4" s="17" t="s">
-        <v>80</v>
+        <v>85</v>
       </c>
       <c r="E4" s="17" t="s">
-        <v>81</v>
+        <v>86</v>
       </c>
       <c r="F4" s="20" t="s">
-        <v>82</v>
+        <v>87</v>
       </c>
       <c r="G4" s="19" t="s">
         <v>13</v>
       </c>
       <c r="H4" s="17" t="s">
-        <v>83</v>
+        <v>88</v>
       </c>
       <c r="I4" s="1">
         <v>232</v>
@@ -2146,14 +2417,14 @@
       <c r="A5" s="8" t="s">
         <v>18</v>
       </c>
-      <c r="B5" s="27"/>
+      <c r="B5" s="30"/>
       <c r="C5" s="8"/>
       <c r="D5" s="17"/>
       <c r="E5" s="17" t="s">
-        <v>84</v>
+        <v>89</v>
       </c>
       <c r="F5" s="20" t="s">
-        <v>85</v>
+        <v>90</v>
       </c>
       <c r="G5" s="19" t="s">
         <v>17</v>
@@ -2168,24 +2439,24 @@
       <c r="A6" s="8" t="s">
         <v>25</v>
       </c>
-      <c r="B6" s="27"/>
+      <c r="B6" s="30"/>
       <c r="C6" s="8">
         <v>21210</v>
       </c>
       <c r="D6" s="17" t="s">
-        <v>86</v>
+        <v>91</v>
       </c>
       <c r="E6" s="17" t="s">
-        <v>87</v>
+        <v>92</v>
       </c>
       <c r="F6" s="18" t="s">
-        <v>88</v>
+        <v>93</v>
       </c>
       <c r="G6" s="19" t="s">
         <v>21</v>
       </c>
       <c r="H6" s="17" t="s">
-        <v>89</v>
+        <v>94</v>
       </c>
       <c r="I6" s="1">
         <v>234</v>
@@ -2196,14 +2467,14 @@
       <c r="A7" s="8" t="s">
         <v>25</v>
       </c>
-      <c r="B7" s="27"/>
+      <c r="B7" s="30"/>
       <c r="C7" s="8"/>
       <c r="D7" s="17"/>
       <c r="E7" s="17" t="s">
-        <v>90</v>
+        <v>95</v>
       </c>
       <c r="F7" s="18" t="s">
-        <v>91</v>
+        <v>96</v>
       </c>
       <c r="G7" s="19" t="s">
         <v>17</v>
@@ -2218,24 +2489,24 @@
       <c r="A8" s="8" t="s">
         <v>32</v>
       </c>
-      <c r="B8" s="27"/>
+      <c r="B8" s="30"/>
       <c r="C8" s="8">
         <v>21085</v>
       </c>
       <c r="D8" s="17" t="s">
-        <v>92</v>
+        <v>97</v>
       </c>
       <c r="E8" s="17" t="s">
-        <v>93</v>
+        <v>98</v>
       </c>
       <c r="F8" s="20" t="s">
-        <v>94</v>
+        <v>99</v>
       </c>
       <c r="G8" s="19" t="s">
         <v>13</v>
       </c>
       <c r="H8" s="17" t="s">
-        <v>95</v>
+        <v>100</v>
       </c>
       <c r="I8" s="1">
         <v>236</v>
@@ -2246,14 +2517,14 @@
       <c r="A9" s="8" t="s">
         <v>32</v>
       </c>
-      <c r="B9" s="27"/>
+      <c r="B9" s="30"/>
       <c r="C9" s="8"/>
       <c r="D9" s="17"/>
       <c r="E9" s="17" t="s">
-        <v>96</v>
+        <v>101</v>
       </c>
       <c r="F9" s="20" t="s">
-        <v>97</v>
+        <v>102</v>
       </c>
       <c r="G9" s="19" t="s">
         <v>21</v>
@@ -2268,24 +2539,24 @@
       <c r="A10" s="8" t="s">
         <v>38</v>
       </c>
-      <c r="B10" s="27"/>
+      <c r="B10" s="30"/>
       <c r="C10" s="8">
         <v>21235</v>
       </c>
       <c r="D10" s="17" t="s">
-        <v>98</v>
+        <v>103</v>
       </c>
       <c r="E10" s="17" t="s">
-        <v>99</v>
+        <v>104</v>
       </c>
       <c r="F10" s="20" t="s">
-        <v>100</v>
+        <v>105</v>
       </c>
       <c r="G10" s="19" t="s">
         <v>13</v>
       </c>
       <c r="H10" s="17" t="s">
-        <v>101</v>
+        <v>106</v>
       </c>
       <c r="I10" s="1">
         <v>238</v>
@@ -2296,14 +2567,14 @@
       <c r="A11" s="8" t="s">
         <v>38</v>
       </c>
-      <c r="B11" s="27"/>
+      <c r="B11" s="30"/>
       <c r="C11" s="8"/>
       <c r="D11" s="17"/>
       <c r="E11" s="17" t="s">
+        <v>107</v>
+      </c>
+      <c r="F11" s="20" t="s">
         <v>102</v>
-      </c>
-      <c r="F11" s="20" t="s">
-        <v>97</v>
       </c>
       <c r="G11" s="19" t="s">
         <v>17</v>
@@ -2347,704 +2618,704 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac">
   <sheetFormatPr defaultRowHeight="14.25"/>
   <cols>
-    <col customWidth="1" min="1" max="1" style="28" width="12"/>
-    <col bestFit="1" customWidth="1" min="2" max="2" style="28" width="11.85546875"/>
-    <col min="3" max="3" style="28" width="9.140625"/>
-    <col customWidth="1" min="4" max="5" style="29" width="42.85546875"/>
-    <col customWidth="1" min="6" max="6" style="29" width="30.85546875"/>
-    <col bestFit="1" customWidth="1" min="7" max="7" style="28" width="17.5703125"/>
-    <col customWidth="1" min="8" max="8" style="29" width="46.42578125"/>
-    <col min="9" max="16384" style="28" width="9.140625"/>
+    <col customWidth="1" min="1" max="1" style="31" width="12"/>
+    <col bestFit="1" customWidth="1" min="2" max="2" style="31" width="11.85546875"/>
+    <col min="3" max="3" style="31" width="9.140625"/>
+    <col customWidth="1" min="4" max="5" style="32" width="42.85546875"/>
+    <col customWidth="1" min="6" max="6" style="32" width="30.85546875"/>
+    <col bestFit="1" customWidth="1" min="7" max="7" style="31" width="17.5703125"/>
+    <col customWidth="1" min="8" max="8" style="32" width="46.42578125"/>
+    <col min="9" max="16384" style="31" width="9.140625"/>
   </cols>
   <sheetData>
-    <row r="1" s="30" customFormat="1">
-      <c r="A1" s="31" t="s">
+    <row r="1" s="33" customFormat="1">
+      <c r="A1" s="34" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="31" t="s">
+      <c r="B1" s="34" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="31" t="s">
-        <v>103</v>
-      </c>
-      <c r="D1" s="32" t="s">
+      <c r="C1" s="34" t="s">
+        <v>108</v>
+      </c>
+      <c r="D1" s="35" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="32" t="s">
+      <c r="E1" s="35" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="32" t="s">
+      <c r="F1" s="35" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="31" t="s">
+      <c r="G1" s="34" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="31" t="s">
+      <c r="H1" s="34" t="s">
         <v>7</v>
       </c>
     </row>
     <row r="2" ht="57">
-      <c r="A2" s="33" t="s">
+      <c r="A2" s="36" t="s">
         <v>71</v>
       </c>
-      <c r="B2" s="34" t="s">
-        <v>104</v>
-      </c>
-      <c r="C2" s="35" t="s">
-        <v>105</v>
-      </c>
-      <c r="D2" s="36" t="s">
-        <v>106</v>
-      </c>
-      <c r="E2" s="37" t="s">
-        <v>107</v>
-      </c>
-      <c r="F2" s="37" t="s">
-        <v>108</v>
-      </c>
-      <c r="G2" s="38" t="s">
+      <c r="B2" s="37" t="s">
+        <v>109</v>
+      </c>
+      <c r="C2" s="38" t="s">
+        <v>110</v>
+      </c>
+      <c r="D2" s="39" t="s">
+        <v>111</v>
+      </c>
+      <c r="E2" s="40" t="s">
+        <v>112</v>
+      </c>
+      <c r="F2" s="40" t="s">
+        <v>113</v>
+      </c>
+      <c r="G2" s="41" t="s">
         <v>13</v>
       </c>
-      <c r="H2" s="37" t="s">
+      <c r="H2" s="40" t="s">
+        <v>114</v>
+      </c>
+      <c r="I2" s="42">
+        <v>260</v>
+      </c>
+      <c r="J2" s="31"/>
+    </row>
+    <row r="3" ht="50.25" customHeight="1">
+      <c r="A3" s="36" t="s">
+        <v>71</v>
+      </c>
+      <c r="B3" s="43"/>
+      <c r="C3" s="44"/>
+      <c r="D3" s="45"/>
+      <c r="E3" s="40" t="s">
+        <v>115</v>
+      </c>
+      <c r="F3" s="40" t="s">
+        <v>116</v>
+      </c>
+      <c r="G3" s="41" t="s">
+        <v>17</v>
+      </c>
+      <c r="H3" s="40" t="s">
+        <v>117</v>
+      </c>
+      <c r="I3" s="42">
+        <v>261</v>
+      </c>
+      <c r="J3" s="31"/>
+    </row>
+    <row r="4" ht="71.25">
+      <c r="A4" s="36" t="s">
+        <v>72</v>
+      </c>
+      <c r="B4" s="37" t="s">
         <v>109</v>
       </c>
-      <c r="I2" s="39">
-        <v>260</v>
-      </c>
-      <c r="J2" s="28"/>
-    </row>
-    <row r="3" ht="50.25" customHeight="1">
-      <c r="A3" s="33" t="s">
-        <v>71</v>
-      </c>
-      <c r="B3" s="40"/>
-      <c r="C3" s="41"/>
-      <c r="D3" s="42"/>
-      <c r="E3" s="37" t="s">
+      <c r="C4" s="38" t="s">
+        <v>118</v>
+      </c>
+      <c r="D4" s="39" t="s">
+        <v>119</v>
+      </c>
+      <c r="E4" s="40" t="s">
+        <v>120</v>
+      </c>
+      <c r="F4" s="40" t="s">
+        <v>121</v>
+      </c>
+      <c r="G4" s="41" t="s">
+        <v>13</v>
+      </c>
+      <c r="H4" s="40" t="s">
+        <v>122</v>
+      </c>
+      <c r="I4" s="42">
+        <v>262</v>
+      </c>
+      <c r="J4" s="31"/>
+    </row>
+    <row r="5" ht="57">
+      <c r="A5" s="36" t="s">
+        <v>72</v>
+      </c>
+      <c r="B5" s="43"/>
+      <c r="C5" s="44"/>
+      <c r="D5" s="45"/>
+      <c r="E5" s="40" t="s">
+        <v>123</v>
+      </c>
+      <c r="F5" s="40" t="s">
+        <v>124</v>
+      </c>
+      <c r="G5" s="41" t="s">
+        <v>17</v>
+      </c>
+      <c r="H5" s="40" t="s">
+        <v>125</v>
+      </c>
+      <c r="I5" s="42">
+        <v>263</v>
+      </c>
+      <c r="J5" s="31"/>
+    </row>
+    <row r="6" ht="57">
+      <c r="A6" s="36" t="s">
+        <v>73</v>
+      </c>
+      <c r="B6" s="37" t="s">
+        <v>109</v>
+      </c>
+      <c r="C6" s="38" t="s">
         <v>110</v>
       </c>
-      <c r="F3" s="37" t="s">
+      <c r="D6" s="39" t="s">
         <v>111</v>
       </c>
-      <c r="G3" s="38" t="s">
+      <c r="E6" s="40" t="s">
+        <v>126</v>
+      </c>
+      <c r="F6" s="40" t="s">
+        <v>127</v>
+      </c>
+      <c r="G6" s="41" t="s">
+        <v>13</v>
+      </c>
+      <c r="H6" s="40" t="s">
+        <v>114</v>
+      </c>
+      <c r="I6" s="42">
+        <v>264</v>
+      </c>
+      <c r="J6" s="31"/>
+    </row>
+    <row r="7" ht="108.75">
+      <c r="A7" s="36" t="s">
+        <v>73</v>
+      </c>
+      <c r="B7" s="43"/>
+      <c r="C7" s="44"/>
+      <c r="D7" s="45"/>
+      <c r="E7" s="46" t="s">
+        <v>128</v>
+      </c>
+      <c r="F7" s="46" t="s">
+        <v>129</v>
+      </c>
+      <c r="G7" s="46" t="s">
         <v>17</v>
       </c>
-      <c r="H3" s="37" t="s">
-        <v>112</v>
-      </c>
-      <c r="I3" s="39">
-        <v>261</v>
-      </c>
-      <c r="J3" s="28"/>
-    </row>
-    <row r="4" ht="71.25">
-      <c r="A4" s="33" t="s">
-        <v>113</v>
-      </c>
-      <c r="B4" s="34" t="s">
-        <v>104</v>
-      </c>
-      <c r="C4" s="35" t="s">
-        <v>114</v>
-      </c>
-      <c r="D4" s="36" t="s">
-        <v>115</v>
-      </c>
-      <c r="E4" s="37" t="s">
-        <v>116</v>
-      </c>
-      <c r="F4" s="37" t="s">
+      <c r="H7" s="46" t="s">
         <v>117</v>
       </c>
-      <c r="G4" s="38" t="s">
+      <c r="I7" s="42">
+        <v>265</v>
+      </c>
+      <c r="J7" s="31"/>
+    </row>
+    <row r="8" ht="108.75">
+      <c r="A8" s="36" t="s">
+        <v>74</v>
+      </c>
+      <c r="B8" s="37" t="s">
+        <v>109</v>
+      </c>
+      <c r="C8" s="38" t="s">
+        <v>118</v>
+      </c>
+      <c r="D8" s="47" t="s">
+        <v>119</v>
+      </c>
+      <c r="E8" s="46" t="s">
+        <v>130</v>
+      </c>
+      <c r="F8" s="46" t="s">
+        <v>131</v>
+      </c>
+      <c r="G8" s="46" t="s">
         <v>13</v>
       </c>
-      <c r="H4" s="37" t="s">
-        <v>118</v>
-      </c>
-      <c r="I4" s="39">
-        <v>262</v>
-      </c>
-      <c r="J4" s="28"/>
-    </row>
-    <row r="5" ht="57">
-      <c r="A5" s="33" t="s">
-        <v>113</v>
-      </c>
-      <c r="B5" s="40"/>
-      <c r="C5" s="41"/>
-      <c r="D5" s="42"/>
-      <c r="E5" s="37" t="s">
-        <v>119</v>
-      </c>
-      <c r="F5" s="37" t="s">
-        <v>120</v>
-      </c>
-      <c r="G5" s="38" t="s">
+      <c r="H8" s="46" t="s">
+        <v>122</v>
+      </c>
+      <c r="I8" s="42">
+        <v>266</v>
+      </c>
+      <c r="J8" s="31"/>
+    </row>
+    <row r="9" ht="108.75">
+      <c r="A9" s="36" t="s">
+        <v>74</v>
+      </c>
+      <c r="B9" s="43"/>
+      <c r="C9" s="44"/>
+      <c r="D9" s="48"/>
+      <c r="E9" s="46" t="s">
+        <v>132</v>
+      </c>
+      <c r="F9" s="46" t="s">
+        <v>133</v>
+      </c>
+      <c r="G9" s="46" t="s">
         <v>17</v>
       </c>
-      <c r="H5" s="37" t="s">
-        <v>121</v>
-      </c>
-      <c r="I5" s="39">
-        <v>263</v>
-      </c>
-      <c r="J5" s="28"/>
-    </row>
-    <row r="6" ht="57">
-      <c r="A6" s="33" t="s">
-        <v>122</v>
-      </c>
-      <c r="B6" s="34" t="s">
-        <v>104</v>
-      </c>
-      <c r="C6" s="35" t="s">
-        <v>105</v>
-      </c>
-      <c r="D6" s="36" t="s">
-        <v>106</v>
-      </c>
-      <c r="E6" s="37" t="s">
-        <v>123</v>
-      </c>
-      <c r="F6" s="37" t="s">
-        <v>124</v>
-      </c>
-      <c r="G6" s="38" t="s">
+      <c r="H9" s="46" t="s">
+        <v>125</v>
+      </c>
+      <c r="I9" s="42">
+        <v>267</v>
+      </c>
+      <c r="J9" s="31"/>
+    </row>
+    <row r="10" ht="108.75">
+      <c r="A10" s="36" t="s">
+        <v>75</v>
+      </c>
+      <c r="B10" s="37" t="s">
+        <v>134</v>
+      </c>
+      <c r="C10" s="38" t="s">
+        <v>135</v>
+      </c>
+      <c r="D10" s="47" t="s">
+        <v>136</v>
+      </c>
+      <c r="E10" s="46" t="s">
+        <v>137</v>
+      </c>
+      <c r="F10" s="46" t="s">
+        <v>138</v>
+      </c>
+      <c r="G10" s="46" t="s">
         <v>13</v>
       </c>
-      <c r="H6" s="37" t="s">
+      <c r="H10" s="46" t="s">
+        <v>139</v>
+      </c>
+      <c r="I10" s="42">
+        <v>268</v>
+      </c>
+      <c r="J10" s="31"/>
+    </row>
+    <row r="11" ht="87">
+      <c r="A11" s="36" t="s">
+        <v>75</v>
+      </c>
+      <c r="B11" s="43"/>
+      <c r="C11" s="44"/>
+      <c r="D11" s="48"/>
+      <c r="E11" s="46" t="s">
+        <v>140</v>
+      </c>
+      <c r="F11" s="46" t="s">
+        <v>141</v>
+      </c>
+      <c r="G11" s="46" t="s">
+        <v>21</v>
+      </c>
+      <c r="H11" s="46" t="s">
+        <v>142</v>
+      </c>
+      <c r="I11" s="42">
+        <v>269</v>
+      </c>
+      <c r="J11" s="31"/>
+    </row>
+    <row r="12" ht="71.25">
+      <c r="A12" s="42" t="s">
+        <v>76</v>
+      </c>
+      <c r="B12" s="49" t="s">
+        <v>143</v>
+      </c>
+      <c r="C12" s="42" t="s">
+        <v>144</v>
+      </c>
+      <c r="D12" s="32" t="s">
+        <v>145</v>
+      </c>
+      <c r="E12" s="32" t="s">
+        <v>146</v>
+      </c>
+      <c r="F12" s="32" t="s">
+        <v>147</v>
+      </c>
+      <c r="G12" s="41" t="s">
+        <v>17</v>
+      </c>
+      <c r="H12" s="32" t="s">
+        <v>142</v>
+      </c>
+      <c r="I12" s="42">
+        <v>270</v>
+      </c>
+    </row>
+    <row r="13" ht="71.25">
+      <c r="A13" s="42" t="s">
+        <v>76</v>
+      </c>
+      <c r="B13" s="49"/>
+      <c r="C13" s="42"/>
+      <c r="D13" s="32"/>
+      <c r="E13" s="32" t="s">
+        <v>148</v>
+      </c>
+      <c r="F13" s="32" t="s">
+        <v>149</v>
+      </c>
+      <c r="G13" s="41" t="s">
+        <v>13</v>
+      </c>
+      <c r="H13" s="32" t="s">
+        <v>150</v>
+      </c>
+      <c r="I13" s="42">
+        <v>271</v>
+      </c>
+    </row>
+    <row r="14" ht="57">
+      <c r="A14" s="36" t="s">
+        <v>151</v>
+      </c>
+      <c r="B14" s="37" t="s">
         <v>109</v>
       </c>
-      <c r="I6" s="39">
-        <v>264</v>
-      </c>
-      <c r="J6" s="28"/>
-    </row>
-    <row r="7" ht="108.75">
-      <c r="A7" s="33" t="s">
-        <v>122</v>
-      </c>
-      <c r="B7" s="40"/>
-      <c r="C7" s="41"/>
-      <c r="D7" s="42"/>
-      <c r="E7" s="43" t="s">
-        <v>125</v>
-      </c>
-      <c r="F7" s="43" t="s">
-        <v>126</v>
-      </c>
-      <c r="G7" s="43" t="s">
+      <c r="C14" s="38">
+        <v>45380</v>
+      </c>
+      <c r="D14" s="39" t="s">
+        <v>152</v>
+      </c>
+      <c r="E14" s="40" t="s">
+        <v>153</v>
+      </c>
+      <c r="F14" s="40" t="s">
+        <v>154</v>
+      </c>
+      <c r="G14" s="41" t="s">
         <v>17</v>
       </c>
-      <c r="H7" s="43" t="s">
-        <v>112</v>
-      </c>
-      <c r="I7" s="39">
-        <v>265</v>
-      </c>
-      <c r="J7" s="28"/>
-    </row>
-    <row r="8" ht="108.75">
-      <c r="A8" s="33" t="s">
-        <v>127</v>
-      </c>
-      <c r="B8" s="34" t="s">
-        <v>104</v>
-      </c>
-      <c r="C8" s="35" t="s">
-        <v>114</v>
-      </c>
-      <c r="D8" s="44" t="s">
-        <v>115</v>
-      </c>
-      <c r="E8" s="43" t="s">
-        <v>128</v>
-      </c>
-      <c r="F8" s="43" t="s">
-        <v>129</v>
-      </c>
-      <c r="G8" s="43" t="s">
+      <c r="H14" s="40" t="s">
+        <v>155</v>
+      </c>
+      <c r="I14" s="42">
+        <v>272</v>
+      </c>
+    </row>
+    <row r="15" ht="99.75">
+      <c r="A15" s="36" t="s">
+        <v>156</v>
+      </c>
+      <c r="B15" s="43"/>
+      <c r="C15" s="44"/>
+      <c r="D15" s="45"/>
+      <c r="E15" s="40" t="s">
+        <v>157</v>
+      </c>
+      <c r="F15" s="40" t="s">
+        <v>158</v>
+      </c>
+      <c r="G15" s="41" t="s">
         <v>13</v>
       </c>
-      <c r="H8" s="43" t="s">
-        <v>118</v>
-      </c>
-      <c r="I8" s="39">
-        <v>266</v>
-      </c>
-      <c r="J8" s="28"/>
-    </row>
-    <row r="9" ht="108.75">
-      <c r="A9" s="33" t="s">
-        <v>127</v>
-      </c>
-      <c r="B9" s="40"/>
-      <c r="C9" s="41"/>
-      <c r="D9" s="45"/>
-      <c r="E9" s="43" t="s">
-        <v>130</v>
-      </c>
-      <c r="F9" s="43" t="s">
-        <v>131</v>
-      </c>
-      <c r="G9" s="43" t="s">
+      <c r="H15" s="40" t="s">
+        <v>159</v>
+      </c>
+      <c r="I15" s="42">
+        <v>273</v>
+      </c>
+    </row>
+    <row r="16" ht="85.5">
+      <c r="A16" s="36" t="s">
+        <v>151</v>
+      </c>
+      <c r="B16" s="37" t="s">
+        <v>109</v>
+      </c>
+      <c r="C16" s="38">
+        <v>43235</v>
+      </c>
+      <c r="D16" s="39" t="s">
+        <v>160</v>
+      </c>
+      <c r="E16" s="40" t="s">
+        <v>161</v>
+      </c>
+      <c r="F16" s="40" t="s">
+        <v>162</v>
+      </c>
+      <c r="G16" s="41" t="s">
         <v>17</v>
       </c>
-      <c r="H9" s="43" t="s">
-        <v>121</v>
-      </c>
-      <c r="I9" s="39">
-        <v>267</v>
-      </c>
-      <c r="J9" s="28"/>
-    </row>
-    <row r="10" ht="108.75">
-      <c r="A10" s="33" t="s">
-        <v>132</v>
-      </c>
-      <c r="B10" s="34" t="s">
-        <v>133</v>
-      </c>
-      <c r="C10" s="35" t="s">
-        <v>134</v>
-      </c>
-      <c r="D10" s="44" t="s">
-        <v>135</v>
-      </c>
-      <c r="E10" s="43" t="s">
-        <v>136</v>
-      </c>
-      <c r="F10" s="43" t="s">
-        <v>137</v>
-      </c>
-      <c r="G10" s="43" t="s">
+      <c r="H16" s="40" t="s">
+        <v>163</v>
+      </c>
+      <c r="I16" s="42">
+        <v>274</v>
+      </c>
+    </row>
+    <row r="17" ht="71.25">
+      <c r="A17" s="36" t="s">
+        <v>156</v>
+      </c>
+      <c r="B17" s="43"/>
+      <c r="C17" s="44"/>
+      <c r="D17" s="45"/>
+      <c r="E17" s="40" t="s">
+        <v>164</v>
+      </c>
+      <c r="F17" s="40" t="s">
+        <v>165</v>
+      </c>
+      <c r="G17" s="41" t="s">
         <v>13</v>
       </c>
-      <c r="H10" s="43" t="s">
-        <v>138</v>
-      </c>
-      <c r="I10" s="39">
-        <v>268</v>
-      </c>
-      <c r="J10" s="28"/>
-    </row>
-    <row r="11" ht="87">
-      <c r="A11" s="33" t="s">
-        <v>132</v>
-      </c>
-      <c r="B11" s="40"/>
-      <c r="C11" s="41"/>
-      <c r="D11" s="45"/>
-      <c r="E11" s="43" t="s">
-        <v>139</v>
-      </c>
-      <c r="F11" s="43" t="s">
-        <v>140</v>
-      </c>
-      <c r="G11" s="43" t="s">
-        <v>21</v>
-      </c>
-      <c r="H11" s="43" t="s">
-        <v>141</v>
-      </c>
-      <c r="I11" s="39">
-        <v>269</v>
-      </c>
-      <c r="J11" s="28"/>
-    </row>
-    <row r="12" ht="71.25">
-      <c r="A12" s="39" t="s">
-        <v>142</v>
-      </c>
-      <c r="B12" s="46" t="s">
-        <v>143</v>
-      </c>
-      <c r="C12" s="39" t="s">
-        <v>144</v>
-      </c>
-      <c r="D12" s="29" t="s">
-        <v>145</v>
-      </c>
-      <c r="E12" s="29" t="s">
-        <v>146</v>
-      </c>
-      <c r="F12" s="29" t="s">
-        <v>147</v>
-      </c>
-      <c r="G12" s="38" t="s">
-        <v>17</v>
-      </c>
-      <c r="H12" s="29" t="s">
-        <v>141</v>
-      </c>
-      <c r="I12" s="39">
-        <v>270</v>
-      </c>
-    </row>
-    <row r="13" ht="71.25">
-      <c r="A13" s="39" t="s">
-        <v>142</v>
-      </c>
-      <c r="B13" s="46"/>
-      <c r="C13" s="39"/>
-      <c r="D13" s="29"/>
-      <c r="E13" s="29" t="s">
-        <v>148</v>
-      </c>
-      <c r="F13" s="29" t="s">
-        <v>149</v>
-      </c>
-      <c r="G13" s="38" t="s">
-        <v>13</v>
-      </c>
-      <c r="H13" s="29" t="s">
-        <v>150</v>
-      </c>
-      <c r="I13" s="39">
-        <v>271</v>
-      </c>
-    </row>
-    <row r="14" ht="57">
-      <c r="A14" s="33" t="s">
-        <v>151</v>
-      </c>
-      <c r="B14" s="34" t="s">
-        <v>104</v>
-      </c>
-      <c r="C14" s="35">
-        <v>45380</v>
-      </c>
-      <c r="D14" s="36" t="s">
-        <v>152</v>
-      </c>
-      <c r="E14" s="37" t="s">
-        <v>153</v>
-      </c>
-      <c r="F14" s="37" t="s">
-        <v>154</v>
-      </c>
-      <c r="G14" s="38" t="s">
-        <v>17</v>
-      </c>
-      <c r="H14" s="37" t="s">
-        <v>155</v>
-      </c>
-      <c r="I14" s="39">
-        <v>272</v>
-      </c>
-    </row>
-    <row r="15" ht="99.75">
-      <c r="A15" s="33" t="s">
-        <v>156</v>
-      </c>
-      <c r="B15" s="40"/>
-      <c r="C15" s="41"/>
-      <c r="D15" s="42"/>
-      <c r="E15" s="37" t="s">
-        <v>157</v>
-      </c>
-      <c r="F15" s="37" t="s">
-        <v>158</v>
-      </c>
-      <c r="G15" s="38" t="s">
-        <v>13</v>
-      </c>
-      <c r="H15" s="37" t="s">
-        <v>159</v>
-      </c>
-      <c r="I15" s="39">
-        <v>273</v>
-      </c>
-    </row>
-    <row r="16" ht="85.5">
-      <c r="A16" s="33" t="s">
-        <v>151</v>
-      </c>
-      <c r="B16" s="34" t="s">
-        <v>104</v>
-      </c>
-      <c r="C16" s="35">
-        <v>43235</v>
-      </c>
-      <c r="D16" s="36" t="s">
-        <v>160</v>
-      </c>
-      <c r="E16" s="37" t="s">
-        <v>161</v>
-      </c>
-      <c r="F16" s="37" t="s">
-        <v>162</v>
-      </c>
-      <c r="G16" s="38" t="s">
-        <v>17</v>
-      </c>
-      <c r="H16" s="37" t="s">
-        <v>163</v>
-      </c>
-      <c r="I16" s="39">
-        <v>274</v>
-      </c>
-    </row>
-    <row r="17" ht="71.25">
-      <c r="A17" s="33" t="s">
-        <v>156</v>
-      </c>
-      <c r="B17" s="40"/>
-      <c r="C17" s="41"/>
-      <c r="D17" s="42"/>
-      <c r="E17" s="37" t="s">
-        <v>164</v>
-      </c>
-      <c r="F17" s="37" t="s">
-        <v>165</v>
-      </c>
-      <c r="G17" s="38" t="s">
-        <v>13</v>
-      </c>
-      <c r="H17" s="37" t="s">
+      <c r="H17" s="40" t="s">
         <v>166</v>
       </c>
-      <c r="I17" s="39">
+      <c r="I17" s="42">
         <v>275</v>
       </c>
     </row>
     <row r="18" ht="14.25">
-      <c r="A18" s="28"/>
-      <c r="B18" s="28"/>
-      <c r="C18" s="28"/>
-      <c r="D18" s="29"/>
-      <c r="E18" s="29"/>
-      <c r="F18" s="29"/>
-      <c r="G18" s="28"/>
-      <c r="H18" s="29"/>
-      <c r="I18" s="28"/>
+      <c r="A18" s="31"/>
+      <c r="B18" s="31"/>
+      <c r="C18" s="31"/>
+      <c r="D18" s="32"/>
+      <c r="E18" s="32"/>
+      <c r="F18" s="32"/>
+      <c r="G18" s="31"/>
+      <c r="H18" s="32"/>
+      <c r="I18" s="31"/>
     </row>
     <row r="19" ht="14.25">
-      <c r="A19" s="28"/>
-      <c r="B19" s="28"/>
-      <c r="C19" s="28"/>
-      <c r="D19" s="29"/>
-      <c r="E19" s="29"/>
-      <c r="F19" s="29"/>
-      <c r="G19" s="28"/>
-      <c r="H19" s="29"/>
-      <c r="I19" s="28"/>
+      <c r="A19" s="31"/>
+      <c r="B19" s="31"/>
+      <c r="C19" s="31"/>
+      <c r="D19" s="32"/>
+      <c r="E19" s="32"/>
+      <c r="F19" s="32"/>
+      <c r="G19" s="31"/>
+      <c r="H19" s="32"/>
+      <c r="I19" s="31"/>
     </row>
     <row r="20" ht="14.25">
-      <c r="A20" s="28"/>
-      <c r="B20" s="28"/>
-      <c r="C20" s="28"/>
-      <c r="D20" s="29"/>
-      <c r="E20" s="29"/>
-      <c r="F20" s="29"/>
-      <c r="G20" s="28"/>
-      <c r="H20" s="29"/>
+      <c r="A20" s="31"/>
+      <c r="B20" s="31"/>
+      <c r="C20" s="31"/>
+      <c r="D20" s="32"/>
+      <c r="E20" s="32"/>
+      <c r="F20" s="32"/>
+      <c r="G20" s="31"/>
+      <c r="H20" s="32"/>
     </row>
     <row r="21" ht="14.25">
-      <c r="A21" s="28"/>
-      <c r="B21" s="28"/>
-      <c r="C21" s="28"/>
-      <c r="D21" s="29"/>
-      <c r="E21" s="29"/>
-      <c r="F21" s="29"/>
-      <c r="G21" s="28"/>
-      <c r="H21" s="29"/>
+      <c r="A21" s="31"/>
+      <c r="B21" s="31"/>
+      <c r="C21" s="31"/>
+      <c r="D21" s="32"/>
+      <c r="E21" s="32"/>
+      <c r="F21" s="32"/>
+      <c r="G21" s="31"/>
+      <c r="H21" s="32"/>
     </row>
     <row r="22" ht="14.25">
-      <c r="A22" s="28"/>
-      <c r="B22" s="28"/>
-      <c r="C22" s="28"/>
-      <c r="D22" s="29"/>
-      <c r="E22" s="29"/>
-      <c r="F22" s="29"/>
-      <c r="G22" s="28"/>
-      <c r="H22" s="29"/>
+      <c r="A22" s="31"/>
+      <c r="B22" s="31"/>
+      <c r="C22" s="31"/>
+      <c r="D22" s="32"/>
+      <c r="E22" s="32"/>
+      <c r="F22" s="32"/>
+      <c r="G22" s="31"/>
+      <c r="H22" s="32"/>
     </row>
     <row r="23" ht="21.75">
-      <c r="A23" s="47"/>
-      <c r="B23" s="47"/>
-      <c r="C23" s="47"/>
-      <c r="D23" s="47"/>
-      <c r="E23" s="47"/>
-      <c r="F23" s="47"/>
-      <c r="G23" s="47"/>
-      <c r="H23" s="47"/>
+      <c r="A23" s="50"/>
+      <c r="B23" s="50"/>
+      <c r="C23" s="50"/>
+      <c r="D23" s="50"/>
+      <c r="E23" s="50"/>
+      <c r="F23" s="50"/>
+      <c r="G23" s="50"/>
+      <c r="H23" s="50"/>
     </row>
     <row r="24" ht="21.75">
-      <c r="A24" s="48"/>
-      <c r="B24" s="48"/>
-      <c r="C24" s="48"/>
-      <c r="D24" s="48"/>
-      <c r="E24" s="48"/>
-      <c r="F24" s="48"/>
-      <c r="G24" s="48"/>
-      <c r="H24" s="48"/>
+      <c r="A24" s="51"/>
+      <c r="B24" s="51"/>
+      <c r="C24" s="51"/>
+      <c r="D24" s="51"/>
+      <c r="E24" s="51"/>
+      <c r="F24" s="51"/>
+      <c r="G24" s="51"/>
+      <c r="H24" s="51"/>
     </row>
     <row r="25" ht="21.75">
-      <c r="A25" s="48"/>
-      <c r="B25" s="29"/>
-      <c r="C25" s="29"/>
-      <c r="D25" s="29"/>
-      <c r="E25" s="48"/>
-      <c r="F25" s="48"/>
-      <c r="G25" s="48"/>
-      <c r="H25" s="48"/>
+      <c r="A25" s="51"/>
+      <c r="B25" s="32"/>
+      <c r="C25" s="32"/>
+      <c r="D25" s="32"/>
+      <c r="E25" s="51"/>
+      <c r="F25" s="51"/>
+      <c r="G25" s="51"/>
+      <c r="H25" s="51"/>
     </row>
     <row r="26" ht="21.75">
-      <c r="A26" s="48"/>
-      <c r="B26" s="48"/>
-      <c r="C26" s="48"/>
-      <c r="D26" s="48"/>
-      <c r="E26" s="48"/>
-      <c r="F26" s="48"/>
-      <c r="G26" s="48"/>
-      <c r="H26" s="48"/>
+      <c r="A26" s="51"/>
+      <c r="B26" s="51"/>
+      <c r="C26" s="51"/>
+      <c r="D26" s="51"/>
+      <c r="E26" s="51"/>
+      <c r="F26" s="51"/>
+      <c r="G26" s="51"/>
+      <c r="H26" s="51"/>
     </row>
     <row r="27" ht="21.75">
-      <c r="A27" s="48"/>
-      <c r="B27" s="29"/>
-      <c r="C27" s="29"/>
-      <c r="D27" s="29"/>
-      <c r="E27" s="48"/>
-      <c r="F27" s="48"/>
-      <c r="G27" s="48"/>
-      <c r="H27" s="48"/>
+      <c r="A27" s="51"/>
+      <c r="B27" s="32"/>
+      <c r="C27" s="32"/>
+      <c r="D27" s="32"/>
+      <c r="E27" s="51"/>
+      <c r="F27" s="51"/>
+      <c r="G27" s="51"/>
+      <c r="H27" s="51"/>
     </row>
     <row r="28" ht="14.25">
-      <c r="A28" s="39"/>
-      <c r="B28" s="28"/>
-      <c r="C28" s="28"/>
-      <c r="D28" s="29"/>
-      <c r="E28" s="29"/>
-      <c r="F28" s="29"/>
-      <c r="G28" s="28"/>
-      <c r="H28" s="29"/>
+      <c r="A28" s="42"/>
+      <c r="B28" s="31"/>
+      <c r="C28" s="31"/>
+      <c r="D28" s="32"/>
+      <c r="E28" s="32"/>
+      <c r="F28" s="32"/>
+      <c r="G28" s="31"/>
+      <c r="H28" s="32"/>
     </row>
     <row r="29" ht="14.25">
-      <c r="A29" s="28"/>
-      <c r="B29" s="28"/>
-      <c r="C29" s="28"/>
-      <c r="D29" s="29"/>
-      <c r="E29" s="29"/>
-      <c r="F29" s="29"/>
-      <c r="G29" s="28"/>
-      <c r="H29" s="29"/>
+      <c r="A29" s="31"/>
+      <c r="B29" s="31"/>
+      <c r="C29" s="31"/>
+      <c r="D29" s="32"/>
+      <c r="E29" s="32"/>
+      <c r="F29" s="32"/>
+      <c r="G29" s="31"/>
+      <c r="H29" s="32"/>
     </row>
     <row r="30" ht="14.25">
-      <c r="A30" s="28"/>
-      <c r="B30" s="28"/>
-      <c r="C30" s="28"/>
-      <c r="D30" s="29"/>
-      <c r="E30" s="29"/>
-      <c r="F30" s="29"/>
-      <c r="G30" s="28"/>
-      <c r="H30" s="29"/>
+      <c r="A30" s="31"/>
+      <c r="B30" s="31"/>
+      <c r="C30" s="31"/>
+      <c r="D30" s="32"/>
+      <c r="E30" s="32"/>
+      <c r="F30" s="32"/>
+      <c r="G30" s="31"/>
+      <c r="H30" s="32"/>
     </row>
     <row r="31" ht="14.25">
-      <c r="A31" s="28"/>
-      <c r="B31" s="28"/>
-      <c r="C31" s="28"/>
-      <c r="D31" s="29"/>
-      <c r="E31" s="29"/>
-      <c r="F31" s="29"/>
-      <c r="G31" s="28"/>
-      <c r="H31" s="29"/>
+      <c r="A31" s="31"/>
+      <c r="B31" s="31"/>
+      <c r="C31" s="31"/>
+      <c r="D31" s="32"/>
+      <c r="E31" s="32"/>
+      <c r="F31" s="32"/>
+      <c r="G31" s="31"/>
+      <c r="H31" s="32"/>
     </row>
     <row r="32" ht="14.25">
-      <c r="A32" s="28"/>
-      <c r="B32" s="28"/>
-      <c r="C32" s="28"/>
-      <c r="D32" s="29"/>
-      <c r="E32" s="29"/>
-      <c r="F32" s="29"/>
-      <c r="G32" s="28"/>
-      <c r="H32" s="29"/>
+      <c r="A32" s="31"/>
+      <c r="B32" s="31"/>
+      <c r="C32" s="31"/>
+      <c r="D32" s="32"/>
+      <c r="E32" s="32"/>
+      <c r="F32" s="32"/>
+      <c r="G32" s="31"/>
+      <c r="H32" s="32"/>
     </row>
     <row r="33" ht="14.25">
-      <c r="A33" s="28"/>
-      <c r="B33" s="28"/>
-      <c r="C33" s="28"/>
-      <c r="D33" s="29"/>
-      <c r="E33" s="29"/>
-      <c r="F33" s="29"/>
-      <c r="G33" s="28"/>
-      <c r="H33" s="29"/>
+      <c r="A33" s="31"/>
+      <c r="B33" s="31"/>
+      <c r="C33" s="31"/>
+      <c r="D33" s="32"/>
+      <c r="E33" s="32"/>
+      <c r="F33" s="32"/>
+      <c r="G33" s="31"/>
+      <c r="H33" s="32"/>
     </row>
     <row r="34" ht="14.25">
-      <c r="A34" s="28"/>
-      <c r="B34" s="28"/>
-      <c r="C34" s="28"/>
-      <c r="D34" s="29"/>
-      <c r="E34" s="29"/>
-      <c r="F34" s="29"/>
-      <c r="G34" s="28"/>
-      <c r="H34" s="29"/>
+      <c r="A34" s="31"/>
+      <c r="B34" s="31"/>
+      <c r="C34" s="31"/>
+      <c r="D34" s="32"/>
+      <c r="E34" s="32"/>
+      <c r="F34" s="32"/>
+      <c r="G34" s="31"/>
+      <c r="H34" s="32"/>
     </row>
     <row r="35" ht="14.25">
-      <c r="A35" s="28"/>
+      <c r="A35" s="31"/>
     </row>
     <row r="36" ht="14.25">
-      <c r="A36" s="28"/>
+      <c r="A36" s="31"/>
     </row>
     <row r="37" ht="14.25">
-      <c r="A37" s="28"/>
+      <c r="A37" s="31"/>
     </row>
     <row r="38" ht="14.25">
-      <c r="A38" s="28"/>
+      <c r="A38" s="31"/>
     </row>
     <row r="39" ht="14.25">
-      <c r="A39" s="28"/>
+      <c r="A39" s="31"/>
     </row>
     <row r="40" ht="14.25">
-      <c r="A40" s="28"/>
+      <c r="A40" s="31"/>
     </row>
     <row r="41" ht="14.25">
-      <c r="A41" s="28"/>
-      <c r="B41" s="28"/>
-      <c r="C41" s="28"/>
-      <c r="D41" s="29"/>
-      <c r="E41" s="29"/>
-      <c r="F41" s="29"/>
-      <c r="G41" s="28"/>
-      <c r="H41" s="29"/>
+      <c r="A41" s="31"/>
+      <c r="B41" s="31"/>
+      <c r="C41" s="31"/>
+      <c r="D41" s="32"/>
+      <c r="E41" s="32"/>
+      <c r="F41" s="32"/>
+      <c r="G41" s="31"/>
+      <c r="H41" s="32"/>
     </row>
     <row r="42" ht="14.25">
-      <c r="A42" s="28"/>
-      <c r="B42" s="28"/>
-      <c r="C42" s="28"/>
-      <c r="D42" s="29"/>
-      <c r="E42" s="29"/>
-      <c r="F42" s="29"/>
-      <c r="G42" s="28"/>
-      <c r="H42" s="29"/>
+      <c r="A42" s="31"/>
+      <c r="B42" s="31"/>
+      <c r="C42" s="31"/>
+      <c r="D42" s="32"/>
+      <c r="E42" s="32"/>
+      <c r="F42" s="32"/>
+      <c r="G42" s="31"/>
+      <c r="H42" s="32"/>
     </row>
     <row r="43" ht="14.25">
-      <c r="A43" s="28"/>
-      <c r="E43" s="29"/>
-      <c r="F43" s="29"/>
-      <c r="G43" s="28"/>
-      <c r="H43" s="29"/>
+      <c r="A43" s="31"/>
+      <c r="E43" s="32"/>
+      <c r="F43" s="32"/>
+      <c r="G43" s="31"/>
+      <c r="H43" s="32"/>
     </row>
     <row r="44" ht="14.25">
-      <c r="A44" s="28"/>
-      <c r="B44" s="28"/>
-      <c r="C44" s="28"/>
-      <c r="D44" s="29"/>
-      <c r="E44" s="29"/>
-      <c r="F44" s="29"/>
-      <c r="G44" s="28"/>
-      <c r="H44" s="29"/>
+      <c r="A44" s="31"/>
+      <c r="B44" s="31"/>
+      <c r="C44" s="31"/>
+      <c r="D44" s="32"/>
+      <c r="E44" s="32"/>
+      <c r="F44" s="32"/>
+      <c r="G44" s="31"/>
+      <c r="H44" s="32"/>
     </row>
     <row r="45" ht="14.25">
-      <c r="A45" s="28"/>
-      <c r="E45" s="29"/>
-      <c r="F45" s="29"/>
-      <c r="G45" s="28"/>
-      <c r="H45" s="29"/>
+      <c r="A45" s="31"/>
+      <c r="E45" s="32"/>
+      <c r="F45" s="32"/>
+      <c r="G45" s="31"/>
+      <c r="H45" s="32"/>
     </row>
     <row r="46" ht="14.25">
-      <c r="A46" s="28"/>
+      <c r="A46" s="31"/>
     </row>
   </sheetData>
   <mergeCells count="24">

</xml_diff>

<commit_message>
standardize patient tracker export to 13 columns with HTML-free TSV and improved HCPCS code detection
</commit_message>
<xml_diff>
--- a/core/UAT Plan.xlsx
+++ b/core/UAT Plan.xlsx
@@ -19,7 +19,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="184" uniqueCount="184">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="223" uniqueCount="223">
   <si>
     <t xml:space="preserve">Test Case #</t>
   </si>
@@ -605,13 +605,130 @@
   </si>
   <si>
     <t xml:space="preserve">Prior authorization placed in pending/moderate review status. Additional documentation requested including iron studies, treatment history, and confirmation of ongoing anemia management protocol.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Patient 17</t>
+  </si>
+  <si>
+    <t>Endocrinology</t>
+  </si>
+  <si>
+    <t>J3490</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ozempic (semaglutide) injection</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Patient: Linda Matthews, 58F, Endocrinology Follow-up</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Patient diagnosed with Type 2 Diabetes Mellitus with HbA1c of 9.2% despite metformin and glipizide therapy. BMI documented at 34. Medication adherence history included. Provider submitted recent labs and diabetic treatment plan.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Prior authorization approved based on uncontrolled Type 2 diabetes after step therapy failure. Documentation includes HbA1c results, previous medication trials, and endocrinology notes.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Patient 18</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Patient: Eric Collins, 45M, Primary Care Visit</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Request submitted for weight loss purposes only. No Type 2 diabetes diagnosis documented. HbA1c within normal range at 5.4%. No prior antidiabetic medication history provided.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Prior authorization denied due to lack of FDA-approved indication and missing Type 2 diabetes diagnosis. Weight loss alone does not meet plan criteria.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Patient 19</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Cardiology / Endocrinology</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Jardiance (empagliflozin) tablet</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Patient: Sharon Lee, 64F, Cardiology and Diabetes Management Visit</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Patient with Type 2 diabetes and established heart failure with reduced ejection fraction. HbA1c at 8.1%. Previously trialed metformin with inadequate glycemic control. Cardiology notes support cardiovascular benefit rationale.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Prior authorization approved based on Type 2 diabetes with cardiovascular comorbidity. Supporting labs, diagnosis history, and prior medication use documented.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Patient 20</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Patient: Michael Perez, 39M, Routine Wellness Encounter</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Medication requested without confirmed diabetes diagnosis, heart failure, or chronic kidney disease. No supporting labs or prior treatment records attached.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Prior authorization placed in moderate/pending review status due to insufficient clinical evidence. Additional diagnostic documentation and lab values requested.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Patient 21</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Kerendia (finerenone) tablet</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Patient: Thomas Grant, 71M, Nephrology Follow-up</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Patient with chronic kidney disease associated with Type 2 diabetes. eGFR and albuminuria levels documented within qualifying range. Current ACE inhibitor therapy noted. Nephrologist submitted full treatment history.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Prior authorization approved based on CKD associated with Type 2 diabetes and concurrent standard-of-care therapy. Required renal labs and treatment documentation included.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Patient 22</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Patient: Rebecca Young, 55F, Internal Medicine Visit</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Request submitted for hypertension management only. No chronic kidney disease diagnosis or albuminuria documentation available. Missing nephrology evaluation.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Prior authorization denied due to absence of qualifying CKD diagnosis and lack of supporting renal function documentation.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Patient 23</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Tarpeyo (budesonide delayed release) capsule</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Patient: Andrew Simmons, 43M, Nephrology Consultation</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Patient diagnosed with primary IgA nephropathy confirmed by kidney biopsy. Persistent proteinuria above threshold despite optimized ACE inhibitor therapy. Nephrology notes and pathology report attached.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Prior authorization approved based on confirmed IgA nephropathy diagnosis with persistent proteinuria despite supportive care treatment.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Patient 24</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Patient: Natalie Brooks, 47F, General Medicine Follow-up</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Medication requested for unspecified renal inflammation. No biopsy confirmation of IgA nephropathy. Proteinuria measurements and prior treatment history incomplete.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Prior authorization pending additional review. Insufficient pathology confirmation and incomplete nephrology documentation require further clinical records.</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
-  <fonts count="6">
+  <fonts count="4">
     <font>
       <sz val="11.000000"/>
       <color theme="1"/>
@@ -631,17 +748,6 @@
     </font>
     <font>
       <sz val="12.000000"/>
-      <name val="Times"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="12.000000"/>
-      <name val="Times"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="12.000000"/>
-      <color indexed="64"/>
       <name val="Times"/>
     </font>
   </fonts>
@@ -751,7 +857,7 @@
   <cellStyleXfs count="1">
     <xf fontId="0" fillId="0" borderId="0" numFmtId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
   </cellStyleXfs>
-  <cellXfs count="59">
+  <cellXfs count="47">
     <xf fontId="0" fillId="0" borderId="0" numFmtId="0" xfId="0"/>
     <xf fontId="0" fillId="0" borderId="0" numFmtId="0" xfId="0" applyAlignment="1">
       <alignment vertical="center"/>
@@ -836,47 +942,32 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf fontId="0" fillId="0" borderId="0" numFmtId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf fontId="0" fillId="0" borderId="0" numFmtId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
     <xf fontId="1" fillId="0" borderId="0" numFmtId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf fontId="1" fillId="2" borderId="1" numFmtId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
     <xf fontId="1" fillId="2" borderId="1" numFmtId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
     <xf fontId="2" fillId="0" borderId="1" numFmtId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
     <xf fontId="2" fillId="0" borderId="2" numFmtId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf fontId="2" fillId="0" borderId="2" numFmtId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
     <xf fontId="0" fillId="0" borderId="2" numFmtId="0" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
     <xf fontId="0" fillId="0" borderId="1" numFmtId="0" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf fontId="0" fillId="0" borderId="1" numFmtId="0" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
     <xf fontId="2" fillId="0" borderId="0" numFmtId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
     <xf fontId="2" fillId="0" borderId="3" numFmtId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf fontId="2" fillId="0" borderId="3" numFmtId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
     <xf fontId="0" fillId="0" borderId="3" numFmtId="0" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
@@ -889,41 +980,20 @@
     <xf fontId="3" fillId="0" borderId="3" numFmtId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf fontId="2" fillId="0" borderId="0" numFmtId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
     <xf fontId="2" fillId="0" borderId="5" numFmtId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf fontId="2" fillId="0" borderId="5" numFmtId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
     <xf fontId="0" fillId="0" borderId="5" numFmtId="0" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf fontId="0" fillId="0" borderId="2" numFmtId="0" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
     <xf fontId="2" fillId="0" borderId="6" numFmtId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
     <xf fontId="2" fillId="0" borderId="6" numFmtId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
-    <xf fontId="2" fillId="0" borderId="6" numFmtId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
     <xf fontId="0" fillId="0" borderId="6" numFmtId="0" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf fontId="0" fillId="0" borderId="6" numFmtId="0" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf fontId="4" fillId="0" borderId="0" numFmtId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf fontId="5" fillId="0" borderId="0" numFmtId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -2725,683 +2795,828 @@
     <col customWidth="1" min="1" max="1" style="29" width="12"/>
     <col bestFit="1" customWidth="1" min="2" max="2" style="29" width="11.85546875"/>
     <col min="3" max="3" style="29" width="9.140625"/>
-    <col customWidth="1" min="4" max="5" style="30" width="42.85546875"/>
-    <col customWidth="1" min="6" max="6" style="30" width="30.85546875"/>
+    <col customWidth="1" min="4" max="5" style="29" width="42.85546875"/>
+    <col customWidth="1" min="6" max="6" style="29" width="30.85546875"/>
     <col bestFit="1" customWidth="1" min="7" max="7" style="29" width="17.5703125"/>
-    <col customWidth="1" min="8" max="8" style="30" width="46.42578125"/>
+    <col customWidth="1" min="8" max="8" style="29" width="46.42578125"/>
     <col min="9" max="16384" style="29" width="9.140625"/>
   </cols>
   <sheetData>
-    <row r="1" s="31" customFormat="1">
-      <c r="A1" s="32" t="s">
+    <row r="1" s="30" customFormat="1">
+      <c r="A1" s="31" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="32" t="s">
+      <c r="B1" s="31" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="32" t="s">
+      <c r="C1" s="31" t="s">
         <v>108</v>
       </c>
-      <c r="D1" s="33" t="s">
+      <c r="D1" s="31" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="33" t="s">
+      <c r="E1" s="31" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="33" t="s">
+      <c r="F1" s="31" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="32" t="s">
+      <c r="G1" s="31" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="32" t="s">
+      <c r="H1" s="31" t="s">
         <v>7</v>
       </c>
     </row>
     <row r="2" ht="57">
-      <c r="A2" s="34" t="s">
+      <c r="A2" s="32" t="s">
         <v>71</v>
       </c>
-      <c r="B2" s="35" t="s">
+      <c r="B2" s="33" t="s">
         <v>109</v>
       </c>
-      <c r="C2" s="36" t="s">
+      <c r="C2" s="33" t="s">
         <v>110</v>
       </c>
-      <c r="D2" s="37" t="s">
+      <c r="D2" s="34" t="s">
         <v>111</v>
       </c>
-      <c r="E2" s="38" t="s">
+      <c r="E2" s="35" t="s">
         <v>112</v>
       </c>
-      <c r="F2" s="38" t="s">
+      <c r="F2" s="35" t="s">
         <v>113</v>
       </c>
-      <c r="G2" s="39" t="s">
+      <c r="G2" s="35" t="s">
         <v>13</v>
       </c>
-      <c r="H2" s="38" t="s">
+      <c r="H2" s="35" t="s">
         <v>114</v>
       </c>
-      <c r="I2" s="40">
+      <c r="I2" s="36">
         <v>260</v>
       </c>
       <c r="J2" s="29"/>
     </row>
     <row r="3" ht="50.25" customHeight="1">
-      <c r="A3" s="34" t="s">
+      <c r="A3" s="32" t="s">
         <v>71</v>
       </c>
-      <c r="B3" s="41"/>
-      <c r="C3" s="42"/>
-      <c r="D3" s="43"/>
-      <c r="E3" s="38" t="s">
+      <c r="B3" s="37"/>
+      <c r="C3" s="37"/>
+      <c r="D3" s="38"/>
+      <c r="E3" s="35" t="s">
         <v>115</v>
       </c>
-      <c r="F3" s="38" t="s">
+      <c r="F3" s="35" t="s">
         <v>116</v>
       </c>
-      <c r="G3" s="39" t="s">
+      <c r="G3" s="35" t="s">
         <v>17</v>
       </c>
-      <c r="H3" s="38" t="s">
+      <c r="H3" s="35" t="s">
         <v>117</v>
       </c>
-      <c r="I3" s="40">
+      <c r="I3" s="36">
         <v>261</v>
       </c>
       <c r="J3" s="29"/>
     </row>
     <row r="4" ht="71.25">
-      <c r="A4" s="34" t="s">
+      <c r="A4" s="32" t="s">
         <v>72</v>
       </c>
-      <c r="B4" s="35" t="s">
+      <c r="B4" s="33" t="s">
         <v>109</v>
       </c>
-      <c r="C4" s="36" t="s">
+      <c r="C4" s="33" t="s">
         <v>118</v>
       </c>
-      <c r="D4" s="37" t="s">
+      <c r="D4" s="34" t="s">
         <v>119</v>
       </c>
-      <c r="E4" s="38" t="s">
+      <c r="E4" s="35" t="s">
         <v>120</v>
       </c>
-      <c r="F4" s="38" t="s">
+      <c r="F4" s="35" t="s">
         <v>121</v>
       </c>
-      <c r="G4" s="39" t="s">
+      <c r="G4" s="35" t="s">
         <v>13</v>
       </c>
-      <c r="H4" s="38" t="s">
+      <c r="H4" s="35" t="s">
         <v>122</v>
       </c>
-      <c r="I4" s="40">
+      <c r="I4" s="36">
         <v>262</v>
       </c>
       <c r="J4" s="29"/>
     </row>
     <row r="5" ht="57">
-      <c r="A5" s="34" t="s">
+      <c r="A5" s="32" t="s">
         <v>72</v>
       </c>
-      <c r="B5" s="41"/>
-      <c r="C5" s="42"/>
-      <c r="D5" s="43"/>
-      <c r="E5" s="38" t="s">
+      <c r="B5" s="37"/>
+      <c r="C5" s="37"/>
+      <c r="D5" s="38"/>
+      <c r="E5" s="35" t="s">
         <v>123</v>
       </c>
-      <c r="F5" s="38" t="s">
+      <c r="F5" s="35" t="s">
         <v>124</v>
       </c>
-      <c r="G5" s="39" t="s">
+      <c r="G5" s="35" t="s">
         <v>17</v>
       </c>
-      <c r="H5" s="38" t="s">
+      <c r="H5" s="35" t="s">
         <v>125</v>
       </c>
-      <c r="I5" s="40">
+      <c r="I5" s="36">
         <v>263</v>
       </c>
       <c r="J5" s="29"/>
     </row>
     <row r="6" ht="57">
-      <c r="A6" s="34" t="s">
+      <c r="A6" s="32" t="s">
         <v>73</v>
       </c>
-      <c r="B6" s="35" t="s">
+      <c r="B6" s="33" t="s">
         <v>109</v>
       </c>
-      <c r="C6" s="36" t="s">
+      <c r="C6" s="33" t="s">
         <v>110</v>
       </c>
-      <c r="D6" s="37" t="s">
+      <c r="D6" s="34" t="s">
         <v>111</v>
       </c>
-      <c r="E6" s="38" t="s">
+      <c r="E6" s="35" t="s">
         <v>126</v>
       </c>
-      <c r="F6" s="38" t="s">
+      <c r="F6" s="35" t="s">
         <v>127</v>
       </c>
-      <c r="G6" s="39" t="s">
+      <c r="G6" s="35" t="s">
         <v>13</v>
       </c>
-      <c r="H6" s="38" t="s">
+      <c r="H6" s="35" t="s">
         <v>114</v>
       </c>
-      <c r="I6" s="40">
+      <c r="I6" s="36">
         <v>264</v>
       </c>
       <c r="J6" s="29"/>
     </row>
     <row r="7" ht="108.75">
-      <c r="A7" s="34" t="s">
+      <c r="A7" s="32" t="s">
         <v>73</v>
       </c>
-      <c r="B7" s="41"/>
-      <c r="C7" s="42"/>
-      <c r="D7" s="43"/>
-      <c r="E7" s="44" t="s">
+      <c r="B7" s="37"/>
+      <c r="C7" s="37"/>
+      <c r="D7" s="38"/>
+      <c r="E7" s="39" t="s">
         <v>128</v>
       </c>
-      <c r="F7" s="44" t="s">
+      <c r="F7" s="39" t="s">
         <v>129</v>
       </c>
-      <c r="G7" s="44" t="s">
+      <c r="G7" s="39" t="s">
         <v>17</v>
       </c>
-      <c r="H7" s="44" t="s">
+      <c r="H7" s="39" t="s">
         <v>117</v>
       </c>
-      <c r="I7" s="40">
+      <c r="I7" s="36">
         <v>265</v>
       </c>
       <c r="J7" s="29"/>
     </row>
     <row r="8" ht="108.75">
-      <c r="A8" s="34" t="s">
+      <c r="A8" s="32" t="s">
         <v>74</v>
       </c>
-      <c r="B8" s="35" t="s">
+      <c r="B8" s="33" t="s">
         <v>109</v>
       </c>
-      <c r="C8" s="36" t="s">
+      <c r="C8" s="33" t="s">
         <v>118</v>
       </c>
-      <c r="D8" s="45" t="s">
+      <c r="D8" s="40" t="s">
         <v>119</v>
       </c>
-      <c r="E8" s="44" t="s">
+      <c r="E8" s="39" t="s">
         <v>130</v>
       </c>
-      <c r="F8" s="44" t="s">
+      <c r="F8" s="39" t="s">
         <v>131</v>
       </c>
-      <c r="G8" s="44" t="s">
+      <c r="G8" s="39" t="s">
         <v>13</v>
       </c>
-      <c r="H8" s="44" t="s">
+      <c r="H8" s="39" t="s">
         <v>122</v>
       </c>
-      <c r="I8" s="40">
+      <c r="I8" s="36">
         <v>266</v>
       </c>
       <c r="J8" s="29"/>
     </row>
     <row r="9" ht="108.75">
-      <c r="A9" s="34" t="s">
+      <c r="A9" s="32" t="s">
         <v>74</v>
       </c>
-      <c r="B9" s="41"/>
-      <c r="C9" s="42"/>
-      <c r="D9" s="46"/>
-      <c r="E9" s="44" t="s">
+      <c r="B9" s="37"/>
+      <c r="C9" s="37"/>
+      <c r="D9" s="41"/>
+      <c r="E9" s="39" t="s">
         <v>132</v>
       </c>
-      <c r="F9" s="44" t="s">
+      <c r="F9" s="39" t="s">
         <v>133</v>
       </c>
-      <c r="G9" s="44" t="s">
+      <c r="G9" s="39" t="s">
         <v>17</v>
       </c>
-      <c r="H9" s="44" t="s">
+      <c r="H9" s="39" t="s">
         <v>125</v>
       </c>
-      <c r="I9" s="40">
+      <c r="I9" s="36">
         <v>267</v>
       </c>
       <c r="J9" s="29"/>
     </row>
     <row r="10" ht="108.75">
-      <c r="A10" s="34" t="s">
+      <c r="A10" s="32" t="s">
         <v>75</v>
       </c>
-      <c r="B10" s="35" t="s">
+      <c r="B10" s="33" t="s">
         <v>134</v>
       </c>
-      <c r="C10" s="36" t="s">
+      <c r="C10" s="33" t="s">
         <v>135</v>
       </c>
-      <c r="D10" s="45" t="s">
+      <c r="D10" s="40" t="s">
         <v>136</v>
       </c>
-      <c r="E10" s="44" t="s">
+      <c r="E10" s="39" t="s">
         <v>137</v>
       </c>
-      <c r="F10" s="44" t="s">
+      <c r="F10" s="39" t="s">
         <v>138</v>
       </c>
-      <c r="G10" s="44" t="s">
+      <c r="G10" s="39" t="s">
         <v>13</v>
       </c>
-      <c r="H10" s="44" t="s">
+      <c r="H10" s="39" t="s">
         <v>139</v>
       </c>
-      <c r="I10" s="40">
+      <c r="I10" s="36">
         <v>268</v>
       </c>
       <c r="J10" s="29"/>
     </row>
     <row r="11" ht="87">
-      <c r="A11" s="34" t="s">
+      <c r="A11" s="32" t="s">
         <v>75</v>
       </c>
-      <c r="B11" s="41"/>
-      <c r="C11" s="42"/>
-      <c r="D11" s="46"/>
-      <c r="E11" s="44" t="s">
+      <c r="B11" s="37"/>
+      <c r="C11" s="37"/>
+      <c r="D11" s="41"/>
+      <c r="E11" s="39" t="s">
         <v>140</v>
       </c>
-      <c r="F11" s="44" t="s">
+      <c r="F11" s="39" t="s">
         <v>141</v>
       </c>
-      <c r="G11" s="44" t="s">
+      <c r="G11" s="39" t="s">
         <v>21</v>
       </c>
-      <c r="H11" s="44" t="s">
+      <c r="H11" s="39" t="s">
         <v>142</v>
       </c>
-      <c r="I11" s="40">
+      <c r="I11" s="36">
         <v>269</v>
       </c>
       <c r="J11" s="29"/>
     </row>
     <row r="12" ht="71.25">
-      <c r="A12" s="40" t="s">
+      <c r="A12" s="36" t="s">
         <v>76</v>
       </c>
-      <c r="B12" s="47" t="s">
+      <c r="B12" s="36" t="s">
         <v>143</v>
       </c>
-      <c r="C12" s="40" t="s">
+      <c r="C12" s="36" t="s">
         <v>144</v>
       </c>
-      <c r="D12" s="30" t="s">
+      <c r="D12" s="29" t="s">
         <v>145</v>
       </c>
-      <c r="E12" s="30" t="s">
+      <c r="E12" s="29" t="s">
         <v>146</v>
       </c>
-      <c r="F12" s="30" t="s">
+      <c r="F12" s="29" t="s">
         <v>147</v>
       </c>
-      <c r="G12" s="39" t="s">
+      <c r="G12" s="35" t="s">
         <v>17</v>
       </c>
-      <c r="H12" s="30" t="s">
+      <c r="H12" s="29" t="s">
         <v>142</v>
       </c>
-      <c r="I12" s="40">
+      <c r="I12" s="36">
         <v>270</v>
       </c>
     </row>
     <row r="13" ht="71.25">
-      <c r="A13" s="40" t="s">
+      <c r="A13" s="36" t="s">
         <v>76</v>
       </c>
-      <c r="B13" s="47"/>
-      <c r="C13" s="40"/>
-      <c r="D13" s="30"/>
-      <c r="E13" s="30" t="s">
+      <c r="B13" s="36"/>
+      <c r="C13" s="36"/>
+      <c r="D13" s="29"/>
+      <c r="E13" s="29" t="s">
         <v>148</v>
       </c>
-      <c r="F13" s="30" t="s">
+      <c r="F13" s="29" t="s">
         <v>149</v>
       </c>
-      <c r="G13" s="39" t="s">
+      <c r="G13" s="35" t="s">
         <v>13</v>
       </c>
-      <c r="H13" s="30" t="s">
+      <c r="H13" s="29" t="s">
         <v>150</v>
       </c>
-      <c r="I13" s="40">
+      <c r="I13" s="36">
         <v>271</v>
       </c>
     </row>
     <row r="14" ht="57">
-      <c r="A14" s="34" t="s">
+      <c r="A14" s="32" t="s">
         <v>151</v>
       </c>
-      <c r="B14" s="35" t="s">
+      <c r="B14" s="33" t="s">
         <v>109</v>
       </c>
-      <c r="C14" s="36">
+      <c r="C14" s="33">
         <v>45380</v>
       </c>
-      <c r="D14" s="37" t="s">
+      <c r="D14" s="34" t="s">
         <v>152</v>
       </c>
-      <c r="E14" s="38" t="s">
+      <c r="E14" s="35" t="s">
         <v>153</v>
       </c>
-      <c r="F14" s="38" t="s">
+      <c r="F14" s="35" t="s">
         <v>154</v>
       </c>
-      <c r="G14" s="39" t="s">
+      <c r="G14" s="35" t="s">
         <v>17</v>
       </c>
-      <c r="H14" s="38" t="s">
+      <c r="H14" s="35" t="s">
         <v>155</v>
       </c>
-      <c r="I14" s="40">
+      <c r="I14" s="36">
         <v>272</v>
       </c>
     </row>
     <row r="15" ht="99.75">
-      <c r="A15" s="34" t="s">
+      <c r="A15" s="32" t="s">
         <v>156</v>
       </c>
-      <c r="B15" s="41"/>
-      <c r="C15" s="42"/>
-      <c r="D15" s="43"/>
-      <c r="E15" s="38" t="s">
+      <c r="B15" s="37"/>
+      <c r="C15" s="37"/>
+      <c r="D15" s="38"/>
+      <c r="E15" s="35" t="s">
         <v>157</v>
       </c>
-      <c r="F15" s="38" t="s">
+      <c r="F15" s="35" t="s">
         <v>158</v>
       </c>
-      <c r="G15" s="39" t="s">
+      <c r="G15" s="35" t="s">
         <v>13</v>
       </c>
-      <c r="H15" s="38" t="s">
+      <c r="H15" s="35" t="s">
         <v>159</v>
       </c>
-      <c r="I15" s="40">
+      <c r="I15" s="36">
         <v>273</v>
       </c>
     </row>
     <row r="16" ht="85.5">
-      <c r="A16" s="34" t="s">
+      <c r="A16" s="32" t="s">
         <v>151</v>
       </c>
-      <c r="B16" s="35" t="s">
+      <c r="B16" s="33" t="s">
         <v>109</v>
       </c>
-      <c r="C16" s="36">
+      <c r="C16" s="33">
         <v>43235</v>
       </c>
-      <c r="D16" s="37" t="s">
+      <c r="D16" s="34" t="s">
         <v>160</v>
       </c>
-      <c r="E16" s="38" t="s">
+      <c r="E16" s="35" t="s">
         <v>161</v>
       </c>
-      <c r="F16" s="38" t="s">
+      <c r="F16" s="35" t="s">
         <v>162</v>
       </c>
-      <c r="G16" s="39" t="s">
+      <c r="G16" s="35" t="s">
         <v>17</v>
       </c>
-      <c r="H16" s="38" t="s">
+      <c r="H16" s="35" t="s">
         <v>163</v>
       </c>
-      <c r="I16" s="40">
+      <c r="I16" s="36">
         <v>274</v>
       </c>
     </row>
     <row r="17" ht="71.25">
-      <c r="A17" s="36" t="s">
+      <c r="A17" s="33" t="s">
         <v>156</v>
       </c>
-      <c r="B17" s="48"/>
-      <c r="C17" s="49"/>
-      <c r="D17" s="50"/>
-      <c r="E17" s="37" t="s">
+      <c r="B17" s="42"/>
+      <c r="C17" s="42"/>
+      <c r="D17" s="43"/>
+      <c r="E17" s="34" t="s">
         <v>164</v>
       </c>
-      <c r="F17" s="37" t="s">
+      <c r="F17" s="34" t="s">
         <v>165</v>
       </c>
-      <c r="G17" s="51" t="s">
+      <c r="G17" s="34" t="s">
         <v>13</v>
       </c>
-      <c r="H17" s="37" t="s">
+      <c r="H17" s="34" t="s">
         <v>166</v>
       </c>
-      <c r="I17" s="40">
+      <c r="I17" s="36">
         <v>275</v>
       </c>
     </row>
     <row r="18" ht="114">
-      <c r="A18" s="52" t="s">
+      <c r="A18" s="44" t="s">
         <v>167</v>
       </c>
-      <c r="B18" s="53" t="s">
+      <c r="B18" s="45" t="s">
         <v>109</v>
       </c>
-      <c r="C18" s="54" t="s">
+      <c r="C18" s="45" t="s">
         <v>168</v>
       </c>
-      <c r="D18" s="55" t="s">
+      <c r="D18" s="46" t="s">
         <v>169</v>
       </c>
-      <c r="E18" s="55" t="s">
+      <c r="E18" s="46" t="s">
         <v>170</v>
       </c>
-      <c r="F18" s="55" t="s">
+      <c r="F18" s="46" t="s">
         <v>171</v>
       </c>
-      <c r="G18" s="56" t="s">
+      <c r="G18" s="46" t="s">
         <v>172</v>
       </c>
-      <c r="H18" s="55" t="s">
+      <c r="H18" s="46" t="s">
         <v>173</v>
       </c>
-      <c r="I18" s="40">
+      <c r="I18" s="36">
         <v>276</v>
       </c>
     </row>
     <row r="19" ht="99.75">
-      <c r="A19" s="52" t="s">
+      <c r="A19" s="44" t="s">
         <v>174</v>
       </c>
-      <c r="B19" s="53"/>
-      <c r="C19" s="54"/>
-      <c r="D19" s="55" t="s">
+      <c r="B19" s="45"/>
+      <c r="C19" s="45"/>
+      <c r="D19" s="46" t="s">
         <v>169</v>
       </c>
-      <c r="E19" s="55" t="s">
+      <c r="E19" s="46" t="s">
         <v>175</v>
       </c>
-      <c r="F19" s="55" t="s">
+      <c r="F19" s="46" t="s">
         <v>176</v>
       </c>
-      <c r="G19" s="56" t="s">
+      <c r="G19" s="46" t="s">
         <v>177</v>
       </c>
-      <c r="H19" s="55" t="s">
+      <c r="H19" s="46" t="s">
         <v>178</v>
       </c>
-      <c r="I19" s="40">
+      <c r="I19" s="36">
         <v>277</v>
       </c>
     </row>
     <row r="20" ht="114">
-      <c r="A20" s="52" t="s">
+      <c r="A20" s="44" t="s">
         <v>179</v>
       </c>
-      <c r="B20" s="53"/>
-      <c r="C20" s="54"/>
-      <c r="D20" s="55" t="s">
+      <c r="B20" s="45"/>
+      <c r="C20" s="45"/>
+      <c r="D20" s="46" t="s">
         <v>169</v>
       </c>
-      <c r="E20" s="55" t="s">
+      <c r="E20" s="46" t="s">
         <v>180</v>
       </c>
-      <c r="F20" s="55" t="s">
+      <c r="F20" s="46" t="s">
         <v>181</v>
       </c>
-      <c r="G20" s="56" t="s">
+      <c r="G20" s="46" t="s">
         <v>182</v>
       </c>
-      <c r="H20" s="55" t="s">
+      <c r="H20" s="46" t="s">
         <v>183</v>
       </c>
       <c r="I20" s="29">
         <v>278</v>
       </c>
     </row>
-    <row r="21" ht="14.25">
-      <c r="A21" s="29"/>
-      <c r="B21" s="29"/>
-      <c r="C21" s="29"/>
-      <c r="D21" s="30"/>
-      <c r="E21" s="30"/>
-      <c r="F21" s="30"/>
-      <c r="G21" s="29"/>
-      <c r="H21" s="30"/>
-    </row>
-    <row r="22" ht="14.25">
-      <c r="A22" s="29"/>
-      <c r="B22" s="29"/>
-      <c r="C22" s="29"/>
-      <c r="D22" s="30"/>
-      <c r="E22" s="30"/>
-      <c r="F22" s="30"/>
-      <c r="G22" s="29"/>
-      <c r="H22" s="30"/>
-    </row>
-    <row r="23" ht="21.75">
-      <c r="A23" s="57"/>
-      <c r="B23" s="58"/>
-      <c r="C23" s="58"/>
-      <c r="D23" s="58"/>
-      <c r="E23" s="58"/>
-      <c r="F23" s="58"/>
-      <c r="G23" s="58"/>
-      <c r="H23" s="57"/>
-    </row>
-    <row r="24" ht="14.25">
-      <c r="A24" s="29"/>
-      <c r="B24" s="29"/>
-      <c r="C24" s="29"/>
-      <c r="D24" s="30"/>
-      <c r="E24" s="30"/>
-      <c r="F24" s="30"/>
-      <c r="G24" s="29"/>
-      <c r="H24" s="30"/>
-    </row>
-    <row r="25" ht="14.25">
-      <c r="A25" s="29"/>
-      <c r="B25" s="29"/>
-      <c r="C25" s="29"/>
-      <c r="D25" s="30"/>
-      <c r="E25" s="30"/>
-      <c r="F25" s="30"/>
-      <c r="G25" s="29"/>
-      <c r="H25" s="30"/>
-    </row>
-    <row r="26" ht="14.25">
-      <c r="A26" s="29"/>
-      <c r="B26" s="29"/>
-      <c r="C26" s="29"/>
-      <c r="D26" s="30"/>
-      <c r="E26" s="30"/>
-      <c r="F26" s="30"/>
-      <c r="G26" s="29"/>
-      <c r="H26" s="30"/>
-    </row>
-    <row r="27" ht="14.25">
-      <c r="A27" s="29"/>
-      <c r="B27" s="29"/>
-      <c r="C27" s="29"/>
-      <c r="D27" s="30"/>
-      <c r="E27" s="30"/>
-      <c r="F27" s="30"/>
-      <c r="G27" s="29"/>
-      <c r="H27" s="30"/>
-    </row>
-    <row r="28" ht="14.25">
-      <c r="A28" s="29"/>
-      <c r="B28" s="29"/>
-      <c r="C28" s="29"/>
-      <c r="D28" s="30"/>
-      <c r="E28" s="30"/>
-      <c r="F28" s="30"/>
-      <c r="G28" s="29"/>
-      <c r="H28" s="30"/>
+    <row r="21" ht="152.25">
+      <c r="A21" s="44" t="s">
+        <v>184</v>
+      </c>
+      <c r="B21" s="44" t="s">
+        <v>185</v>
+      </c>
+      <c r="C21" s="44" t="s">
+        <v>186</v>
+      </c>
+      <c r="D21" s="44" t="s">
+        <v>187</v>
+      </c>
+      <c r="E21" s="44" t="s">
+        <v>188</v>
+      </c>
+      <c r="F21" s="44" t="s">
+        <v>189</v>
+      </c>
+      <c r="G21" s="44" t="s">
+        <v>172</v>
+      </c>
+      <c r="H21" s="44" t="s">
+        <v>190</v>
+      </c>
+      <c r="I21" s="36">
+        <v>279</v>
+      </c>
+    </row>
+    <row r="22" ht="130.5">
+      <c r="A22" s="44" t="s">
+        <v>191</v>
+      </c>
+      <c r="B22" s="44" t="s">
+        <v>185</v>
+      </c>
+      <c r="C22" s="44" t="s">
+        <v>186</v>
+      </c>
+      <c r="D22" s="44" t="s">
+        <v>187</v>
+      </c>
+      <c r="E22" s="44" t="s">
+        <v>192</v>
+      </c>
+      <c r="F22" s="44" t="s">
+        <v>193</v>
+      </c>
+      <c r="G22" s="44" t="s">
+        <v>177</v>
+      </c>
+      <c r="H22" s="44" t="s">
+        <v>194</v>
+      </c>
+      <c r="I22" s="36">
+        <v>280</v>
+      </c>
+    </row>
+    <row r="23" ht="152.25">
+      <c r="A23" s="44" t="s">
+        <v>195</v>
+      </c>
+      <c r="B23" s="44" t="s">
+        <v>196</v>
+      </c>
+      <c r="C23" s="44" t="s">
+        <v>186</v>
+      </c>
+      <c r="D23" s="44" t="s">
+        <v>197</v>
+      </c>
+      <c r="E23" s="44" t="s">
+        <v>198</v>
+      </c>
+      <c r="F23" s="44" t="s">
+        <v>199</v>
+      </c>
+      <c r="G23" s="44" t="s">
+        <v>172</v>
+      </c>
+      <c r="H23" s="44" t="s">
+        <v>200</v>
+      </c>
+      <c r="I23" s="29">
+        <v>281</v>
+      </c>
+    </row>
+    <row r="24" ht="108.75">
+      <c r="A24" s="44" t="s">
+        <v>201</v>
+      </c>
+      <c r="B24" s="44" t="s">
+        <v>196</v>
+      </c>
+      <c r="C24" s="44" t="s">
+        <v>186</v>
+      </c>
+      <c r="D24" s="44" t="s">
+        <v>197</v>
+      </c>
+      <c r="E24" s="44" t="s">
+        <v>202</v>
+      </c>
+      <c r="F24" s="44" t="s">
+        <v>203</v>
+      </c>
+      <c r="G24" s="44" t="s">
+        <v>182</v>
+      </c>
+      <c r="H24" s="44" t="s">
+        <v>204</v>
+      </c>
+      <c r="I24" s="36">
+        <v>282</v>
+      </c>
+    </row>
+    <row r="25" ht="152.25">
+      <c r="A25" s="44" t="s">
+        <v>205</v>
+      </c>
+      <c r="B25" s="44" t="s">
+        <v>44</v>
+      </c>
+      <c r="C25" s="44" t="s">
+        <v>186</v>
+      </c>
+      <c r="D25" s="44" t="s">
+        <v>206</v>
+      </c>
+      <c r="E25" s="44" t="s">
+        <v>207</v>
+      </c>
+      <c r="F25" s="44" t="s">
+        <v>208</v>
+      </c>
+      <c r="G25" s="44" t="s">
+        <v>172</v>
+      </c>
+      <c r="H25" s="44" t="s">
+        <v>209</v>
+      </c>
+      <c r="I25" s="36">
+        <v>283</v>
+      </c>
+    </row>
+    <row r="26" ht="108.75">
+      <c r="A26" s="44" t="s">
+        <v>210</v>
+      </c>
+      <c r="B26" s="44" t="s">
+        <v>44</v>
+      </c>
+      <c r="C26" s="44" t="s">
+        <v>186</v>
+      </c>
+      <c r="D26" s="44" t="s">
+        <v>206</v>
+      </c>
+      <c r="E26" s="44" t="s">
+        <v>211</v>
+      </c>
+      <c r="F26" s="44" t="s">
+        <v>212</v>
+      </c>
+      <c r="G26" s="44" t="s">
+        <v>177</v>
+      </c>
+      <c r="H26" s="44" t="s">
+        <v>213</v>
+      </c>
+      <c r="I26" s="29">
+        <v>284</v>
+      </c>
+    </row>
+    <row r="27" ht="130.5">
+      <c r="A27" s="44" t="s">
+        <v>214</v>
+      </c>
+      <c r="B27" s="44" t="s">
+        <v>44</v>
+      </c>
+      <c r="C27" s="44" t="s">
+        <v>186</v>
+      </c>
+      <c r="D27" s="44" t="s">
+        <v>215</v>
+      </c>
+      <c r="E27" s="44" t="s">
+        <v>216</v>
+      </c>
+      <c r="F27" s="44" t="s">
+        <v>217</v>
+      </c>
+      <c r="G27" s="44" t="s">
+        <v>172</v>
+      </c>
+      <c r="H27" s="44" t="s">
+        <v>218</v>
+      </c>
+      <c r="I27" s="36">
+        <v>285</v>
+      </c>
+    </row>
+    <row r="28" ht="108.75">
+      <c r="A28" s="44" t="s">
+        <v>219</v>
+      </c>
+      <c r="B28" s="44" t="s">
+        <v>44</v>
+      </c>
+      <c r="C28" s="44" t="s">
+        <v>186</v>
+      </c>
+      <c r="D28" s="44" t="s">
+        <v>215</v>
+      </c>
+      <c r="E28" s="44" t="s">
+        <v>220</v>
+      </c>
+      <c r="F28" s="44" t="s">
+        <v>221</v>
+      </c>
+      <c r="G28" s="44" t="s">
+        <v>182</v>
+      </c>
+      <c r="H28" s="44" t="s">
+        <v>222</v>
+      </c>
+      <c r="I28" s="36">
+        <v>286</v>
+      </c>
     </row>
     <row r="29" ht="14.25">
       <c r="A29" s="29"/>
       <c r="B29" s="29"/>
       <c r="C29" s="29"/>
-      <c r="D29" s="30"/>
-      <c r="E29" s="30"/>
-      <c r="F29" s="30"/>
+      <c r="D29" s="29"/>
+      <c r="E29" s="29"/>
+      <c r="F29" s="29"/>
       <c r="G29" s="29"/>
-      <c r="H29" s="30"/>
+      <c r="H29" s="29"/>
     </row>
     <row r="30" ht="14.25">
       <c r="A30" s="29"/>
       <c r="B30" s="29"/>
       <c r="C30" s="29"/>
-      <c r="D30" s="30"/>
-      <c r="E30" s="30"/>
-      <c r="F30" s="30"/>
+      <c r="D30" s="29"/>
+      <c r="E30" s="29"/>
+      <c r="F30" s="29"/>
       <c r="G30" s="29"/>
-      <c r="H30" s="30"/>
+      <c r="H30" s="29"/>
     </row>
     <row r="31" ht="14.25">
       <c r="A31" s="29"/>
       <c r="B31" s="29"/>
       <c r="C31" s="29"/>
-      <c r="D31" s="30"/>
-      <c r="E31" s="30"/>
-      <c r="F31" s="30"/>
+      <c r="D31" s="29"/>
+      <c r="E31" s="29"/>
+      <c r="F31" s="29"/>
       <c r="G31" s="29"/>
-      <c r="H31" s="30"/>
+      <c r="H31" s="29"/>
     </row>
     <row r="32" ht="14.25">
       <c r="A32" s="29"/>
       <c r="B32" s="29"/>
       <c r="C32" s="29"/>
-      <c r="D32" s="30"/>
-      <c r="E32" s="30"/>
-      <c r="F32" s="30"/>
+      <c r="D32" s="29"/>
+      <c r="E32" s="29"/>
+      <c r="F32" s="29"/>
       <c r="G32" s="29"/>
-      <c r="H32" s="30"/>
+      <c r="H32" s="29"/>
     </row>
     <row r="33" ht="14.25">
       <c r="A33" s="29"/>
       <c r="B33" s="29"/>
       <c r="C33" s="29"/>
-      <c r="D33" s="30"/>
-      <c r="E33" s="30"/>
-      <c r="F33" s="30"/>
+      <c r="D33" s="29"/>
+      <c r="E33" s="29"/>
+      <c r="F33" s="29"/>
       <c r="G33" s="29"/>
-      <c r="H33" s="30"/>
+      <c r="H33" s="29"/>
     </row>
     <row r="34" ht="14.25">
       <c r="A34" s="29"/>
-      <c r="B34" s="29"/>
-      <c r="C34" s="29"/>
-      <c r="D34" s="30"/>
-      <c r="E34" s="30"/>
-      <c r="F34" s="30"/>
-      <c r="G34" s="29"/>
-      <c r="H34" s="30"/>
     </row>
     <row r="35" ht="14.25">
       <c r="A35" s="29"/>
@@ -3411,9 +3626,6 @@
     </row>
     <row r="37" ht="14.25">
       <c r="A37" s="29"/>
-    </row>
-    <row r="38" ht="14.25">
-      <c r="A38" s="29"/>
     </row>
   </sheetData>
   <mergeCells count="26">

</xml_diff>